<commit_message>
Phase 5 step 1: batch input reader, resolution to targets, stored inputs
- engine/batch/reader.py: pasted list, CSV (; or ,; UTF-8/BOM or Windows-1257)
  and XLSX (Testa_kopa sheet or first sheet); columns vertiba, projekta_nr,
  pieteicejs_reg_nr, adrese, veids; limit 1,000 rows; nothing written to disk.
- engine/batch/plan.py: /resolve rules; property-or-parcel numbers checked both
  ways (labelled "divdomīgs: …") unless veids decides; addresses checked on every
  linked object; unresolved rows kept with reason and suggestions; adrese as the
  given address; applicant reg. no. only with the legal-entity pattern and
  personal-code-like values never stored (rule 5).
- Migration: work.run_input (cleaned list, insert-only) and run_target input_no,
  label, applicant_reg_no; pinned sources carry coverage and processing notes.
- test_set_template.xlsx: optional veids column (rebuilt); check compare uses it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data/test_set_template.xlsx
+++ b/tests/data/test_set_template.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -508,126 +508,133 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>• vertiba: kadastra numurs (11 cipari), kadastra apzīmējums (11, 14 vai 17 cipari) vai adrese. Kolonnas A–C ir teksta formātā: ievadiet ciparus ar sākuma nullēm (piem., 05000041006).</t>
+          <t>• vertiba: kadastra numurs (11 cipari), kadastra apzīmējums (11, 14 vai 17 cipari) vai adrese. Kolonnas A–D ir teksta formātā: ievadiet ciparus ar sākuma nullēm (piem., 05000041006).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• pieteicejs_reg_nr: pieteicēja juridiskās personas reģistrācijas numurs (ja ir). Fizisko personu vārdus un personas kodus neievadiet.</t>
+          <t>• veids (neobligāts): īpašums, zemes vienība vai būve. Aizpildiet, ja 11 ciparu numurs var būt gan īpašuma numurs, gan citam īpašumam piederošas zemes vienības apzīmējums; bez tā rīks pārbauda abus.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>• m1–m6: jūsu manuālās pārbaudes atbilde katram modulim. Sāciet ar vienu no: «Ir: …» (atrasts, īsi ko), «Nav», «Nav datu» (objekts nav atrasts / nav ģeometrijas), «Nav pārklājuma» (avotā šai teritorijai nav datu, piem., nav plūdu kartes). Pēc tam īss paskaidrojums.</t>
+          <t>• pieteicejs_reg_nr: pieteicēja juridiskās personas reģistrācijas numurs (ja ir). Fizisko personu vārdus un personas kodus neievadiet.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>• parbaudes_datums: datums, kad veicāt pārbaudi (GGGG-MM-DD). Svarīgi, jo dati laika gaitā mainās.</t>
+          <t>• m1–m6: jūsu manuālās pārbaudes atbilde katram modulim. Sāciet ar vienu no: «Ir: …» (atrasts, īsi ko), «Nav», «Nav datu» (objekts nav atrasts / nav ģeometrijas), «Nav pārklājuma» (avotā šai teritorijai nav datu, piem., nav plūdu kartes). Pēc tam īss paskaidrojums.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>• parbaudes_datums: datums, kad veicāt pārbaudi (GGGG-MM-DD). Svarīgi, jo dati laika gaitā mainās.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>• avots_piezimes: kurus portālus izmantojāt un citas piezīmes.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Moduļi:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>m1 Kadastra dati: zemes vienības / būves, platība, lietošanas mērķis, būves uz zemes vienības.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>m2 Adreses atbilstība: vai norādītā adrese atbilst kadastra objektam («Neatbilst»).</t>
+          <t>m1 Kadastra dati: zemes vienības / būves, platība, lietošanas mērķis, būves uz zemes vienības.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>m3 Aizsargājamā daba: ĪADT, mikroliegums, mikrolieguma buferzona, dabas piemineklis, aizsargājams biotops (katru atsevišķi).</t>
+          <t>m2 Adreses atbilstība: vai norādītā adrese atbilst kadastra objektam («Neatbilst»).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>m4 Plūdi: 3. cikla pavasara palu karte, reizi 10 gados (10 % varbūtība). Vai objekts ir plūdu zonā, aptuvenais pārklājums.</t>
+          <t>m3 Aizsargājamā daba: ĪADT, mikroliegums, mikrolieguma buferzona, dabas piemineklis, aizsargājams biotops (katru atsevišķi).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>m5 Būvniecības lietas (BIS): lietas uz šī objekta; norādiet BIS lietas numurus un vai tās ir tieši uz objekta vai blakus.</t>
+          <t>m4 Plūdi: 3. cikla pavasara palu karte, reizi 10 gados (10 % varbūtība). Vai objekts ir plūdu zonā, aptuvenais pārklājums.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>m5 Būvniecības lietas (BIS): lietas uz šī objekta; norādiet BIS lietas numurus un vai tās ir tieši uz objekta vai blakus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>m6 Apgrūtinājumi: kadastrā reģistrētie apgrūtinājumi (kods vai nosaukums).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Lūdzam testa kopā iekļaut:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• vismaz vienu zemes vienību, kas atrodas 10 gadu plūdu zonā;</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>• vismaz vienu objektu ārpus plūdu karšu pārklājuma (teritorijā, kurai plūdu karte nav izstrādāta);</t>
+          <t>• vismaz vienu zemes vienību, kas atrodas 10 gadu plūdu zonā;</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>• vismaz vienu objektu ārpus plūdu karšu pārklājuma (teritorijā, kurai plūdu karte nav izstrādāta);</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>• ja iespējams: objektu ar būvniecības lietu, objektu dabas teritorijā un objektu ar vairākām zemes vienībām vai būvēm.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Dzeltenās rindas ir piemēri: izdzēsiet tās vai aizstājiet ar saviem datiem.</t>
         </is>
@@ -644,20 +651,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K501"/>
+  <dimension ref="A1:L501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -673,45 +681,50 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>veids</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>pieteicejs_reg_nr</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>m1_kadastra_dati</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>m2_adreses_atbilstiba</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>m3_aizsargajama_daba</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>m4_pludi_10_gadi</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>m5_buvniecibas_lietas</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>m6_apgrutinajumi</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>parbaudes_datums</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>avots_piezimes</t>
         </is>
@@ -730,41 +743,46 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
+          <t>īpašums</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
           <t>90000077325</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="J2" s="7" t="n"/>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="7" t="n"/>
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>Piemērs no sākotnējiem datiem: Daugavpils, Tautas iela 11. Atbildes aizpilda kolēģis.</t>
         </is>
@@ -782,38 +800,39 @@
         </is>
       </c>
       <c r="C3" s="5" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="J3" s="7" t="n"/>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="7" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Piemērs no sākotnējiem datiem: Jelgava. Atbildes aizpilda kolēģis.</t>
         </is>
@@ -823,2994 +842,3495 @@
       <c r="A4" s="8" t="n"/>
       <c r="B4" s="8" t="n"/>
       <c r="C4" s="8" t="n"/>
-      <c r="J4" s="9" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="K4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="n"/>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="J5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="K5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
-      <c r="J6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="K6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
       <c r="B7" s="8" t="n"/>
       <c r="C7" s="8" t="n"/>
-      <c r="J7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="K7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
-      <c r="J8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="K8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="n"/>
       <c r="C9" s="8" t="n"/>
-      <c r="J9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="K9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
-      <c r="J10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="K10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
-      <c r="J11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="K11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="J12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="K12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="8" t="n"/>
       <c r="C13" s="8" t="n"/>
-      <c r="J13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="K13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
-      <c r="J14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="K14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
       <c r="B15" s="8" t="n"/>
       <c r="C15" s="8" t="n"/>
-      <c r="J15" s="9" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="K15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="8" t="n"/>
       <c r="C16" s="8" t="n"/>
-      <c r="J16" s="9" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="K16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
-      <c r="J17" s="9" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="K17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="8" t="n"/>
       <c r="C18" s="8" t="n"/>
-      <c r="J18" s="9" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="K18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="8" t="n"/>
-      <c r="J19" s="9" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="K19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="8" t="n"/>
       <c r="C20" s="8" t="n"/>
-      <c r="J20" s="9" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="K20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
-      <c r="J21" s="9" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="K21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="J22" s="9" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="K22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n"/>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="J23" s="9" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="K23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n"/>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
-      <c r="J24" s="9" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="K24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
-      <c r="J25" s="9" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="K25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n"/>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="J26" s="9" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="K26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n"/>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="J27" s="9" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="K27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n"/>
       <c r="B28" s="8" t="n"/>
       <c r="C28" s="8" t="n"/>
-      <c r="J28" s="9" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="K28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="J29" s="9" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="K29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="8" t="n"/>
-      <c r="J30" s="9" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="K30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="J31" s="9" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="K31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
-      <c r="J32" s="9" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="K32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="J33" s="9" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="K33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="J34" s="9" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="K34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
       <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
-      <c r="J35" s="9" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="K35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
       <c r="B36" s="8" t="n"/>
       <c r="C36" s="8" t="n"/>
-      <c r="J36" s="9" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="K36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
       <c r="B37" s="8" t="n"/>
       <c r="C37" s="8" t="n"/>
-      <c r="J37" s="9" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="K37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="8" t="n"/>
       <c r="C38" s="8" t="n"/>
-      <c r="J38" s="9" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="K38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
       <c r="B39" s="8" t="n"/>
       <c r="C39" s="8" t="n"/>
-      <c r="J39" s="9" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="K39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="8" t="n"/>
       <c r="C40" s="8" t="n"/>
-      <c r="J40" s="9" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="K40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
       <c r="B41" s="8" t="n"/>
       <c r="C41" s="8" t="n"/>
-      <c r="J41" s="9" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="K41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
       <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
-      <c r="J42" s="9" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="K42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
       <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="J43" s="9" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="K43" s="9" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
       <c r="B44" s="8" t="n"/>
       <c r="C44" s="8" t="n"/>
-      <c r="J44" s="9" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="K44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
       <c r="B45" s="8" t="n"/>
       <c r="C45" s="8" t="n"/>
-      <c r="J45" s="9" t="n"/>
+      <c r="D45" s="8" t="n"/>
+      <c r="K45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n"/>
       <c r="B46" s="8" t="n"/>
       <c r="C46" s="8" t="n"/>
-      <c r="J46" s="9" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="K46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
       <c r="B47" s="8" t="n"/>
       <c r="C47" s="8" t="n"/>
-      <c r="J47" s="9" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="K47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
       <c r="B48" s="8" t="n"/>
       <c r="C48" s="8" t="n"/>
-      <c r="J48" s="9" t="n"/>
+      <c r="D48" s="8" t="n"/>
+      <c r="K48" s="9" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
       <c r="B49" s="8" t="n"/>
       <c r="C49" s="8" t="n"/>
-      <c r="J49" s="9" t="n"/>
+      <c r="D49" s="8" t="n"/>
+      <c r="K49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n"/>
       <c r="B50" s="8" t="n"/>
       <c r="C50" s="8" t="n"/>
-      <c r="J50" s="9" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="K50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
       <c r="B51" s="8" t="n"/>
       <c r="C51" s="8" t="n"/>
-      <c r="J51" s="9" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="K51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="8" t="n"/>
-      <c r="J52" s="9" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="K52" s="9" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="8" t="n"/>
-      <c r="J53" s="9" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="K53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n"/>
       <c r="B54" s="8" t="n"/>
       <c r="C54" s="8" t="n"/>
-      <c r="J54" s="9" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="K54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
       <c r="B55" s="8" t="n"/>
       <c r="C55" s="8" t="n"/>
-      <c r="J55" s="9" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="K55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n"/>
       <c r="B56" s="8" t="n"/>
       <c r="C56" s="8" t="n"/>
-      <c r="J56" s="9" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="K56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="8" t="n"/>
       <c r="C57" s="8" t="n"/>
-      <c r="J57" s="9" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="K57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n"/>
       <c r="B58" s="8" t="n"/>
       <c r="C58" s="8" t="n"/>
-      <c r="J58" s="9" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="K58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
       <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
-      <c r="J59" s="9" t="n"/>
+      <c r="D59" s="8" t="n"/>
+      <c r="K59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="8" t="n"/>
       <c r="C60" s="8" t="n"/>
-      <c r="J60" s="9" t="n"/>
+      <c r="D60" s="8" t="n"/>
+      <c r="K60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="8" t="n"/>
       <c r="C61" s="8" t="n"/>
-      <c r="J61" s="9" t="n"/>
+      <c r="D61" s="8" t="n"/>
+      <c r="K61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="8" t="n"/>
       <c r="C62" s="8" t="n"/>
-      <c r="J62" s="9" t="n"/>
+      <c r="D62" s="8" t="n"/>
+      <c r="K62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="8" t="n"/>
       <c r="C63" s="8" t="n"/>
-      <c r="J63" s="9" t="n"/>
+      <c r="D63" s="8" t="n"/>
+      <c r="K63" s="9" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n"/>
       <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
-      <c r="J64" s="9" t="n"/>
+      <c r="D64" s="8" t="n"/>
+      <c r="K64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
       <c r="B65" s="8" t="n"/>
       <c r="C65" s="8" t="n"/>
-      <c r="J65" s="9" t="n"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="K65" s="9" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n"/>
       <c r="B66" s="8" t="n"/>
       <c r="C66" s="8" t="n"/>
-      <c r="J66" s="9" t="n"/>
+      <c r="D66" s="8" t="n"/>
+      <c r="K66" s="9" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n"/>
       <c r="B67" s="8" t="n"/>
       <c r="C67" s="8" t="n"/>
-      <c r="J67" s="9" t="n"/>
+      <c r="D67" s="8" t="n"/>
+      <c r="K67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n"/>
       <c r="B68" s="8" t="n"/>
       <c r="C68" s="8" t="n"/>
-      <c r="J68" s="9" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="K68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
       <c r="B69" s="8" t="n"/>
       <c r="C69" s="8" t="n"/>
-      <c r="J69" s="9" t="n"/>
+      <c r="D69" s="8" t="n"/>
+      <c r="K69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n"/>
       <c r="B70" s="8" t="n"/>
       <c r="C70" s="8" t="n"/>
-      <c r="J70" s="9" t="n"/>
+      <c r="D70" s="8" t="n"/>
+      <c r="K70" s="9" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
       <c r="B71" s="8" t="n"/>
       <c r="C71" s="8" t="n"/>
-      <c r="J71" s="9" t="n"/>
+      <c r="D71" s="8" t="n"/>
+      <c r="K71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n"/>
       <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
-      <c r="J72" s="9" t="n"/>
+      <c r="D72" s="8" t="n"/>
+      <c r="K72" s="9" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
       <c r="B73" s="8" t="n"/>
       <c r="C73" s="8" t="n"/>
-      <c r="J73" s="9" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="K73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n"/>
       <c r="B74" s="8" t="n"/>
       <c r="C74" s="8" t="n"/>
-      <c r="J74" s="9" t="n"/>
+      <c r="D74" s="8" t="n"/>
+      <c r="K74" s="9" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n"/>
       <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
-      <c r="J75" s="9" t="n"/>
+      <c r="D75" s="8" t="n"/>
+      <c r="K75" s="9" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n"/>
       <c r="B76" s="8" t="n"/>
       <c r="C76" s="8" t="n"/>
-      <c r="J76" s="9" t="n"/>
+      <c r="D76" s="8" t="n"/>
+      <c r="K76" s="9" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n"/>
       <c r="B77" s="8" t="n"/>
       <c r="C77" s="8" t="n"/>
-      <c r="J77" s="9" t="n"/>
+      <c r="D77" s="8" t="n"/>
+      <c r="K77" s="9" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n"/>
       <c r="B78" s="8" t="n"/>
       <c r="C78" s="8" t="n"/>
-      <c r="J78" s="9" t="n"/>
+      <c r="D78" s="8" t="n"/>
+      <c r="K78" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n"/>
       <c r="B79" s="8" t="n"/>
       <c r="C79" s="8" t="n"/>
-      <c r="J79" s="9" t="n"/>
+      <c r="D79" s="8" t="n"/>
+      <c r="K79" s="9" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n"/>
       <c r="B80" s="8" t="n"/>
       <c r="C80" s="8" t="n"/>
-      <c r="J80" s="9" t="n"/>
+      <c r="D80" s="8" t="n"/>
+      <c r="K80" s="9" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n"/>
       <c r="B81" s="8" t="n"/>
       <c r="C81" s="8" t="n"/>
-      <c r="J81" s="9" t="n"/>
+      <c r="D81" s="8" t="n"/>
+      <c r="K81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n"/>
       <c r="B82" s="8" t="n"/>
       <c r="C82" s="8" t="n"/>
-      <c r="J82" s="9" t="n"/>
+      <c r="D82" s="8" t="n"/>
+      <c r="K82" s="9" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n"/>
       <c r="B83" s="8" t="n"/>
       <c r="C83" s="8" t="n"/>
-      <c r="J83" s="9" t="n"/>
+      <c r="D83" s="8" t="n"/>
+      <c r="K83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n"/>
       <c r="B84" s="8" t="n"/>
       <c r="C84" s="8" t="n"/>
-      <c r="J84" s="9" t="n"/>
+      <c r="D84" s="8" t="n"/>
+      <c r="K84" s="9" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n"/>
       <c r="B85" s="8" t="n"/>
       <c r="C85" s="8" t="n"/>
-      <c r="J85" s="9" t="n"/>
+      <c r="D85" s="8" t="n"/>
+      <c r="K85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="8" t="n"/>
       <c r="B86" s="8" t="n"/>
       <c r="C86" s="8" t="n"/>
-      <c r="J86" s="9" t="n"/>
+      <c r="D86" s="8" t="n"/>
+      <c r="K86" s="9" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="8" t="n"/>
       <c r="B87" s="8" t="n"/>
       <c r="C87" s="8" t="n"/>
-      <c r="J87" s="9" t="n"/>
+      <c r="D87" s="8" t="n"/>
+      <c r="K87" s="9" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="8" t="n"/>
       <c r="B88" s="8" t="n"/>
       <c r="C88" s="8" t="n"/>
-      <c r="J88" s="9" t="n"/>
+      <c r="D88" s="8" t="n"/>
+      <c r="K88" s="9" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="8" t="n"/>
       <c r="B89" s="8" t="n"/>
       <c r="C89" s="8" t="n"/>
-      <c r="J89" s="9" t="n"/>
+      <c r="D89" s="8" t="n"/>
+      <c r="K89" s="9" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n"/>
       <c r="B90" s="8" t="n"/>
       <c r="C90" s="8" t="n"/>
-      <c r="J90" s="9" t="n"/>
+      <c r="D90" s="8" t="n"/>
+      <c r="K90" s="9" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n"/>
       <c r="B91" s="8" t="n"/>
       <c r="C91" s="8" t="n"/>
-      <c r="J91" s="9" t="n"/>
+      <c r="D91" s="8" t="n"/>
+      <c r="K91" s="9" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n"/>
       <c r="B92" s="8" t="n"/>
       <c r="C92" s="8" t="n"/>
-      <c r="J92" s="9" t="n"/>
+      <c r="D92" s="8" t="n"/>
+      <c r="K92" s="9" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n"/>
       <c r="B93" s="8" t="n"/>
       <c r="C93" s="8" t="n"/>
-      <c r="J93" s="9" t="n"/>
+      <c r="D93" s="8" t="n"/>
+      <c r="K93" s="9" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n"/>
       <c r="B94" s="8" t="n"/>
       <c r="C94" s="8" t="n"/>
-      <c r="J94" s="9" t="n"/>
+      <c r="D94" s="8" t="n"/>
+      <c r="K94" s="9" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n"/>
       <c r="B95" s="8" t="n"/>
       <c r="C95" s="8" t="n"/>
-      <c r="J95" s="9" t="n"/>
+      <c r="D95" s="8" t="n"/>
+      <c r="K95" s="9" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n"/>
       <c r="B96" s="8" t="n"/>
       <c r="C96" s="8" t="n"/>
-      <c r="J96" s="9" t="n"/>
+      <c r="D96" s="8" t="n"/>
+      <c r="K96" s="9" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n"/>
       <c r="B97" s="8" t="n"/>
       <c r="C97" s="8" t="n"/>
-      <c r="J97" s="9" t="n"/>
+      <c r="D97" s="8" t="n"/>
+      <c r="K97" s="9" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n"/>
       <c r="B98" s="8" t="n"/>
       <c r="C98" s="8" t="n"/>
-      <c r="J98" s="9" t="n"/>
+      <c r="D98" s="8" t="n"/>
+      <c r="K98" s="9" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n"/>
       <c r="B99" s="8" t="n"/>
       <c r="C99" s="8" t="n"/>
-      <c r="J99" s="9" t="n"/>
+      <c r="D99" s="8" t="n"/>
+      <c r="K99" s="9" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n"/>
       <c r="B100" s="8" t="n"/>
       <c r="C100" s="8" t="n"/>
-      <c r="J100" s="9" t="n"/>
+      <c r="D100" s="8" t="n"/>
+      <c r="K100" s="9" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n"/>
       <c r="B101" s="8" t="n"/>
       <c r="C101" s="8" t="n"/>
-      <c r="J101" s="9" t="n"/>
+      <c r="D101" s="8" t="n"/>
+      <c r="K101" s="9" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n"/>
       <c r="B102" s="8" t="n"/>
       <c r="C102" s="8" t="n"/>
-      <c r="J102" s="9" t="n"/>
+      <c r="D102" s="8" t="n"/>
+      <c r="K102" s="9" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="8" t="n"/>
       <c r="B103" s="8" t="n"/>
       <c r="C103" s="8" t="n"/>
-      <c r="J103" s="9" t="n"/>
+      <c r="D103" s="8" t="n"/>
+      <c r="K103" s="9" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="8" t="n"/>
       <c r="B104" s="8" t="n"/>
       <c r="C104" s="8" t="n"/>
-      <c r="J104" s="9" t="n"/>
+      <c r="D104" s="8" t="n"/>
+      <c r="K104" s="9" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="8" t="n"/>
       <c r="B105" s="8" t="n"/>
       <c r="C105" s="8" t="n"/>
-      <c r="J105" s="9" t="n"/>
+      <c r="D105" s="8" t="n"/>
+      <c r="K105" s="9" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="8" t="n"/>
       <c r="B106" s="8" t="n"/>
       <c r="C106" s="8" t="n"/>
-      <c r="J106" s="9" t="n"/>
+      <c r="D106" s="8" t="n"/>
+      <c r="K106" s="9" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="8" t="n"/>
       <c r="B107" s="8" t="n"/>
       <c r="C107" s="8" t="n"/>
-      <c r="J107" s="9" t="n"/>
+      <c r="D107" s="8" t="n"/>
+      <c r="K107" s="9" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="8" t="n"/>
       <c r="B108" s="8" t="n"/>
       <c r="C108" s="8" t="n"/>
-      <c r="J108" s="9" t="n"/>
+      <c r="D108" s="8" t="n"/>
+      <c r="K108" s="9" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="8" t="n"/>
       <c r="B109" s="8" t="n"/>
       <c r="C109" s="8" t="n"/>
-      <c r="J109" s="9" t="n"/>
+      <c r="D109" s="8" t="n"/>
+      <c r="K109" s="9" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="8" t="n"/>
       <c r="B110" s="8" t="n"/>
       <c r="C110" s="8" t="n"/>
-      <c r="J110" s="9" t="n"/>
+      <c r="D110" s="8" t="n"/>
+      <c r="K110" s="9" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="8" t="n"/>
       <c r="B111" s="8" t="n"/>
       <c r="C111" s="8" t="n"/>
-      <c r="J111" s="9" t="n"/>
+      <c r="D111" s="8" t="n"/>
+      <c r="K111" s="9" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="8" t="n"/>
       <c r="B112" s="8" t="n"/>
       <c r="C112" s="8" t="n"/>
-      <c r="J112" s="9" t="n"/>
+      <c r="D112" s="8" t="n"/>
+      <c r="K112" s="9" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="8" t="n"/>
       <c r="B113" s="8" t="n"/>
       <c r="C113" s="8" t="n"/>
-      <c r="J113" s="9" t="n"/>
+      <c r="D113" s="8" t="n"/>
+      <c r="K113" s="9" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="8" t="n"/>
       <c r="B114" s="8" t="n"/>
       <c r="C114" s="8" t="n"/>
-      <c r="J114" s="9" t="n"/>
+      <c r="D114" s="8" t="n"/>
+      <c r="K114" s="9" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="8" t="n"/>
       <c r="B115" s="8" t="n"/>
       <c r="C115" s="8" t="n"/>
-      <c r="J115" s="9" t="n"/>
+      <c r="D115" s="8" t="n"/>
+      <c r="K115" s="9" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="8" t="n"/>
       <c r="B116" s="8" t="n"/>
       <c r="C116" s="8" t="n"/>
-      <c r="J116" s="9" t="n"/>
+      <c r="D116" s="8" t="n"/>
+      <c r="K116" s="9" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="8" t="n"/>
       <c r="B117" s="8" t="n"/>
       <c r="C117" s="8" t="n"/>
-      <c r="J117" s="9" t="n"/>
+      <c r="D117" s="8" t="n"/>
+      <c r="K117" s="9" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="8" t="n"/>
       <c r="B118" s="8" t="n"/>
       <c r="C118" s="8" t="n"/>
-      <c r="J118" s="9" t="n"/>
+      <c r="D118" s="8" t="n"/>
+      <c r="K118" s="9" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="8" t="n"/>
       <c r="B119" s="8" t="n"/>
       <c r="C119" s="8" t="n"/>
-      <c r="J119" s="9" t="n"/>
+      <c r="D119" s="8" t="n"/>
+      <c r="K119" s="9" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n"/>
       <c r="B120" s="8" t="n"/>
       <c r="C120" s="8" t="n"/>
-      <c r="J120" s="9" t="n"/>
+      <c r="D120" s="8" t="n"/>
+      <c r="K120" s="9" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="8" t="n"/>
       <c r="B121" s="8" t="n"/>
       <c r="C121" s="8" t="n"/>
-      <c r="J121" s="9" t="n"/>
+      <c r="D121" s="8" t="n"/>
+      <c r="K121" s="9" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="8" t="n"/>
       <c r="B122" s="8" t="n"/>
       <c r="C122" s="8" t="n"/>
-      <c r="J122" s="9" t="n"/>
+      <c r="D122" s="8" t="n"/>
+      <c r="K122" s="9" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="8" t="n"/>
       <c r="B123" s="8" t="n"/>
       <c r="C123" s="8" t="n"/>
-      <c r="J123" s="9" t="n"/>
+      <c r="D123" s="8" t="n"/>
+      <c r="K123" s="9" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="8" t="n"/>
       <c r="B124" s="8" t="n"/>
       <c r="C124" s="8" t="n"/>
-      <c r="J124" s="9" t="n"/>
+      <c r="D124" s="8" t="n"/>
+      <c r="K124" s="9" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="8" t="n"/>
       <c r="B125" s="8" t="n"/>
       <c r="C125" s="8" t="n"/>
-      <c r="J125" s="9" t="n"/>
+      <c r="D125" s="8" t="n"/>
+      <c r="K125" s="9" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="8" t="n"/>
       <c r="B126" s="8" t="n"/>
       <c r="C126" s="8" t="n"/>
-      <c r="J126" s="9" t="n"/>
+      <c r="D126" s="8" t="n"/>
+      <c r="K126" s="9" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="8" t="n"/>
       <c r="B127" s="8" t="n"/>
       <c r="C127" s="8" t="n"/>
-      <c r="J127" s="9" t="n"/>
+      <c r="D127" s="8" t="n"/>
+      <c r="K127" s="9" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="8" t="n"/>
       <c r="B128" s="8" t="n"/>
       <c r="C128" s="8" t="n"/>
-      <c r="J128" s="9" t="n"/>
+      <c r="D128" s="8" t="n"/>
+      <c r="K128" s="9" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="8" t="n"/>
       <c r="B129" s="8" t="n"/>
       <c r="C129" s="8" t="n"/>
-      <c r="J129" s="9" t="n"/>
+      <c r="D129" s="8" t="n"/>
+      <c r="K129" s="9" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="8" t="n"/>
       <c r="B130" s="8" t="n"/>
       <c r="C130" s="8" t="n"/>
-      <c r="J130" s="9" t="n"/>
+      <c r="D130" s="8" t="n"/>
+      <c r="K130" s="9" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="8" t="n"/>
       <c r="B131" s="8" t="n"/>
       <c r="C131" s="8" t="n"/>
-      <c r="J131" s="9" t="n"/>
+      <c r="D131" s="8" t="n"/>
+      <c r="K131" s="9" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="8" t="n"/>
       <c r="B132" s="8" t="n"/>
       <c r="C132" s="8" t="n"/>
-      <c r="J132" s="9" t="n"/>
+      <c r="D132" s="8" t="n"/>
+      <c r="K132" s="9" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="8" t="n"/>
       <c r="B133" s="8" t="n"/>
       <c r="C133" s="8" t="n"/>
-      <c r="J133" s="9" t="n"/>
+      <c r="D133" s="8" t="n"/>
+      <c r="K133" s="9" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="8" t="n"/>
       <c r="B134" s="8" t="n"/>
       <c r="C134" s="8" t="n"/>
-      <c r="J134" s="9" t="n"/>
+      <c r="D134" s="8" t="n"/>
+      <c r="K134" s="9" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="8" t="n"/>
       <c r="B135" s="8" t="n"/>
       <c r="C135" s="8" t="n"/>
-      <c r="J135" s="9" t="n"/>
+      <c r="D135" s="8" t="n"/>
+      <c r="K135" s="9" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="8" t="n"/>
       <c r="B136" s="8" t="n"/>
       <c r="C136" s="8" t="n"/>
-      <c r="J136" s="9" t="n"/>
+      <c r="D136" s="8" t="n"/>
+      <c r="K136" s="9" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="8" t="n"/>
       <c r="B137" s="8" t="n"/>
       <c r="C137" s="8" t="n"/>
-      <c r="J137" s="9" t="n"/>
+      <c r="D137" s="8" t="n"/>
+      <c r="K137" s="9" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="8" t="n"/>
       <c r="B138" s="8" t="n"/>
       <c r="C138" s="8" t="n"/>
-      <c r="J138" s="9" t="n"/>
+      <c r="D138" s="8" t="n"/>
+      <c r="K138" s="9" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="8" t="n"/>
       <c r="B139" s="8" t="n"/>
       <c r="C139" s="8" t="n"/>
-      <c r="J139" s="9" t="n"/>
+      <c r="D139" s="8" t="n"/>
+      <c r="K139" s="9" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="8" t="n"/>
       <c r="B140" s="8" t="n"/>
       <c r="C140" s="8" t="n"/>
-      <c r="J140" s="9" t="n"/>
+      <c r="D140" s="8" t="n"/>
+      <c r="K140" s="9" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="8" t="n"/>
       <c r="B141" s="8" t="n"/>
       <c r="C141" s="8" t="n"/>
-      <c r="J141" s="9" t="n"/>
+      <c r="D141" s="8" t="n"/>
+      <c r="K141" s="9" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="8" t="n"/>
       <c r="B142" s="8" t="n"/>
       <c r="C142" s="8" t="n"/>
-      <c r="J142" s="9" t="n"/>
+      <c r="D142" s="8" t="n"/>
+      <c r="K142" s="9" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="8" t="n"/>
       <c r="B143" s="8" t="n"/>
       <c r="C143" s="8" t="n"/>
-      <c r="J143" s="9" t="n"/>
+      <c r="D143" s="8" t="n"/>
+      <c r="K143" s="9" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="8" t="n"/>
       <c r="B144" s="8" t="n"/>
       <c r="C144" s="8" t="n"/>
-      <c r="J144" s="9" t="n"/>
+      <c r="D144" s="8" t="n"/>
+      <c r="K144" s="9" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="8" t="n"/>
       <c r="B145" s="8" t="n"/>
       <c r="C145" s="8" t="n"/>
-      <c r="J145" s="9" t="n"/>
+      <c r="D145" s="8" t="n"/>
+      <c r="K145" s="9" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="8" t="n"/>
       <c r="B146" s="8" t="n"/>
       <c r="C146" s="8" t="n"/>
-      <c r="J146" s="9" t="n"/>
+      <c r="D146" s="8" t="n"/>
+      <c r="K146" s="9" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="8" t="n"/>
       <c r="B147" s="8" t="n"/>
       <c r="C147" s="8" t="n"/>
-      <c r="J147" s="9" t="n"/>
+      <c r="D147" s="8" t="n"/>
+      <c r="K147" s="9" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="8" t="n"/>
       <c r="B148" s="8" t="n"/>
       <c r="C148" s="8" t="n"/>
-      <c r="J148" s="9" t="n"/>
+      <c r="D148" s="8" t="n"/>
+      <c r="K148" s="9" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="8" t="n"/>
       <c r="B149" s="8" t="n"/>
       <c r="C149" s="8" t="n"/>
-      <c r="J149" s="9" t="n"/>
+      <c r="D149" s="8" t="n"/>
+      <c r="K149" s="9" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="8" t="n"/>
       <c r="B150" s="8" t="n"/>
       <c r="C150" s="8" t="n"/>
-      <c r="J150" s="9" t="n"/>
+      <c r="D150" s="8" t="n"/>
+      <c r="K150" s="9" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="8" t="n"/>
       <c r="B151" s="8" t="n"/>
       <c r="C151" s="8" t="n"/>
-      <c r="J151" s="9" t="n"/>
+      <c r="D151" s="8" t="n"/>
+      <c r="K151" s="9" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="8" t="n"/>
       <c r="B152" s="8" t="n"/>
       <c r="C152" s="8" t="n"/>
-      <c r="J152" s="9" t="n"/>
+      <c r="D152" s="8" t="n"/>
+      <c r="K152" s="9" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="8" t="n"/>
       <c r="B153" s="8" t="n"/>
       <c r="C153" s="8" t="n"/>
-      <c r="J153" s="9" t="n"/>
+      <c r="D153" s="8" t="n"/>
+      <c r="K153" s="9" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="8" t="n"/>
       <c r="B154" s="8" t="n"/>
       <c r="C154" s="8" t="n"/>
-      <c r="J154" s="9" t="n"/>
+      <c r="D154" s="8" t="n"/>
+      <c r="K154" s="9" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="8" t="n"/>
       <c r="B155" s="8" t="n"/>
       <c r="C155" s="8" t="n"/>
-      <c r="J155" s="9" t="n"/>
+      <c r="D155" s="8" t="n"/>
+      <c r="K155" s="9" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="8" t="n"/>
       <c r="B156" s="8" t="n"/>
       <c r="C156" s="8" t="n"/>
-      <c r="J156" s="9" t="n"/>
+      <c r="D156" s="8" t="n"/>
+      <c r="K156" s="9" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="8" t="n"/>
       <c r="B157" s="8" t="n"/>
       <c r="C157" s="8" t="n"/>
-      <c r="J157" s="9" t="n"/>
+      <c r="D157" s="8" t="n"/>
+      <c r="K157" s="9" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="8" t="n"/>
       <c r="B158" s="8" t="n"/>
       <c r="C158" s="8" t="n"/>
-      <c r="J158" s="9" t="n"/>
+      <c r="D158" s="8" t="n"/>
+      <c r="K158" s="9" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="8" t="n"/>
       <c r="B159" s="8" t="n"/>
       <c r="C159" s="8" t="n"/>
-      <c r="J159" s="9" t="n"/>
+      <c r="D159" s="8" t="n"/>
+      <c r="K159" s="9" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="8" t="n"/>
       <c r="B160" s="8" t="n"/>
       <c r="C160" s="8" t="n"/>
-      <c r="J160" s="9" t="n"/>
+      <c r="D160" s="8" t="n"/>
+      <c r="K160" s="9" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="8" t="n"/>
       <c r="B161" s="8" t="n"/>
       <c r="C161" s="8" t="n"/>
-      <c r="J161" s="9" t="n"/>
+      <c r="D161" s="8" t="n"/>
+      <c r="K161" s="9" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="8" t="n"/>
       <c r="B162" s="8" t="n"/>
       <c r="C162" s="8" t="n"/>
-      <c r="J162" s="9" t="n"/>
+      <c r="D162" s="8" t="n"/>
+      <c r="K162" s="9" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="8" t="n"/>
       <c r="B163" s="8" t="n"/>
       <c r="C163" s="8" t="n"/>
-      <c r="J163" s="9" t="n"/>
+      <c r="D163" s="8" t="n"/>
+      <c r="K163" s="9" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="8" t="n"/>
       <c r="B164" s="8" t="n"/>
       <c r="C164" s="8" t="n"/>
-      <c r="J164" s="9" t="n"/>
+      <c r="D164" s="8" t="n"/>
+      <c r="K164" s="9" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="8" t="n"/>
       <c r="B165" s="8" t="n"/>
       <c r="C165" s="8" t="n"/>
-      <c r="J165" s="9" t="n"/>
+      <c r="D165" s="8" t="n"/>
+      <c r="K165" s="9" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="8" t="n"/>
       <c r="B166" s="8" t="n"/>
       <c r="C166" s="8" t="n"/>
-      <c r="J166" s="9" t="n"/>
+      <c r="D166" s="8" t="n"/>
+      <c r="K166" s="9" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="8" t="n"/>
       <c r="B167" s="8" t="n"/>
       <c r="C167" s="8" t="n"/>
-      <c r="J167" s="9" t="n"/>
+      <c r="D167" s="8" t="n"/>
+      <c r="K167" s="9" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="8" t="n"/>
       <c r="B168" s="8" t="n"/>
       <c r="C168" s="8" t="n"/>
-      <c r="J168" s="9" t="n"/>
+      <c r="D168" s="8" t="n"/>
+      <c r="K168" s="9" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="8" t="n"/>
       <c r="B169" s="8" t="n"/>
       <c r="C169" s="8" t="n"/>
-      <c r="J169" s="9" t="n"/>
+      <c r="D169" s="8" t="n"/>
+      <c r="K169" s="9" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="8" t="n"/>
       <c r="B170" s="8" t="n"/>
       <c r="C170" s="8" t="n"/>
-      <c r="J170" s="9" t="n"/>
+      <c r="D170" s="8" t="n"/>
+      <c r="K170" s="9" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="8" t="n"/>
       <c r="B171" s="8" t="n"/>
       <c r="C171" s="8" t="n"/>
-      <c r="J171" s="9" t="n"/>
+      <c r="D171" s="8" t="n"/>
+      <c r="K171" s="9" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="8" t="n"/>
       <c r="B172" s="8" t="n"/>
       <c r="C172" s="8" t="n"/>
-      <c r="J172" s="9" t="n"/>
+      <c r="D172" s="8" t="n"/>
+      <c r="K172" s="9" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="8" t="n"/>
       <c r="B173" s="8" t="n"/>
       <c r="C173" s="8" t="n"/>
-      <c r="J173" s="9" t="n"/>
+      <c r="D173" s="8" t="n"/>
+      <c r="K173" s="9" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="8" t="n"/>
       <c r="B174" s="8" t="n"/>
       <c r="C174" s="8" t="n"/>
-      <c r="J174" s="9" t="n"/>
+      <c r="D174" s="8" t="n"/>
+      <c r="K174" s="9" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="8" t="n"/>
       <c r="B175" s="8" t="n"/>
       <c r="C175" s="8" t="n"/>
-      <c r="J175" s="9" t="n"/>
+      <c r="D175" s="8" t="n"/>
+      <c r="K175" s="9" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="8" t="n"/>
       <c r="B176" s="8" t="n"/>
       <c r="C176" s="8" t="n"/>
-      <c r="J176" s="9" t="n"/>
+      <c r="D176" s="8" t="n"/>
+      <c r="K176" s="9" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="8" t="n"/>
       <c r="B177" s="8" t="n"/>
       <c r="C177" s="8" t="n"/>
-      <c r="J177" s="9" t="n"/>
+      <c r="D177" s="8" t="n"/>
+      <c r="K177" s="9" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="8" t="n"/>
       <c r="B178" s="8" t="n"/>
       <c r="C178" s="8" t="n"/>
-      <c r="J178" s="9" t="n"/>
+      <c r="D178" s="8" t="n"/>
+      <c r="K178" s="9" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="8" t="n"/>
       <c r="B179" s="8" t="n"/>
       <c r="C179" s="8" t="n"/>
-      <c r="J179" s="9" t="n"/>
+      <c r="D179" s="8" t="n"/>
+      <c r="K179" s="9" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="8" t="n"/>
       <c r="B180" s="8" t="n"/>
       <c r="C180" s="8" t="n"/>
-      <c r="J180" s="9" t="n"/>
+      <c r="D180" s="8" t="n"/>
+      <c r="K180" s="9" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="8" t="n"/>
       <c r="B181" s="8" t="n"/>
       <c r="C181" s="8" t="n"/>
-      <c r="J181" s="9" t="n"/>
+      <c r="D181" s="8" t="n"/>
+      <c r="K181" s="9" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="8" t="n"/>
       <c r="B182" s="8" t="n"/>
       <c r="C182" s="8" t="n"/>
-      <c r="J182" s="9" t="n"/>
+      <c r="D182" s="8" t="n"/>
+      <c r="K182" s="9" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="8" t="n"/>
       <c r="B183" s="8" t="n"/>
       <c r="C183" s="8" t="n"/>
-      <c r="J183" s="9" t="n"/>
+      <c r="D183" s="8" t="n"/>
+      <c r="K183" s="9" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="8" t="n"/>
       <c r="B184" s="8" t="n"/>
       <c r="C184" s="8" t="n"/>
-      <c r="J184" s="9" t="n"/>
+      <c r="D184" s="8" t="n"/>
+      <c r="K184" s="9" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="8" t="n"/>
       <c r="B185" s="8" t="n"/>
       <c r="C185" s="8" t="n"/>
-      <c r="J185" s="9" t="n"/>
+      <c r="D185" s="8" t="n"/>
+      <c r="K185" s="9" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="8" t="n"/>
       <c r="B186" s="8" t="n"/>
       <c r="C186" s="8" t="n"/>
-      <c r="J186" s="9" t="n"/>
+      <c r="D186" s="8" t="n"/>
+      <c r="K186" s="9" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="8" t="n"/>
       <c r="B187" s="8" t="n"/>
       <c r="C187" s="8" t="n"/>
-      <c r="J187" s="9" t="n"/>
+      <c r="D187" s="8" t="n"/>
+      <c r="K187" s="9" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="8" t="n"/>
       <c r="B188" s="8" t="n"/>
       <c r="C188" s="8" t="n"/>
-      <c r="J188" s="9" t="n"/>
+      <c r="D188" s="8" t="n"/>
+      <c r="K188" s="9" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="8" t="n"/>
       <c r="B189" s="8" t="n"/>
       <c r="C189" s="8" t="n"/>
-      <c r="J189" s="9" t="n"/>
+      <c r="D189" s="8" t="n"/>
+      <c r="K189" s="9" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="8" t="n"/>
       <c r="B190" s="8" t="n"/>
       <c r="C190" s="8" t="n"/>
-      <c r="J190" s="9" t="n"/>
+      <c r="D190" s="8" t="n"/>
+      <c r="K190" s="9" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="8" t="n"/>
       <c r="B191" s="8" t="n"/>
       <c r="C191" s="8" t="n"/>
-      <c r="J191" s="9" t="n"/>
+      <c r="D191" s="8" t="n"/>
+      <c r="K191" s="9" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="8" t="n"/>
       <c r="B192" s="8" t="n"/>
       <c r="C192" s="8" t="n"/>
-      <c r="J192" s="9" t="n"/>
+      <c r="D192" s="8" t="n"/>
+      <c r="K192" s="9" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="8" t="n"/>
       <c r="B193" s="8" t="n"/>
       <c r="C193" s="8" t="n"/>
-      <c r="J193" s="9" t="n"/>
+      <c r="D193" s="8" t="n"/>
+      <c r="K193" s="9" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="8" t="n"/>
       <c r="B194" s="8" t="n"/>
       <c r="C194" s="8" t="n"/>
-      <c r="J194" s="9" t="n"/>
+      <c r="D194" s="8" t="n"/>
+      <c r="K194" s="9" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="8" t="n"/>
       <c r="B195" s="8" t="n"/>
       <c r="C195" s="8" t="n"/>
-      <c r="J195" s="9" t="n"/>
+      <c r="D195" s="8" t="n"/>
+      <c r="K195" s="9" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="8" t="n"/>
       <c r="B196" s="8" t="n"/>
       <c r="C196" s="8" t="n"/>
-      <c r="J196" s="9" t="n"/>
+      <c r="D196" s="8" t="n"/>
+      <c r="K196" s="9" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="8" t="n"/>
       <c r="B197" s="8" t="n"/>
       <c r="C197" s="8" t="n"/>
-      <c r="J197" s="9" t="n"/>
+      <c r="D197" s="8" t="n"/>
+      <c r="K197" s="9" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="8" t="n"/>
       <c r="B198" s="8" t="n"/>
       <c r="C198" s="8" t="n"/>
-      <c r="J198" s="9" t="n"/>
+      <c r="D198" s="8" t="n"/>
+      <c r="K198" s="9" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="8" t="n"/>
       <c r="B199" s="8" t="n"/>
       <c r="C199" s="8" t="n"/>
-      <c r="J199" s="9" t="n"/>
+      <c r="D199" s="8" t="n"/>
+      <c r="K199" s="9" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="8" t="n"/>
       <c r="B200" s="8" t="n"/>
       <c r="C200" s="8" t="n"/>
-      <c r="J200" s="9" t="n"/>
+      <c r="D200" s="8" t="n"/>
+      <c r="K200" s="9" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="8" t="n"/>
       <c r="B201" s="8" t="n"/>
       <c r="C201" s="8" t="n"/>
-      <c r="J201" s="9" t="n"/>
+      <c r="D201" s="8" t="n"/>
+      <c r="K201" s="9" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="8" t="n"/>
       <c r="B202" s="8" t="n"/>
       <c r="C202" s="8" t="n"/>
-      <c r="J202" s="9" t="n"/>
+      <c r="D202" s="8" t="n"/>
+      <c r="K202" s="9" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="8" t="n"/>
       <c r="B203" s="8" t="n"/>
       <c r="C203" s="8" t="n"/>
-      <c r="J203" s="9" t="n"/>
+      <c r="D203" s="8" t="n"/>
+      <c r="K203" s="9" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="8" t="n"/>
       <c r="B204" s="8" t="n"/>
       <c r="C204" s="8" t="n"/>
-      <c r="J204" s="9" t="n"/>
+      <c r="D204" s="8" t="n"/>
+      <c r="K204" s="9" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="8" t="n"/>
       <c r="B205" s="8" t="n"/>
       <c r="C205" s="8" t="n"/>
-      <c r="J205" s="9" t="n"/>
+      <c r="D205" s="8" t="n"/>
+      <c r="K205" s="9" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="8" t="n"/>
       <c r="B206" s="8" t="n"/>
       <c r="C206" s="8" t="n"/>
-      <c r="J206" s="9" t="n"/>
+      <c r="D206" s="8" t="n"/>
+      <c r="K206" s="9" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="8" t="n"/>
       <c r="B207" s="8" t="n"/>
       <c r="C207" s="8" t="n"/>
-      <c r="J207" s="9" t="n"/>
+      <c r="D207" s="8" t="n"/>
+      <c r="K207" s="9" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="8" t="n"/>
       <c r="B208" s="8" t="n"/>
       <c r="C208" s="8" t="n"/>
-      <c r="J208" s="9" t="n"/>
+      <c r="D208" s="8" t="n"/>
+      <c r="K208" s="9" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="8" t="n"/>
       <c r="B209" s="8" t="n"/>
       <c r="C209" s="8" t="n"/>
-      <c r="J209" s="9" t="n"/>
+      <c r="D209" s="8" t="n"/>
+      <c r="K209" s="9" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="8" t="n"/>
       <c r="B210" s="8" t="n"/>
       <c r="C210" s="8" t="n"/>
-      <c r="J210" s="9" t="n"/>
+      <c r="D210" s="8" t="n"/>
+      <c r="K210" s="9" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="8" t="n"/>
       <c r="B211" s="8" t="n"/>
       <c r="C211" s="8" t="n"/>
-      <c r="J211" s="9" t="n"/>
+      <c r="D211" s="8" t="n"/>
+      <c r="K211" s="9" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="8" t="n"/>
       <c r="B212" s="8" t="n"/>
       <c r="C212" s="8" t="n"/>
-      <c r="J212" s="9" t="n"/>
+      <c r="D212" s="8" t="n"/>
+      <c r="K212" s="9" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="8" t="n"/>
       <c r="B213" s="8" t="n"/>
       <c r="C213" s="8" t="n"/>
-      <c r="J213" s="9" t="n"/>
+      <c r="D213" s="8" t="n"/>
+      <c r="K213" s="9" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="8" t="n"/>
       <c r="B214" s="8" t="n"/>
       <c r="C214" s="8" t="n"/>
-      <c r="J214" s="9" t="n"/>
+      <c r="D214" s="8" t="n"/>
+      <c r="K214" s="9" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="8" t="n"/>
       <c r="B215" s="8" t="n"/>
       <c r="C215" s="8" t="n"/>
-      <c r="J215" s="9" t="n"/>
+      <c r="D215" s="8" t="n"/>
+      <c r="K215" s="9" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="8" t="n"/>
       <c r="B216" s="8" t="n"/>
       <c r="C216" s="8" t="n"/>
-      <c r="J216" s="9" t="n"/>
+      <c r="D216" s="8" t="n"/>
+      <c r="K216" s="9" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="8" t="n"/>
       <c r="B217" s="8" t="n"/>
       <c r="C217" s="8" t="n"/>
-      <c r="J217" s="9" t="n"/>
+      <c r="D217" s="8" t="n"/>
+      <c r="K217" s="9" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="8" t="n"/>
       <c r="B218" s="8" t="n"/>
       <c r="C218" s="8" t="n"/>
-      <c r="J218" s="9" t="n"/>
+      <c r="D218" s="8" t="n"/>
+      <c r="K218" s="9" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="8" t="n"/>
       <c r="B219" s="8" t="n"/>
       <c r="C219" s="8" t="n"/>
-      <c r="J219" s="9" t="n"/>
+      <c r="D219" s="8" t="n"/>
+      <c r="K219" s="9" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="8" t="n"/>
       <c r="B220" s="8" t="n"/>
       <c r="C220" s="8" t="n"/>
-      <c r="J220" s="9" t="n"/>
+      <c r="D220" s="8" t="n"/>
+      <c r="K220" s="9" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="8" t="n"/>
       <c r="B221" s="8" t="n"/>
       <c r="C221" s="8" t="n"/>
-      <c r="J221" s="9" t="n"/>
+      <c r="D221" s="8" t="n"/>
+      <c r="K221" s="9" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="8" t="n"/>
       <c r="B222" s="8" t="n"/>
       <c r="C222" s="8" t="n"/>
-      <c r="J222" s="9" t="n"/>
+      <c r="D222" s="8" t="n"/>
+      <c r="K222" s="9" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="8" t="n"/>
       <c r="B223" s="8" t="n"/>
       <c r="C223" s="8" t="n"/>
-      <c r="J223" s="9" t="n"/>
+      <c r="D223" s="8" t="n"/>
+      <c r="K223" s="9" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="8" t="n"/>
       <c r="B224" s="8" t="n"/>
       <c r="C224" s="8" t="n"/>
-      <c r="J224" s="9" t="n"/>
+      <c r="D224" s="8" t="n"/>
+      <c r="K224" s="9" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="8" t="n"/>
       <c r="B225" s="8" t="n"/>
       <c r="C225" s="8" t="n"/>
-      <c r="J225" s="9" t="n"/>
+      <c r="D225" s="8" t="n"/>
+      <c r="K225" s="9" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="8" t="n"/>
       <c r="B226" s="8" t="n"/>
       <c r="C226" s="8" t="n"/>
-      <c r="J226" s="9" t="n"/>
+      <c r="D226" s="8" t="n"/>
+      <c r="K226" s="9" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="8" t="n"/>
       <c r="B227" s="8" t="n"/>
       <c r="C227" s="8" t="n"/>
-      <c r="J227" s="9" t="n"/>
+      <c r="D227" s="8" t="n"/>
+      <c r="K227" s="9" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="8" t="n"/>
       <c r="B228" s="8" t="n"/>
       <c r="C228" s="8" t="n"/>
-      <c r="J228" s="9" t="n"/>
+      <c r="D228" s="8" t="n"/>
+      <c r="K228" s="9" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="8" t="n"/>
       <c r="B229" s="8" t="n"/>
       <c r="C229" s="8" t="n"/>
-      <c r="J229" s="9" t="n"/>
+      <c r="D229" s="8" t="n"/>
+      <c r="K229" s="9" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="8" t="n"/>
       <c r="B230" s="8" t="n"/>
       <c r="C230" s="8" t="n"/>
-      <c r="J230" s="9" t="n"/>
+      <c r="D230" s="8" t="n"/>
+      <c r="K230" s="9" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="8" t="n"/>
       <c r="B231" s="8" t="n"/>
       <c r="C231" s="8" t="n"/>
-      <c r="J231" s="9" t="n"/>
+      <c r="D231" s="8" t="n"/>
+      <c r="K231" s="9" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="8" t="n"/>
       <c r="B232" s="8" t="n"/>
       <c r="C232" s="8" t="n"/>
-      <c r="J232" s="9" t="n"/>
+      <c r="D232" s="8" t="n"/>
+      <c r="K232" s="9" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="8" t="n"/>
       <c r="B233" s="8" t="n"/>
       <c r="C233" s="8" t="n"/>
-      <c r="J233" s="9" t="n"/>
+      <c r="D233" s="8" t="n"/>
+      <c r="K233" s="9" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="8" t="n"/>
       <c r="B234" s="8" t="n"/>
       <c r="C234" s="8" t="n"/>
-      <c r="J234" s="9" t="n"/>
+      <c r="D234" s="8" t="n"/>
+      <c r="K234" s="9" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="8" t="n"/>
       <c r="B235" s="8" t="n"/>
       <c r="C235" s="8" t="n"/>
-      <c r="J235" s="9" t="n"/>
+      <c r="D235" s="8" t="n"/>
+      <c r="K235" s="9" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="8" t="n"/>
       <c r="B236" s="8" t="n"/>
       <c r="C236" s="8" t="n"/>
-      <c r="J236" s="9" t="n"/>
+      <c r="D236" s="8" t="n"/>
+      <c r="K236" s="9" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="8" t="n"/>
       <c r="B237" s="8" t="n"/>
       <c r="C237" s="8" t="n"/>
-      <c r="J237" s="9" t="n"/>
+      <c r="D237" s="8" t="n"/>
+      <c r="K237" s="9" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="8" t="n"/>
       <c r="B238" s="8" t="n"/>
       <c r="C238" s="8" t="n"/>
-      <c r="J238" s="9" t="n"/>
+      <c r="D238" s="8" t="n"/>
+      <c r="K238" s="9" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="8" t="n"/>
       <c r="B239" s="8" t="n"/>
       <c r="C239" s="8" t="n"/>
-      <c r="J239" s="9" t="n"/>
+      <c r="D239" s="8" t="n"/>
+      <c r="K239" s="9" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="8" t="n"/>
       <c r="B240" s="8" t="n"/>
       <c r="C240" s="8" t="n"/>
-      <c r="J240" s="9" t="n"/>
+      <c r="D240" s="8" t="n"/>
+      <c r="K240" s="9" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="8" t="n"/>
       <c r="B241" s="8" t="n"/>
       <c r="C241" s="8" t="n"/>
-      <c r="J241" s="9" t="n"/>
+      <c r="D241" s="8" t="n"/>
+      <c r="K241" s="9" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="8" t="n"/>
       <c r="B242" s="8" t="n"/>
       <c r="C242" s="8" t="n"/>
-      <c r="J242" s="9" t="n"/>
+      <c r="D242" s="8" t="n"/>
+      <c r="K242" s="9" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="8" t="n"/>
       <c r="B243" s="8" t="n"/>
       <c r="C243" s="8" t="n"/>
-      <c r="J243" s="9" t="n"/>
+      <c r="D243" s="8" t="n"/>
+      <c r="K243" s="9" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="8" t="n"/>
       <c r="B244" s="8" t="n"/>
       <c r="C244" s="8" t="n"/>
-      <c r="J244" s="9" t="n"/>
+      <c r="D244" s="8" t="n"/>
+      <c r="K244" s="9" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="8" t="n"/>
       <c r="B245" s="8" t="n"/>
       <c r="C245" s="8" t="n"/>
-      <c r="J245" s="9" t="n"/>
+      <c r="D245" s="8" t="n"/>
+      <c r="K245" s="9" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="8" t="n"/>
       <c r="B246" s="8" t="n"/>
       <c r="C246" s="8" t="n"/>
-      <c r="J246" s="9" t="n"/>
+      <c r="D246" s="8" t="n"/>
+      <c r="K246" s="9" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="8" t="n"/>
       <c r="B247" s="8" t="n"/>
       <c r="C247" s="8" t="n"/>
-      <c r="J247" s="9" t="n"/>
+      <c r="D247" s="8" t="n"/>
+      <c r="K247" s="9" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="8" t="n"/>
       <c r="B248" s="8" t="n"/>
       <c r="C248" s="8" t="n"/>
-      <c r="J248" s="9" t="n"/>
+      <c r="D248" s="8" t="n"/>
+      <c r="K248" s="9" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="8" t="n"/>
       <c r="B249" s="8" t="n"/>
       <c r="C249" s="8" t="n"/>
-      <c r="J249" s="9" t="n"/>
+      <c r="D249" s="8" t="n"/>
+      <c r="K249" s="9" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="8" t="n"/>
       <c r="B250" s="8" t="n"/>
       <c r="C250" s="8" t="n"/>
-      <c r="J250" s="9" t="n"/>
+      <c r="D250" s="8" t="n"/>
+      <c r="K250" s="9" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="8" t="n"/>
       <c r="B251" s="8" t="n"/>
       <c r="C251" s="8" t="n"/>
-      <c r="J251" s="9" t="n"/>
+      <c r="D251" s="8" t="n"/>
+      <c r="K251" s="9" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="8" t="n"/>
       <c r="B252" s="8" t="n"/>
       <c r="C252" s="8" t="n"/>
-      <c r="J252" s="9" t="n"/>
+      <c r="D252" s="8" t="n"/>
+      <c r="K252" s="9" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="8" t="n"/>
       <c r="B253" s="8" t="n"/>
       <c r="C253" s="8" t="n"/>
-      <c r="J253" s="9" t="n"/>
+      <c r="D253" s="8" t="n"/>
+      <c r="K253" s="9" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="8" t="n"/>
       <c r="B254" s="8" t="n"/>
       <c r="C254" s="8" t="n"/>
-      <c r="J254" s="9" t="n"/>
+      <c r="D254" s="8" t="n"/>
+      <c r="K254" s="9" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="8" t="n"/>
       <c r="B255" s="8" t="n"/>
       <c r="C255" s="8" t="n"/>
-      <c r="J255" s="9" t="n"/>
+      <c r="D255" s="8" t="n"/>
+      <c r="K255" s="9" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="8" t="n"/>
       <c r="B256" s="8" t="n"/>
       <c r="C256" s="8" t="n"/>
-      <c r="J256" s="9" t="n"/>
+      <c r="D256" s="8" t="n"/>
+      <c r="K256" s="9" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="8" t="n"/>
       <c r="B257" s="8" t="n"/>
       <c r="C257" s="8" t="n"/>
-      <c r="J257" s="9" t="n"/>
+      <c r="D257" s="8" t="n"/>
+      <c r="K257" s="9" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="8" t="n"/>
       <c r="B258" s="8" t="n"/>
       <c r="C258" s="8" t="n"/>
-      <c r="J258" s="9" t="n"/>
+      <c r="D258" s="8" t="n"/>
+      <c r="K258" s="9" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="8" t="n"/>
       <c r="B259" s="8" t="n"/>
       <c r="C259" s="8" t="n"/>
-      <c r="J259" s="9" t="n"/>
+      <c r="D259" s="8" t="n"/>
+      <c r="K259" s="9" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="8" t="n"/>
       <c r="B260" s="8" t="n"/>
       <c r="C260" s="8" t="n"/>
-      <c r="J260" s="9" t="n"/>
+      <c r="D260" s="8" t="n"/>
+      <c r="K260" s="9" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="8" t="n"/>
       <c r="B261" s="8" t="n"/>
       <c r="C261" s="8" t="n"/>
-      <c r="J261" s="9" t="n"/>
+      <c r="D261" s="8" t="n"/>
+      <c r="K261" s="9" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="8" t="n"/>
       <c r="B262" s="8" t="n"/>
       <c r="C262" s="8" t="n"/>
-      <c r="J262" s="9" t="n"/>
+      <c r="D262" s="8" t="n"/>
+      <c r="K262" s="9" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="8" t="n"/>
       <c r="B263" s="8" t="n"/>
       <c r="C263" s="8" t="n"/>
-      <c r="J263" s="9" t="n"/>
+      <c r="D263" s="8" t="n"/>
+      <c r="K263" s="9" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="8" t="n"/>
       <c r="B264" s="8" t="n"/>
       <c r="C264" s="8" t="n"/>
-      <c r="J264" s="9" t="n"/>
+      <c r="D264" s="8" t="n"/>
+      <c r="K264" s="9" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="8" t="n"/>
       <c r="B265" s="8" t="n"/>
       <c r="C265" s="8" t="n"/>
-      <c r="J265" s="9" t="n"/>
+      <c r="D265" s="8" t="n"/>
+      <c r="K265" s="9" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="8" t="n"/>
       <c r="B266" s="8" t="n"/>
       <c r="C266" s="8" t="n"/>
-      <c r="J266" s="9" t="n"/>
+      <c r="D266" s="8" t="n"/>
+      <c r="K266" s="9" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="8" t="n"/>
       <c r="B267" s="8" t="n"/>
       <c r="C267" s="8" t="n"/>
-      <c r="J267" s="9" t="n"/>
+      <c r="D267" s="8" t="n"/>
+      <c r="K267" s="9" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="8" t="n"/>
       <c r="B268" s="8" t="n"/>
       <c r="C268" s="8" t="n"/>
-      <c r="J268" s="9" t="n"/>
+      <c r="D268" s="8" t="n"/>
+      <c r="K268" s="9" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="8" t="n"/>
       <c r="B269" s="8" t="n"/>
       <c r="C269" s="8" t="n"/>
-      <c r="J269" s="9" t="n"/>
+      <c r="D269" s="8" t="n"/>
+      <c r="K269" s="9" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="8" t="n"/>
       <c r="B270" s="8" t="n"/>
       <c r="C270" s="8" t="n"/>
-      <c r="J270" s="9" t="n"/>
+      <c r="D270" s="8" t="n"/>
+      <c r="K270" s="9" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="8" t="n"/>
       <c r="B271" s="8" t="n"/>
       <c r="C271" s="8" t="n"/>
-      <c r="J271" s="9" t="n"/>
+      <c r="D271" s="8" t="n"/>
+      <c r="K271" s="9" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="8" t="n"/>
       <c r="B272" s="8" t="n"/>
       <c r="C272" s="8" t="n"/>
-      <c r="J272" s="9" t="n"/>
+      <c r="D272" s="8" t="n"/>
+      <c r="K272" s="9" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="8" t="n"/>
       <c r="B273" s="8" t="n"/>
       <c r="C273" s="8" t="n"/>
-      <c r="J273" s="9" t="n"/>
+      <c r="D273" s="8" t="n"/>
+      <c r="K273" s="9" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="8" t="n"/>
       <c r="B274" s="8" t="n"/>
       <c r="C274" s="8" t="n"/>
-      <c r="J274" s="9" t="n"/>
+      <c r="D274" s="8" t="n"/>
+      <c r="K274" s="9" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="8" t="n"/>
       <c r="B275" s="8" t="n"/>
       <c r="C275" s="8" t="n"/>
-      <c r="J275" s="9" t="n"/>
+      <c r="D275" s="8" t="n"/>
+      <c r="K275" s="9" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="8" t="n"/>
       <c r="B276" s="8" t="n"/>
       <c r="C276" s="8" t="n"/>
-      <c r="J276" s="9" t="n"/>
+      <c r="D276" s="8" t="n"/>
+      <c r="K276" s="9" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="8" t="n"/>
       <c r="B277" s="8" t="n"/>
       <c r="C277" s="8" t="n"/>
-      <c r="J277" s="9" t="n"/>
+      <c r="D277" s="8" t="n"/>
+      <c r="K277" s="9" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="8" t="n"/>
       <c r="B278" s="8" t="n"/>
       <c r="C278" s="8" t="n"/>
-      <c r="J278" s="9" t="n"/>
+      <c r="D278" s="8" t="n"/>
+      <c r="K278" s="9" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="8" t="n"/>
       <c r="B279" s="8" t="n"/>
       <c r="C279" s="8" t="n"/>
-      <c r="J279" s="9" t="n"/>
+      <c r="D279" s="8" t="n"/>
+      <c r="K279" s="9" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="8" t="n"/>
       <c r="B280" s="8" t="n"/>
       <c r="C280" s="8" t="n"/>
-      <c r="J280" s="9" t="n"/>
+      <c r="D280" s="8" t="n"/>
+      <c r="K280" s="9" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="8" t="n"/>
       <c r="B281" s="8" t="n"/>
       <c r="C281" s="8" t="n"/>
-      <c r="J281" s="9" t="n"/>
+      <c r="D281" s="8" t="n"/>
+      <c r="K281" s="9" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="8" t="n"/>
       <c r="B282" s="8" t="n"/>
       <c r="C282" s="8" t="n"/>
-      <c r="J282" s="9" t="n"/>
+      <c r="D282" s="8" t="n"/>
+      <c r="K282" s="9" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="8" t="n"/>
       <c r="B283" s="8" t="n"/>
       <c r="C283" s="8" t="n"/>
-      <c r="J283" s="9" t="n"/>
+      <c r="D283" s="8" t="n"/>
+      <c r="K283" s="9" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="8" t="n"/>
       <c r="B284" s="8" t="n"/>
       <c r="C284" s="8" t="n"/>
-      <c r="J284" s="9" t="n"/>
+      <c r="D284" s="8" t="n"/>
+      <c r="K284" s="9" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="8" t="n"/>
       <c r="B285" s="8" t="n"/>
       <c r="C285" s="8" t="n"/>
-      <c r="J285" s="9" t="n"/>
+      <c r="D285" s="8" t="n"/>
+      <c r="K285" s="9" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="8" t="n"/>
       <c r="B286" s="8" t="n"/>
       <c r="C286" s="8" t="n"/>
-      <c r="J286" s="9" t="n"/>
+      <c r="D286" s="8" t="n"/>
+      <c r="K286" s="9" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="8" t="n"/>
       <c r="B287" s="8" t="n"/>
       <c r="C287" s="8" t="n"/>
-      <c r="J287" s="9" t="n"/>
+      <c r="D287" s="8" t="n"/>
+      <c r="K287" s="9" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="8" t="n"/>
       <c r="B288" s="8" t="n"/>
       <c r="C288" s="8" t="n"/>
-      <c r="J288" s="9" t="n"/>
+      <c r="D288" s="8" t="n"/>
+      <c r="K288" s="9" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="8" t="n"/>
       <c r="B289" s="8" t="n"/>
       <c r="C289" s="8" t="n"/>
-      <c r="J289" s="9" t="n"/>
+      <c r="D289" s="8" t="n"/>
+      <c r="K289" s="9" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="8" t="n"/>
       <c r="B290" s="8" t="n"/>
       <c r="C290" s="8" t="n"/>
-      <c r="J290" s="9" t="n"/>
+      <c r="D290" s="8" t="n"/>
+      <c r="K290" s="9" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="8" t="n"/>
       <c r="B291" s="8" t="n"/>
       <c r="C291" s="8" t="n"/>
-      <c r="J291" s="9" t="n"/>
+      <c r="D291" s="8" t="n"/>
+      <c r="K291" s="9" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="8" t="n"/>
       <c r="B292" s="8" t="n"/>
       <c r="C292" s="8" t="n"/>
-      <c r="J292" s="9" t="n"/>
+      <c r="D292" s="8" t="n"/>
+      <c r="K292" s="9" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="8" t="n"/>
       <c r="B293" s="8" t="n"/>
       <c r="C293" s="8" t="n"/>
-      <c r="J293" s="9" t="n"/>
+      <c r="D293" s="8" t="n"/>
+      <c r="K293" s="9" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="8" t="n"/>
       <c r="B294" s="8" t="n"/>
       <c r="C294" s="8" t="n"/>
-      <c r="J294" s="9" t="n"/>
+      <c r="D294" s="8" t="n"/>
+      <c r="K294" s="9" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="8" t="n"/>
       <c r="B295" s="8" t="n"/>
       <c r="C295" s="8" t="n"/>
-      <c r="J295" s="9" t="n"/>
+      <c r="D295" s="8" t="n"/>
+      <c r="K295" s="9" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="8" t="n"/>
       <c r="B296" s="8" t="n"/>
       <c r="C296" s="8" t="n"/>
-      <c r="J296" s="9" t="n"/>
+      <c r="D296" s="8" t="n"/>
+      <c r="K296" s="9" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="8" t="n"/>
       <c r="B297" s="8" t="n"/>
       <c r="C297" s="8" t="n"/>
-      <c r="J297" s="9" t="n"/>
+      <c r="D297" s="8" t="n"/>
+      <c r="K297" s="9" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="8" t="n"/>
       <c r="B298" s="8" t="n"/>
       <c r="C298" s="8" t="n"/>
-      <c r="J298" s="9" t="n"/>
+      <c r="D298" s="8" t="n"/>
+      <c r="K298" s="9" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="8" t="n"/>
       <c r="B299" s="8" t="n"/>
       <c r="C299" s="8" t="n"/>
-      <c r="J299" s="9" t="n"/>
+      <c r="D299" s="8" t="n"/>
+      <c r="K299" s="9" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="8" t="n"/>
       <c r="B300" s="8" t="n"/>
       <c r="C300" s="8" t="n"/>
-      <c r="J300" s="9" t="n"/>
+      <c r="D300" s="8" t="n"/>
+      <c r="K300" s="9" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="8" t="n"/>
       <c r="B301" s="8" t="n"/>
       <c r="C301" s="8" t="n"/>
-      <c r="J301" s="9" t="n"/>
+      <c r="D301" s="8" t="n"/>
+      <c r="K301" s="9" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="8" t="n"/>
       <c r="B302" s="8" t="n"/>
       <c r="C302" s="8" t="n"/>
-      <c r="J302" s="9" t="n"/>
+      <c r="D302" s="8" t="n"/>
+      <c r="K302" s="9" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="8" t="n"/>
       <c r="B303" s="8" t="n"/>
       <c r="C303" s="8" t="n"/>
-      <c r="J303" s="9" t="n"/>
+      <c r="D303" s="8" t="n"/>
+      <c r="K303" s="9" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="8" t="n"/>
       <c r="B304" s="8" t="n"/>
       <c r="C304" s="8" t="n"/>
-      <c r="J304" s="9" t="n"/>
+      <c r="D304" s="8" t="n"/>
+      <c r="K304" s="9" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="8" t="n"/>
       <c r="B305" s="8" t="n"/>
       <c r="C305" s="8" t="n"/>
-      <c r="J305" s="9" t="n"/>
+      <c r="D305" s="8" t="n"/>
+      <c r="K305" s="9" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="8" t="n"/>
       <c r="B306" s="8" t="n"/>
       <c r="C306" s="8" t="n"/>
-      <c r="J306" s="9" t="n"/>
+      <c r="D306" s="8" t="n"/>
+      <c r="K306" s="9" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="8" t="n"/>
       <c r="B307" s="8" t="n"/>
       <c r="C307" s="8" t="n"/>
-      <c r="J307" s="9" t="n"/>
+      <c r="D307" s="8" t="n"/>
+      <c r="K307" s="9" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="8" t="n"/>
       <c r="B308" s="8" t="n"/>
       <c r="C308" s="8" t="n"/>
-      <c r="J308" s="9" t="n"/>
+      <c r="D308" s="8" t="n"/>
+      <c r="K308" s="9" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="8" t="n"/>
       <c r="B309" s="8" t="n"/>
       <c r="C309" s="8" t="n"/>
-      <c r="J309" s="9" t="n"/>
+      <c r="D309" s="8" t="n"/>
+      <c r="K309" s="9" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="8" t="n"/>
       <c r="B310" s="8" t="n"/>
       <c r="C310" s="8" t="n"/>
-      <c r="J310" s="9" t="n"/>
+      <c r="D310" s="8" t="n"/>
+      <c r="K310" s="9" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="8" t="n"/>
       <c r="B311" s="8" t="n"/>
       <c r="C311" s="8" t="n"/>
-      <c r="J311" s="9" t="n"/>
+      <c r="D311" s="8" t="n"/>
+      <c r="K311" s="9" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="8" t="n"/>
       <c r="B312" s="8" t="n"/>
       <c r="C312" s="8" t="n"/>
-      <c r="J312" s="9" t="n"/>
+      <c r="D312" s="8" t="n"/>
+      <c r="K312" s="9" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="8" t="n"/>
       <c r="B313" s="8" t="n"/>
       <c r="C313" s="8" t="n"/>
-      <c r="J313" s="9" t="n"/>
+      <c r="D313" s="8" t="n"/>
+      <c r="K313" s="9" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="8" t="n"/>
       <c r="B314" s="8" t="n"/>
       <c r="C314" s="8" t="n"/>
-      <c r="J314" s="9" t="n"/>
+      <c r="D314" s="8" t="n"/>
+      <c r="K314" s="9" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="8" t="n"/>
       <c r="B315" s="8" t="n"/>
       <c r="C315" s="8" t="n"/>
-      <c r="J315" s="9" t="n"/>
+      <c r="D315" s="8" t="n"/>
+      <c r="K315" s="9" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="8" t="n"/>
       <c r="B316" s="8" t="n"/>
       <c r="C316" s="8" t="n"/>
-      <c r="J316" s="9" t="n"/>
+      <c r="D316" s="8" t="n"/>
+      <c r="K316" s="9" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="8" t="n"/>
       <c r="B317" s="8" t="n"/>
       <c r="C317" s="8" t="n"/>
-      <c r="J317" s="9" t="n"/>
+      <c r="D317" s="8" t="n"/>
+      <c r="K317" s="9" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="8" t="n"/>
       <c r="B318" s="8" t="n"/>
       <c r="C318" s="8" t="n"/>
-      <c r="J318" s="9" t="n"/>
+      <c r="D318" s="8" t="n"/>
+      <c r="K318" s="9" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="8" t="n"/>
       <c r="B319" s="8" t="n"/>
       <c r="C319" s="8" t="n"/>
-      <c r="J319" s="9" t="n"/>
+      <c r="D319" s="8" t="n"/>
+      <c r="K319" s="9" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="8" t="n"/>
       <c r="B320" s="8" t="n"/>
       <c r="C320" s="8" t="n"/>
-      <c r="J320" s="9" t="n"/>
+      <c r="D320" s="8" t="n"/>
+      <c r="K320" s="9" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="8" t="n"/>
       <c r="B321" s="8" t="n"/>
       <c r="C321" s="8" t="n"/>
-      <c r="J321" s="9" t="n"/>
+      <c r="D321" s="8" t="n"/>
+      <c r="K321" s="9" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="8" t="n"/>
       <c r="B322" s="8" t="n"/>
       <c r="C322" s="8" t="n"/>
-      <c r="J322" s="9" t="n"/>
+      <c r="D322" s="8" t="n"/>
+      <c r="K322" s="9" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="8" t="n"/>
       <c r="B323" s="8" t="n"/>
       <c r="C323" s="8" t="n"/>
-      <c r="J323" s="9" t="n"/>
+      <c r="D323" s="8" t="n"/>
+      <c r="K323" s="9" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="8" t="n"/>
       <c r="B324" s="8" t="n"/>
       <c r="C324" s="8" t="n"/>
-      <c r="J324" s="9" t="n"/>
+      <c r="D324" s="8" t="n"/>
+      <c r="K324" s="9" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="8" t="n"/>
       <c r="B325" s="8" t="n"/>
       <c r="C325" s="8" t="n"/>
-      <c r="J325" s="9" t="n"/>
+      <c r="D325" s="8" t="n"/>
+      <c r="K325" s="9" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="8" t="n"/>
       <c r="B326" s="8" t="n"/>
       <c r="C326" s="8" t="n"/>
-      <c r="J326" s="9" t="n"/>
+      <c r="D326" s="8" t="n"/>
+      <c r="K326" s="9" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="8" t="n"/>
       <c r="B327" s="8" t="n"/>
       <c r="C327" s="8" t="n"/>
-      <c r="J327" s="9" t="n"/>
+      <c r="D327" s="8" t="n"/>
+      <c r="K327" s="9" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="8" t="n"/>
       <c r="B328" s="8" t="n"/>
       <c r="C328" s="8" t="n"/>
-      <c r="J328" s="9" t="n"/>
+      <c r="D328" s="8" t="n"/>
+      <c r="K328" s="9" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="8" t="n"/>
       <c r="B329" s="8" t="n"/>
       <c r="C329" s="8" t="n"/>
-      <c r="J329" s="9" t="n"/>
+      <c r="D329" s="8" t="n"/>
+      <c r="K329" s="9" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="8" t="n"/>
       <c r="B330" s="8" t="n"/>
       <c r="C330" s="8" t="n"/>
-      <c r="J330" s="9" t="n"/>
+      <c r="D330" s="8" t="n"/>
+      <c r="K330" s="9" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="8" t="n"/>
       <c r="B331" s="8" t="n"/>
       <c r="C331" s="8" t="n"/>
-      <c r="J331" s="9" t="n"/>
+      <c r="D331" s="8" t="n"/>
+      <c r="K331" s="9" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="8" t="n"/>
       <c r="B332" s="8" t="n"/>
       <c r="C332" s="8" t="n"/>
-      <c r="J332" s="9" t="n"/>
+      <c r="D332" s="8" t="n"/>
+      <c r="K332" s="9" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="8" t="n"/>
       <c r="B333" s="8" t="n"/>
       <c r="C333" s="8" t="n"/>
-      <c r="J333" s="9" t="n"/>
+      <c r="D333" s="8" t="n"/>
+      <c r="K333" s="9" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="8" t="n"/>
       <c r="B334" s="8" t="n"/>
       <c r="C334" s="8" t="n"/>
-      <c r="J334" s="9" t="n"/>
+      <c r="D334" s="8" t="n"/>
+      <c r="K334" s="9" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="8" t="n"/>
       <c r="B335" s="8" t="n"/>
       <c r="C335" s="8" t="n"/>
-      <c r="J335" s="9" t="n"/>
+      <c r="D335" s="8" t="n"/>
+      <c r="K335" s="9" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="8" t="n"/>
       <c r="B336" s="8" t="n"/>
       <c r="C336" s="8" t="n"/>
-      <c r="J336" s="9" t="n"/>
+      <c r="D336" s="8" t="n"/>
+      <c r="K336" s="9" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="8" t="n"/>
       <c r="B337" s="8" t="n"/>
       <c r="C337" s="8" t="n"/>
-      <c r="J337" s="9" t="n"/>
+      <c r="D337" s="8" t="n"/>
+      <c r="K337" s="9" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="8" t="n"/>
       <c r="B338" s="8" t="n"/>
       <c r="C338" s="8" t="n"/>
-      <c r="J338" s="9" t="n"/>
+      <c r="D338" s="8" t="n"/>
+      <c r="K338" s="9" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="8" t="n"/>
       <c r="B339" s="8" t="n"/>
       <c r="C339" s="8" t="n"/>
-      <c r="J339" s="9" t="n"/>
+      <c r="D339" s="8" t="n"/>
+      <c r="K339" s="9" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="8" t="n"/>
       <c r="B340" s="8" t="n"/>
       <c r="C340" s="8" t="n"/>
-      <c r="J340" s="9" t="n"/>
+      <c r="D340" s="8" t="n"/>
+      <c r="K340" s="9" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="8" t="n"/>
       <c r="B341" s="8" t="n"/>
       <c r="C341" s="8" t="n"/>
-      <c r="J341" s="9" t="n"/>
+      <c r="D341" s="8" t="n"/>
+      <c r="K341" s="9" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="8" t="n"/>
       <c r="B342" s="8" t="n"/>
       <c r="C342" s="8" t="n"/>
-      <c r="J342" s="9" t="n"/>
+      <c r="D342" s="8" t="n"/>
+      <c r="K342" s="9" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="8" t="n"/>
       <c r="B343" s="8" t="n"/>
       <c r="C343" s="8" t="n"/>
-      <c r="J343" s="9" t="n"/>
+      <c r="D343" s="8" t="n"/>
+      <c r="K343" s="9" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="8" t="n"/>
       <c r="B344" s="8" t="n"/>
       <c r="C344" s="8" t="n"/>
-      <c r="J344" s="9" t="n"/>
+      <c r="D344" s="8" t="n"/>
+      <c r="K344" s="9" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="8" t="n"/>
       <c r="B345" s="8" t="n"/>
       <c r="C345" s="8" t="n"/>
-      <c r="J345" s="9" t="n"/>
+      <c r="D345" s="8" t="n"/>
+      <c r="K345" s="9" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="8" t="n"/>
       <c r="B346" s="8" t="n"/>
       <c r="C346" s="8" t="n"/>
-      <c r="J346" s="9" t="n"/>
+      <c r="D346" s="8" t="n"/>
+      <c r="K346" s="9" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="8" t="n"/>
       <c r="B347" s="8" t="n"/>
       <c r="C347" s="8" t="n"/>
-      <c r="J347" s="9" t="n"/>
+      <c r="D347" s="8" t="n"/>
+      <c r="K347" s="9" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="8" t="n"/>
       <c r="B348" s="8" t="n"/>
       <c r="C348" s="8" t="n"/>
-      <c r="J348" s="9" t="n"/>
+      <c r="D348" s="8" t="n"/>
+      <c r="K348" s="9" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="8" t="n"/>
       <c r="B349" s="8" t="n"/>
       <c r="C349" s="8" t="n"/>
-      <c r="J349" s="9" t="n"/>
+      <c r="D349" s="8" t="n"/>
+      <c r="K349" s="9" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="8" t="n"/>
       <c r="B350" s="8" t="n"/>
       <c r="C350" s="8" t="n"/>
-      <c r="J350" s="9" t="n"/>
+      <c r="D350" s="8" t="n"/>
+      <c r="K350" s="9" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="8" t="n"/>
       <c r="B351" s="8" t="n"/>
       <c r="C351" s="8" t="n"/>
-      <c r="J351" s="9" t="n"/>
+      <c r="D351" s="8" t="n"/>
+      <c r="K351" s="9" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="8" t="n"/>
       <c r="B352" s="8" t="n"/>
       <c r="C352" s="8" t="n"/>
-      <c r="J352" s="9" t="n"/>
+      <c r="D352" s="8" t="n"/>
+      <c r="K352" s="9" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="8" t="n"/>
       <c r="B353" s="8" t="n"/>
       <c r="C353" s="8" t="n"/>
-      <c r="J353" s="9" t="n"/>
+      <c r="D353" s="8" t="n"/>
+      <c r="K353" s="9" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="8" t="n"/>
       <c r="B354" s="8" t="n"/>
       <c r="C354" s="8" t="n"/>
-      <c r="J354" s="9" t="n"/>
+      <c r="D354" s="8" t="n"/>
+      <c r="K354" s="9" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="8" t="n"/>
       <c r="B355" s="8" t="n"/>
       <c r="C355" s="8" t="n"/>
-      <c r="J355" s="9" t="n"/>
+      <c r="D355" s="8" t="n"/>
+      <c r="K355" s="9" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="8" t="n"/>
       <c r="B356" s="8" t="n"/>
       <c r="C356" s="8" t="n"/>
-      <c r="J356" s="9" t="n"/>
+      <c r="D356" s="8" t="n"/>
+      <c r="K356" s="9" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="8" t="n"/>
       <c r="B357" s="8" t="n"/>
       <c r="C357" s="8" t="n"/>
-      <c r="J357" s="9" t="n"/>
+      <c r="D357" s="8" t="n"/>
+      <c r="K357" s="9" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="8" t="n"/>
       <c r="B358" s="8" t="n"/>
       <c r="C358" s="8" t="n"/>
-      <c r="J358" s="9" t="n"/>
+      <c r="D358" s="8" t="n"/>
+      <c r="K358" s="9" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="8" t="n"/>
       <c r="B359" s="8" t="n"/>
       <c r="C359" s="8" t="n"/>
-      <c r="J359" s="9" t="n"/>
+      <c r="D359" s="8" t="n"/>
+      <c r="K359" s="9" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="8" t="n"/>
       <c r="B360" s="8" t="n"/>
       <c r="C360" s="8" t="n"/>
-      <c r="J360" s="9" t="n"/>
+      <c r="D360" s="8" t="n"/>
+      <c r="K360" s="9" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="8" t="n"/>
       <c r="B361" s="8" t="n"/>
       <c r="C361" s="8" t="n"/>
-      <c r="J361" s="9" t="n"/>
+      <c r="D361" s="8" t="n"/>
+      <c r="K361" s="9" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="8" t="n"/>
       <c r="B362" s="8" t="n"/>
       <c r="C362" s="8" t="n"/>
-      <c r="J362" s="9" t="n"/>
+      <c r="D362" s="8" t="n"/>
+      <c r="K362" s="9" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="8" t="n"/>
       <c r="B363" s="8" t="n"/>
       <c r="C363" s="8" t="n"/>
-      <c r="J363" s="9" t="n"/>
+      <c r="D363" s="8" t="n"/>
+      <c r="K363" s="9" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="8" t="n"/>
       <c r="B364" s="8" t="n"/>
       <c r="C364" s="8" t="n"/>
-      <c r="J364" s="9" t="n"/>
+      <c r="D364" s="8" t="n"/>
+      <c r="K364" s="9" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="8" t="n"/>
       <c r="B365" s="8" t="n"/>
       <c r="C365" s="8" t="n"/>
-      <c r="J365" s="9" t="n"/>
+      <c r="D365" s="8" t="n"/>
+      <c r="K365" s="9" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="8" t="n"/>
       <c r="B366" s="8" t="n"/>
       <c r="C366" s="8" t="n"/>
-      <c r="J366" s="9" t="n"/>
+      <c r="D366" s="8" t="n"/>
+      <c r="K366" s="9" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="8" t="n"/>
       <c r="B367" s="8" t="n"/>
       <c r="C367" s="8" t="n"/>
-      <c r="J367" s="9" t="n"/>
+      <c r="D367" s="8" t="n"/>
+      <c r="K367" s="9" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="8" t="n"/>
       <c r="B368" s="8" t="n"/>
       <c r="C368" s="8" t="n"/>
-      <c r="J368" s="9" t="n"/>
+      <c r="D368" s="8" t="n"/>
+      <c r="K368" s="9" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="8" t="n"/>
       <c r="B369" s="8" t="n"/>
       <c r="C369" s="8" t="n"/>
-      <c r="J369" s="9" t="n"/>
+      <c r="D369" s="8" t="n"/>
+      <c r="K369" s="9" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="8" t="n"/>
       <c r="B370" s="8" t="n"/>
       <c r="C370" s="8" t="n"/>
-      <c r="J370" s="9" t="n"/>
+      <c r="D370" s="8" t="n"/>
+      <c r="K370" s="9" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="8" t="n"/>
       <c r="B371" s="8" t="n"/>
       <c r="C371" s="8" t="n"/>
-      <c r="J371" s="9" t="n"/>
+      <c r="D371" s="8" t="n"/>
+      <c r="K371" s="9" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="8" t="n"/>
       <c r="B372" s="8" t="n"/>
       <c r="C372" s="8" t="n"/>
-      <c r="J372" s="9" t="n"/>
+      <c r="D372" s="8" t="n"/>
+      <c r="K372" s="9" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="8" t="n"/>
       <c r="B373" s="8" t="n"/>
       <c r="C373" s="8" t="n"/>
-      <c r="J373" s="9" t="n"/>
+      <c r="D373" s="8" t="n"/>
+      <c r="K373" s="9" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="8" t="n"/>
       <c r="B374" s="8" t="n"/>
       <c r="C374" s="8" t="n"/>
-      <c r="J374" s="9" t="n"/>
+      <c r="D374" s="8" t="n"/>
+      <c r="K374" s="9" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="8" t="n"/>
       <c r="B375" s="8" t="n"/>
       <c r="C375" s="8" t="n"/>
-      <c r="J375" s="9" t="n"/>
+      <c r="D375" s="8" t="n"/>
+      <c r="K375" s="9" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="8" t="n"/>
       <c r="B376" s="8" t="n"/>
       <c r="C376" s="8" t="n"/>
-      <c r="J376" s="9" t="n"/>
+      <c r="D376" s="8" t="n"/>
+      <c r="K376" s="9" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="8" t="n"/>
       <c r="B377" s="8" t="n"/>
       <c r="C377" s="8" t="n"/>
-      <c r="J377" s="9" t="n"/>
+      <c r="D377" s="8" t="n"/>
+      <c r="K377" s="9" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="8" t="n"/>
       <c r="B378" s="8" t="n"/>
       <c r="C378" s="8" t="n"/>
-      <c r="J378" s="9" t="n"/>
+      <c r="D378" s="8" t="n"/>
+      <c r="K378" s="9" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="8" t="n"/>
       <c r="B379" s="8" t="n"/>
       <c r="C379" s="8" t="n"/>
-      <c r="J379" s="9" t="n"/>
+      <c r="D379" s="8" t="n"/>
+      <c r="K379" s="9" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="8" t="n"/>
       <c r="B380" s="8" t="n"/>
       <c r="C380" s="8" t="n"/>
-      <c r="J380" s="9" t="n"/>
+      <c r="D380" s="8" t="n"/>
+      <c r="K380" s="9" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="8" t="n"/>
       <c r="B381" s="8" t="n"/>
       <c r="C381" s="8" t="n"/>
-      <c r="J381" s="9" t="n"/>
+      <c r="D381" s="8" t="n"/>
+      <c r="K381" s="9" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="8" t="n"/>
       <c r="B382" s="8" t="n"/>
       <c r="C382" s="8" t="n"/>
-      <c r="J382" s="9" t="n"/>
+      <c r="D382" s="8" t="n"/>
+      <c r="K382" s="9" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="8" t="n"/>
       <c r="B383" s="8" t="n"/>
       <c r="C383" s="8" t="n"/>
-      <c r="J383" s="9" t="n"/>
+      <c r="D383" s="8" t="n"/>
+      <c r="K383" s="9" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="8" t="n"/>
       <c r="B384" s="8" t="n"/>
       <c r="C384" s="8" t="n"/>
-      <c r="J384" s="9" t="n"/>
+      <c r="D384" s="8" t="n"/>
+      <c r="K384" s="9" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="8" t="n"/>
       <c r="B385" s="8" t="n"/>
       <c r="C385" s="8" t="n"/>
-      <c r="J385" s="9" t="n"/>
+      <c r="D385" s="8" t="n"/>
+      <c r="K385" s="9" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="8" t="n"/>
       <c r="B386" s="8" t="n"/>
       <c r="C386" s="8" t="n"/>
-      <c r="J386" s="9" t="n"/>
+      <c r="D386" s="8" t="n"/>
+      <c r="K386" s="9" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="8" t="n"/>
       <c r="B387" s="8" t="n"/>
       <c r="C387" s="8" t="n"/>
-      <c r="J387" s="9" t="n"/>
+      <c r="D387" s="8" t="n"/>
+      <c r="K387" s="9" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="8" t="n"/>
       <c r="B388" s="8" t="n"/>
       <c r="C388" s="8" t="n"/>
-      <c r="J388" s="9" t="n"/>
+      <c r="D388" s="8" t="n"/>
+      <c r="K388" s="9" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="8" t="n"/>
       <c r="B389" s="8" t="n"/>
       <c r="C389" s="8" t="n"/>
-      <c r="J389" s="9" t="n"/>
+      <c r="D389" s="8" t="n"/>
+      <c r="K389" s="9" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="8" t="n"/>
       <c r="B390" s="8" t="n"/>
       <c r="C390" s="8" t="n"/>
-      <c r="J390" s="9" t="n"/>
+      <c r="D390" s="8" t="n"/>
+      <c r="K390" s="9" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="8" t="n"/>
       <c r="B391" s="8" t="n"/>
       <c r="C391" s="8" t="n"/>
-      <c r="J391" s="9" t="n"/>
+      <c r="D391" s="8" t="n"/>
+      <c r="K391" s="9" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="8" t="n"/>
       <c r="B392" s="8" t="n"/>
       <c r="C392" s="8" t="n"/>
-      <c r="J392" s="9" t="n"/>
+      <c r="D392" s="8" t="n"/>
+      <c r="K392" s="9" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="8" t="n"/>
       <c r="B393" s="8" t="n"/>
       <c r="C393" s="8" t="n"/>
-      <c r="J393" s="9" t="n"/>
+      <c r="D393" s="8" t="n"/>
+      <c r="K393" s="9" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="8" t="n"/>
       <c r="B394" s="8" t="n"/>
       <c r="C394" s="8" t="n"/>
-      <c r="J394" s="9" t="n"/>
+      <c r="D394" s="8" t="n"/>
+      <c r="K394" s="9" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="8" t="n"/>
       <c r="B395" s="8" t="n"/>
       <c r="C395" s="8" t="n"/>
-      <c r="J395" s="9" t="n"/>
+      <c r="D395" s="8" t="n"/>
+      <c r="K395" s="9" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="8" t="n"/>
       <c r="B396" s="8" t="n"/>
       <c r="C396" s="8" t="n"/>
-      <c r="J396" s="9" t="n"/>
+      <c r="D396" s="8" t="n"/>
+      <c r="K396" s="9" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="8" t="n"/>
       <c r="B397" s="8" t="n"/>
       <c r="C397" s="8" t="n"/>
-      <c r="J397" s="9" t="n"/>
+      <c r="D397" s="8" t="n"/>
+      <c r="K397" s="9" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="8" t="n"/>
       <c r="B398" s="8" t="n"/>
       <c r="C398" s="8" t="n"/>
-      <c r="J398" s="9" t="n"/>
+      <c r="D398" s="8" t="n"/>
+      <c r="K398" s="9" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="8" t="n"/>
       <c r="B399" s="8" t="n"/>
       <c r="C399" s="8" t="n"/>
-      <c r="J399" s="9" t="n"/>
+      <c r="D399" s="8" t="n"/>
+      <c r="K399" s="9" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="8" t="n"/>
       <c r="B400" s="8" t="n"/>
       <c r="C400" s="8" t="n"/>
-      <c r="J400" s="9" t="n"/>
+      <c r="D400" s="8" t="n"/>
+      <c r="K400" s="9" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="8" t="n"/>
       <c r="B401" s="8" t="n"/>
       <c r="C401" s="8" t="n"/>
-      <c r="J401" s="9" t="n"/>
+      <c r="D401" s="8" t="n"/>
+      <c r="K401" s="9" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="8" t="n"/>
       <c r="B402" s="8" t="n"/>
       <c r="C402" s="8" t="n"/>
-      <c r="J402" s="9" t="n"/>
+      <c r="D402" s="8" t="n"/>
+      <c r="K402" s="9" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="8" t="n"/>
       <c r="B403" s="8" t="n"/>
       <c r="C403" s="8" t="n"/>
-      <c r="J403" s="9" t="n"/>
+      <c r="D403" s="8" t="n"/>
+      <c r="K403" s="9" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="8" t="n"/>
       <c r="B404" s="8" t="n"/>
       <c r="C404" s="8" t="n"/>
-      <c r="J404" s="9" t="n"/>
+      <c r="D404" s="8" t="n"/>
+      <c r="K404" s="9" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="8" t="n"/>
       <c r="B405" s="8" t="n"/>
       <c r="C405" s="8" t="n"/>
-      <c r="J405" s="9" t="n"/>
+      <c r="D405" s="8" t="n"/>
+      <c r="K405" s="9" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="8" t="n"/>
       <c r="B406" s="8" t="n"/>
       <c r="C406" s="8" t="n"/>
-      <c r="J406" s="9" t="n"/>
+      <c r="D406" s="8" t="n"/>
+      <c r="K406" s="9" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="8" t="n"/>
       <c r="B407" s="8" t="n"/>
       <c r="C407" s="8" t="n"/>
-      <c r="J407" s="9" t="n"/>
+      <c r="D407" s="8" t="n"/>
+      <c r="K407" s="9" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="8" t="n"/>
       <c r="B408" s="8" t="n"/>
       <c r="C408" s="8" t="n"/>
-      <c r="J408" s="9" t="n"/>
+      <c r="D408" s="8" t="n"/>
+      <c r="K408" s="9" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="8" t="n"/>
       <c r="B409" s="8" t="n"/>
       <c r="C409" s="8" t="n"/>
-      <c r="J409" s="9" t="n"/>
+      <c r="D409" s="8" t="n"/>
+      <c r="K409" s="9" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="8" t="n"/>
       <c r="B410" s="8" t="n"/>
       <c r="C410" s="8" t="n"/>
-      <c r="J410" s="9" t="n"/>
+      <c r="D410" s="8" t="n"/>
+      <c r="K410" s="9" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="8" t="n"/>
       <c r="B411" s="8" t="n"/>
       <c r="C411" s="8" t="n"/>
-      <c r="J411" s="9" t="n"/>
+      <c r="D411" s="8" t="n"/>
+      <c r="K411" s="9" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="8" t="n"/>
       <c r="B412" s="8" t="n"/>
       <c r="C412" s="8" t="n"/>
-      <c r="J412" s="9" t="n"/>
+      <c r="D412" s="8" t="n"/>
+      <c r="K412" s="9" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="8" t="n"/>
       <c r="B413" s="8" t="n"/>
       <c r="C413" s="8" t="n"/>
-      <c r="J413" s="9" t="n"/>
+      <c r="D413" s="8" t="n"/>
+      <c r="K413" s="9" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="8" t="n"/>
       <c r="B414" s="8" t="n"/>
       <c r="C414" s="8" t="n"/>
-      <c r="J414" s="9" t="n"/>
+      <c r="D414" s="8" t="n"/>
+      <c r="K414" s="9" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="8" t="n"/>
       <c r="B415" s="8" t="n"/>
       <c r="C415" s="8" t="n"/>
-      <c r="J415" s="9" t="n"/>
+      <c r="D415" s="8" t="n"/>
+      <c r="K415" s="9" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="8" t="n"/>
       <c r="B416" s="8" t="n"/>
       <c r="C416" s="8" t="n"/>
-      <c r="J416" s="9" t="n"/>
+      <c r="D416" s="8" t="n"/>
+      <c r="K416" s="9" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="8" t="n"/>
       <c r="B417" s="8" t="n"/>
       <c r="C417" s="8" t="n"/>
-      <c r="J417" s="9" t="n"/>
+      <c r="D417" s="8" t="n"/>
+      <c r="K417" s="9" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="8" t="n"/>
       <c r="B418" s="8" t="n"/>
       <c r="C418" s="8" t="n"/>
-      <c r="J418" s="9" t="n"/>
+      <c r="D418" s="8" t="n"/>
+      <c r="K418" s="9" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="8" t="n"/>
       <c r="B419" s="8" t="n"/>
       <c r="C419" s="8" t="n"/>
-      <c r="J419" s="9" t="n"/>
+      <c r="D419" s="8" t="n"/>
+      <c r="K419" s="9" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="8" t="n"/>
       <c r="B420" s="8" t="n"/>
       <c r="C420" s="8" t="n"/>
-      <c r="J420" s="9" t="n"/>
+      <c r="D420" s="8" t="n"/>
+      <c r="K420" s="9" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="8" t="n"/>
       <c r="B421" s="8" t="n"/>
       <c r="C421" s="8" t="n"/>
-      <c r="J421" s="9" t="n"/>
+      <c r="D421" s="8" t="n"/>
+      <c r="K421" s="9" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="8" t="n"/>
       <c r="B422" s="8" t="n"/>
       <c r="C422" s="8" t="n"/>
-      <c r="J422" s="9" t="n"/>
+      <c r="D422" s="8" t="n"/>
+      <c r="K422" s="9" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="8" t="n"/>
       <c r="B423" s="8" t="n"/>
       <c r="C423" s="8" t="n"/>
-      <c r="J423" s="9" t="n"/>
+      <c r="D423" s="8" t="n"/>
+      <c r="K423" s="9" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="8" t="n"/>
       <c r="B424" s="8" t="n"/>
       <c r="C424" s="8" t="n"/>
-      <c r="J424" s="9" t="n"/>
+      <c r="D424" s="8" t="n"/>
+      <c r="K424" s="9" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="8" t="n"/>
       <c r="B425" s="8" t="n"/>
       <c r="C425" s="8" t="n"/>
-      <c r="J425" s="9" t="n"/>
+      <c r="D425" s="8" t="n"/>
+      <c r="K425" s="9" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="8" t="n"/>
       <c r="B426" s="8" t="n"/>
       <c r="C426" s="8" t="n"/>
-      <c r="J426" s="9" t="n"/>
+      <c r="D426" s="8" t="n"/>
+      <c r="K426" s="9" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="8" t="n"/>
       <c r="B427" s="8" t="n"/>
       <c r="C427" s="8" t="n"/>
-      <c r="J427" s="9" t="n"/>
+      <c r="D427" s="8" t="n"/>
+      <c r="K427" s="9" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="8" t="n"/>
       <c r="B428" s="8" t="n"/>
       <c r="C428" s="8" t="n"/>
-      <c r="J428" s="9" t="n"/>
+      <c r="D428" s="8" t="n"/>
+      <c r="K428" s="9" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="8" t="n"/>
       <c r="B429" s="8" t="n"/>
       <c r="C429" s="8" t="n"/>
-      <c r="J429" s="9" t="n"/>
+      <c r="D429" s="8" t="n"/>
+      <c r="K429" s="9" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="8" t="n"/>
       <c r="B430" s="8" t="n"/>
       <c r="C430" s="8" t="n"/>
-      <c r="J430" s="9" t="n"/>
+      <c r="D430" s="8" t="n"/>
+      <c r="K430" s="9" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="8" t="n"/>
       <c r="B431" s="8" t="n"/>
       <c r="C431" s="8" t="n"/>
-      <c r="J431" s="9" t="n"/>
+      <c r="D431" s="8" t="n"/>
+      <c r="K431" s="9" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="8" t="n"/>
       <c r="B432" s="8" t="n"/>
       <c r="C432" s="8" t="n"/>
-      <c r="J432" s="9" t="n"/>
+      <c r="D432" s="8" t="n"/>
+      <c r="K432" s="9" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="8" t="n"/>
       <c r="B433" s="8" t="n"/>
       <c r="C433" s="8" t="n"/>
-      <c r="J433" s="9" t="n"/>
+      <c r="D433" s="8" t="n"/>
+      <c r="K433" s="9" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="8" t="n"/>
       <c r="B434" s="8" t="n"/>
       <c r="C434" s="8" t="n"/>
-      <c r="J434" s="9" t="n"/>
+      <c r="D434" s="8" t="n"/>
+      <c r="K434" s="9" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="8" t="n"/>
       <c r="B435" s="8" t="n"/>
       <c r="C435" s="8" t="n"/>
-      <c r="J435" s="9" t="n"/>
+      <c r="D435" s="8" t="n"/>
+      <c r="K435" s="9" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="8" t="n"/>
       <c r="B436" s="8" t="n"/>
       <c r="C436" s="8" t="n"/>
-      <c r="J436" s="9" t="n"/>
+      <c r="D436" s="8" t="n"/>
+      <c r="K436" s="9" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="8" t="n"/>
       <c r="B437" s="8" t="n"/>
       <c r="C437" s="8" t="n"/>
-      <c r="J437" s="9" t="n"/>
+      <c r="D437" s="8" t="n"/>
+      <c r="K437" s="9" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="8" t="n"/>
       <c r="B438" s="8" t="n"/>
       <c r="C438" s="8" t="n"/>
-      <c r="J438" s="9" t="n"/>
+      <c r="D438" s="8" t="n"/>
+      <c r="K438" s="9" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="8" t="n"/>
       <c r="B439" s="8" t="n"/>
       <c r="C439" s="8" t="n"/>
-      <c r="J439" s="9" t="n"/>
+      <c r="D439" s="8" t="n"/>
+      <c r="K439" s="9" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="8" t="n"/>
       <c r="B440" s="8" t="n"/>
       <c r="C440" s="8" t="n"/>
-      <c r="J440" s="9" t="n"/>
+      <c r="D440" s="8" t="n"/>
+      <c r="K440" s="9" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="8" t="n"/>
       <c r="B441" s="8" t="n"/>
       <c r="C441" s="8" t="n"/>
-      <c r="J441" s="9" t="n"/>
+      <c r="D441" s="8" t="n"/>
+      <c r="K441" s="9" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="8" t="n"/>
       <c r="B442" s="8" t="n"/>
       <c r="C442" s="8" t="n"/>
-      <c r="J442" s="9" t="n"/>
+      <c r="D442" s="8" t="n"/>
+      <c r="K442" s="9" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="8" t="n"/>
       <c r="B443" s="8" t="n"/>
       <c r="C443" s="8" t="n"/>
-      <c r="J443" s="9" t="n"/>
+      <c r="D443" s="8" t="n"/>
+      <c r="K443" s="9" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="8" t="n"/>
       <c r="B444" s="8" t="n"/>
       <c r="C444" s="8" t="n"/>
-      <c r="J444" s="9" t="n"/>
+      <c r="D444" s="8" t="n"/>
+      <c r="K444" s="9" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="8" t="n"/>
       <c r="B445" s="8" t="n"/>
       <c r="C445" s="8" t="n"/>
-      <c r="J445" s="9" t="n"/>
+      <c r="D445" s="8" t="n"/>
+      <c r="K445" s="9" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="8" t="n"/>
       <c r="B446" s="8" t="n"/>
       <c r="C446" s="8" t="n"/>
-      <c r="J446" s="9" t="n"/>
+      <c r="D446" s="8" t="n"/>
+      <c r="K446" s="9" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="8" t="n"/>
       <c r="B447" s="8" t="n"/>
       <c r="C447" s="8" t="n"/>
-      <c r="J447" s="9" t="n"/>
+      <c r="D447" s="8" t="n"/>
+      <c r="K447" s="9" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="8" t="n"/>
       <c r="B448" s="8" t="n"/>
       <c r="C448" s="8" t="n"/>
-      <c r="J448" s="9" t="n"/>
+      <c r="D448" s="8" t="n"/>
+      <c r="K448" s="9" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="8" t="n"/>
       <c r="B449" s="8" t="n"/>
       <c r="C449" s="8" t="n"/>
-      <c r="J449" s="9" t="n"/>
+      <c r="D449" s="8" t="n"/>
+      <c r="K449" s="9" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="8" t="n"/>
       <c r="B450" s="8" t="n"/>
       <c r="C450" s="8" t="n"/>
-      <c r="J450" s="9" t="n"/>
+      <c r="D450" s="8" t="n"/>
+      <c r="K450" s="9" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="8" t="n"/>
       <c r="B451" s="8" t="n"/>
       <c r="C451" s="8" t="n"/>
-      <c r="J451" s="9" t="n"/>
+      <c r="D451" s="8" t="n"/>
+      <c r="K451" s="9" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="8" t="n"/>
       <c r="B452" s="8" t="n"/>
       <c r="C452" s="8" t="n"/>
-      <c r="J452" s="9" t="n"/>
+      <c r="D452" s="8" t="n"/>
+      <c r="K452" s="9" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="8" t="n"/>
       <c r="B453" s="8" t="n"/>
       <c r="C453" s="8" t="n"/>
-      <c r="J453" s="9" t="n"/>
+      <c r="D453" s="8" t="n"/>
+      <c r="K453" s="9" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="8" t="n"/>
       <c r="B454" s="8" t="n"/>
       <c r="C454" s="8" t="n"/>
-      <c r="J454" s="9" t="n"/>
+      <c r="D454" s="8" t="n"/>
+      <c r="K454" s="9" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="8" t="n"/>
       <c r="B455" s="8" t="n"/>
       <c r="C455" s="8" t="n"/>
-      <c r="J455" s="9" t="n"/>
+      <c r="D455" s="8" t="n"/>
+      <c r="K455" s="9" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="8" t="n"/>
       <c r="B456" s="8" t="n"/>
       <c r="C456" s="8" t="n"/>
-      <c r="J456" s="9" t="n"/>
+      <c r="D456" s="8" t="n"/>
+      <c r="K456" s="9" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="8" t="n"/>
       <c r="B457" s="8" t="n"/>
       <c r="C457" s="8" t="n"/>
-      <c r="J457" s="9" t="n"/>
+      <c r="D457" s="8" t="n"/>
+      <c r="K457" s="9" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="8" t="n"/>
       <c r="B458" s="8" t="n"/>
       <c r="C458" s="8" t="n"/>
-      <c r="J458" s="9" t="n"/>
+      <c r="D458" s="8" t="n"/>
+      <c r="K458" s="9" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="8" t="n"/>
       <c r="B459" s="8" t="n"/>
       <c r="C459" s="8" t="n"/>
-      <c r="J459" s="9" t="n"/>
+      <c r="D459" s="8" t="n"/>
+      <c r="K459" s="9" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="8" t="n"/>
       <c r="B460" s="8" t="n"/>
       <c r="C460" s="8" t="n"/>
-      <c r="J460" s="9" t="n"/>
+      <c r="D460" s="8" t="n"/>
+      <c r="K460" s="9" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="8" t="n"/>
       <c r="B461" s="8" t="n"/>
       <c r="C461" s="8" t="n"/>
-      <c r="J461" s="9" t="n"/>
+      <c r="D461" s="8" t="n"/>
+      <c r="K461" s="9" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="8" t="n"/>
       <c r="B462" s="8" t="n"/>
       <c r="C462" s="8" t="n"/>
-      <c r="J462" s="9" t="n"/>
+      <c r="D462" s="8" t="n"/>
+      <c r="K462" s="9" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="8" t="n"/>
       <c r="B463" s="8" t="n"/>
       <c r="C463" s="8" t="n"/>
-      <c r="J463" s="9" t="n"/>
+      <c r="D463" s="8" t="n"/>
+      <c r="K463" s="9" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="8" t="n"/>
       <c r="B464" s="8" t="n"/>
       <c r="C464" s="8" t="n"/>
-      <c r="J464" s="9" t="n"/>
+      <c r="D464" s="8" t="n"/>
+      <c r="K464" s="9" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="8" t="n"/>
       <c r="B465" s="8" t="n"/>
       <c r="C465" s="8" t="n"/>
-      <c r="J465" s="9" t="n"/>
+      <c r="D465" s="8" t="n"/>
+      <c r="K465" s="9" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="8" t="n"/>
       <c r="B466" s="8" t="n"/>
       <c r="C466" s="8" t="n"/>
-      <c r="J466" s="9" t="n"/>
+      <c r="D466" s="8" t="n"/>
+      <c r="K466" s="9" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="8" t="n"/>
       <c r="B467" s="8" t="n"/>
       <c r="C467" s="8" t="n"/>
-      <c r="J467" s="9" t="n"/>
+      <c r="D467" s="8" t="n"/>
+      <c r="K467" s="9" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="8" t="n"/>
       <c r="B468" s="8" t="n"/>
       <c r="C468" s="8" t="n"/>
-      <c r="J468" s="9" t="n"/>
+      <c r="D468" s="8" t="n"/>
+      <c r="K468" s="9" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="8" t="n"/>
       <c r="B469" s="8" t="n"/>
       <c r="C469" s="8" t="n"/>
-      <c r="J469" s="9" t="n"/>
+      <c r="D469" s="8" t="n"/>
+      <c r="K469" s="9" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="8" t="n"/>
       <c r="B470" s="8" t="n"/>
       <c r="C470" s="8" t="n"/>
-      <c r="J470" s="9" t="n"/>
+      <c r="D470" s="8" t="n"/>
+      <c r="K470" s="9" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="8" t="n"/>
       <c r="B471" s="8" t="n"/>
       <c r="C471" s="8" t="n"/>
-      <c r="J471" s="9" t="n"/>
+      <c r="D471" s="8" t="n"/>
+      <c r="K471" s="9" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="8" t="n"/>
       <c r="B472" s="8" t="n"/>
       <c r="C472" s="8" t="n"/>
-      <c r="J472" s="9" t="n"/>
+      <c r="D472" s="8" t="n"/>
+      <c r="K472" s="9" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="8" t="n"/>
       <c r="B473" s="8" t="n"/>
       <c r="C473" s="8" t="n"/>
-      <c r="J473" s="9" t="n"/>
+      <c r="D473" s="8" t="n"/>
+      <c r="K473" s="9" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="8" t="n"/>
       <c r="B474" s="8" t="n"/>
       <c r="C474" s="8" t="n"/>
-      <c r="J474" s="9" t="n"/>
+      <c r="D474" s="8" t="n"/>
+      <c r="K474" s="9" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="8" t="n"/>
       <c r="B475" s="8" t="n"/>
       <c r="C475" s="8" t="n"/>
-      <c r="J475" s="9" t="n"/>
+      <c r="D475" s="8" t="n"/>
+      <c r="K475" s="9" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="8" t="n"/>
       <c r="B476" s="8" t="n"/>
       <c r="C476" s="8" t="n"/>
-      <c r="J476" s="9" t="n"/>
+      <c r="D476" s="8" t="n"/>
+      <c r="K476" s="9" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="8" t="n"/>
       <c r="B477" s="8" t="n"/>
       <c r="C477" s="8" t="n"/>
-      <c r="J477" s="9" t="n"/>
+      <c r="D477" s="8" t="n"/>
+      <c r="K477" s="9" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="8" t="n"/>
       <c r="B478" s="8" t="n"/>
       <c r="C478" s="8" t="n"/>
-      <c r="J478" s="9" t="n"/>
+      <c r="D478" s="8" t="n"/>
+      <c r="K478" s="9" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="8" t="n"/>
       <c r="B479" s="8" t="n"/>
       <c r="C479" s="8" t="n"/>
-      <c r="J479" s="9" t="n"/>
+      <c r="D479" s="8" t="n"/>
+      <c r="K479" s="9" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="8" t="n"/>
       <c r="B480" s="8" t="n"/>
       <c r="C480" s="8" t="n"/>
-      <c r="J480" s="9" t="n"/>
+      <c r="D480" s="8" t="n"/>
+      <c r="K480" s="9" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="8" t="n"/>
       <c r="B481" s="8" t="n"/>
       <c r="C481" s="8" t="n"/>
-      <c r="J481" s="9" t="n"/>
+      <c r="D481" s="8" t="n"/>
+      <c r="K481" s="9" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="8" t="n"/>
       <c r="B482" s="8" t="n"/>
       <c r="C482" s="8" t="n"/>
-      <c r="J482" s="9" t="n"/>
+      <c r="D482" s="8" t="n"/>
+      <c r="K482" s="9" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="8" t="n"/>
       <c r="B483" s="8" t="n"/>
       <c r="C483" s="8" t="n"/>
-      <c r="J483" s="9" t="n"/>
+      <c r="D483" s="8" t="n"/>
+      <c r="K483" s="9" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="8" t="n"/>
       <c r="B484" s="8" t="n"/>
       <c r="C484" s="8" t="n"/>
-      <c r="J484" s="9" t="n"/>
+      <c r="D484" s="8" t="n"/>
+      <c r="K484" s="9" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="8" t="n"/>
       <c r="B485" s="8" t="n"/>
       <c r="C485" s="8" t="n"/>
-      <c r="J485" s="9" t="n"/>
+      <c r="D485" s="8" t="n"/>
+      <c r="K485" s="9" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="8" t="n"/>
       <c r="B486" s="8" t="n"/>
       <c r="C486" s="8" t="n"/>
-      <c r="J486" s="9" t="n"/>
+      <c r="D486" s="8" t="n"/>
+      <c r="K486" s="9" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="8" t="n"/>
       <c r="B487" s="8" t="n"/>
       <c r="C487" s="8" t="n"/>
-      <c r="J487" s="9" t="n"/>
+      <c r="D487" s="8" t="n"/>
+      <c r="K487" s="9" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="8" t="n"/>
       <c r="B488" s="8" t="n"/>
       <c r="C488" s="8" t="n"/>
-      <c r="J488" s="9" t="n"/>
+      <c r="D488" s="8" t="n"/>
+      <c r="K488" s="9" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="8" t="n"/>
       <c r="B489" s="8" t="n"/>
       <c r="C489" s="8" t="n"/>
-      <c r="J489" s="9" t="n"/>
+      <c r="D489" s="8" t="n"/>
+      <c r="K489" s="9" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="8" t="n"/>
       <c r="B490" s="8" t="n"/>
       <c r="C490" s="8" t="n"/>
-      <c r="J490" s="9" t="n"/>
+      <c r="D490" s="8" t="n"/>
+      <c r="K490" s="9" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="8" t="n"/>
       <c r="B491" s="8" t="n"/>
       <c r="C491" s="8" t="n"/>
-      <c r="J491" s="9" t="n"/>
+      <c r="D491" s="8" t="n"/>
+      <c r="K491" s="9" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="8" t="n"/>
       <c r="B492" s="8" t="n"/>
       <c r="C492" s="8" t="n"/>
-      <c r="J492" s="9" t="n"/>
+      <c r="D492" s="8" t="n"/>
+      <c r="K492" s="9" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="8" t="n"/>
       <c r="B493" s="8" t="n"/>
       <c r="C493" s="8" t="n"/>
-      <c r="J493" s="9" t="n"/>
+      <c r="D493" s="8" t="n"/>
+      <c r="K493" s="9" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="8" t="n"/>
       <c r="B494" s="8" t="n"/>
       <c r="C494" s="8" t="n"/>
-      <c r="J494" s="9" t="n"/>
+      <c r="D494" s="8" t="n"/>
+      <c r="K494" s="9" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="8" t="n"/>
       <c r="B495" s="8" t="n"/>
       <c r="C495" s="8" t="n"/>
-      <c r="J495" s="9" t="n"/>
+      <c r="D495" s="8" t="n"/>
+      <c r="K495" s="9" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="8" t="n"/>
       <c r="B496" s="8" t="n"/>
       <c r="C496" s="8" t="n"/>
-      <c r="J496" s="9" t="n"/>
+      <c r="D496" s="8" t="n"/>
+      <c r="K496" s="9" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="8" t="n"/>
       <c r="B497" s="8" t="n"/>
       <c r="C497" s="8" t="n"/>
-      <c r="J497" s="9" t="n"/>
+      <c r="D497" s="8" t="n"/>
+      <c r="K497" s="9" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="8" t="n"/>
       <c r="B498" s="8" t="n"/>
       <c r="C498" s="8" t="n"/>
-      <c r="J498" s="9" t="n"/>
+      <c r="D498" s="8" t="n"/>
+      <c r="K498" s="9" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="8" t="n"/>
       <c r="B499" s="8" t="n"/>
       <c r="C499" s="8" t="n"/>
-      <c r="J499" s="9" t="n"/>
+      <c r="D499" s="8" t="n"/>
+      <c r="K499" s="9" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="8" t="n"/>
       <c r="B500" s="8" t="n"/>
       <c r="C500" s="8" t="n"/>
-      <c r="J500" s="9" t="n"/>
+      <c r="D500" s="8" t="n"/>
+      <c r="K500" s="9" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="8" t="n"/>
       <c r="B501" s="8" t="n"/>
       <c r="C501" s="8" t="n"/>
-      <c r="J501" s="9" t="n"/>
+      <c r="D501" s="8" t="n"/>
+      <c r="K501" s="9" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Datums" error="Ievadiet datumu (GGGG-MM-DD)." type="date" operator="greaterThan">
+  <dataValidations count="2">
+    <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Datums" error="Ievadiet datumu (GGGG-MM-DD)." type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Veids" error="Izvēlieties: īpašums, zemes vienība vai būve." type="list">
+      <formula1>"īpašums,zemes vienība,būve"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Test set: "Adrese pieteikumā" column, given address for M2 in check compare
- test_set_template.xlsx: new column "Adrese pieteikumā (atbilstības
  pārbaudei)" after the value (text format; instructions and M2 note updated).
- check compare reads it and resolves it like the batch adrese column (shared
  engine/batch/plan.py given_address): it is module 2's given address, so the
  M2 answer is compared; it wins over an address typed as the value; an
  address that is not found leaves the object checked, M2 not compared, with
  a note.
- Tests: a mismatching address agrees with "Ir: neatbilst", the object's own
  address with "Nav", an unknown address gives the note.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data/test_set_template.xlsx
+++ b/tests/data/test_set_template.xlsx
@@ -202,17 +202,17 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Neobligāta. Izvēlieties, ja 11 ciparu numurs var būt gan īpašums, gan citam īpašumam piederoša zemes vienība; bez tā rīks pārbauda abus.</t>
+        <t>Neobligāta. Adrese, kā norādīta pieteikumā: rīks pārbauda, vai tā atbilst objektam.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Neobligāta. Tikai juridiskas personas reģistrācijas numurs (11 cipari, sākas ar 4, 5 vai 9). Personas kodus neievadiet: tie netiek saglabāti.</t>
+        <t>Neobligāta. Izvēlieties, ja 11 ciparu numurs var būt gan īpašums, gan citam īpašumam piederoša zemes vienība; bez tā rīks pārbauda abus.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Neobligāta.</t>
+        <t>Neobligāta. Tikai juridiskas personas reģistrācijas numurs (11 cipari, sākas ar 4, 5 vai 9). Personas kodus neievadiet: tie netiek saglabāti.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -246,6 +246,11 @@
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Neobligāta.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Neobligāta.</t>
       </text>
@@ -543,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -590,150 +595,157 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>• Kadastra Nr., apzīmējums vai adrese (obligāta): kadastra numurs (11 cipari), kadastra apzīmējums (11, 14 vai 17 cipari) vai adrese. Kolonnas A–D ir teksta formātā: ievadiet ciparus ar sākuma nullēm (piem., 05000041006).</t>
+          <t>• Kadastra Nr., apzīmējums vai adrese (obligāta): kadastra numurs (11 cipari), kadastra apzīmējums (11, 14 vai 17 cipari) vai adrese. Kolonnas A–E ir teksta formātā: ievadiet ciparus ar sākuma nullēm (piem., 05000041006).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• Objekta veids: īpašums / zemes vienība / būve (ja numurs divdomīgs): izvēlieties no saraksta, ja 11 ciparu numurs var būt gan īpašuma numurs, gan citam īpašumam piederošas zemes vienības apzīmējums; bez tā rīks pārbauda abus.</t>
+          <t>• Adrese pieteikumā (atbilstības pārbaudei): adrese, kā tā norādīta pieteikumā. Rīks pārbauda, vai tā atbilst objektam (M2); bez tās M2 netiek salīdzināts.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>• Pieteicēja reģ. Nr. (tikai juridiskām personām): pieteicēja juridiskās personas reģistrācijas numurs (ja ir). Fizisko personu vārdus un personas kodus neievadiet.</t>
+          <t>• Objekta veids: īpašums / zemes vienība / būve (ja numurs divdomīgs): izvēlieties no saraksta, ja 11 ciparu numurs var būt gan īpašuma numurs, gan citam īpašumam piederošas zemes vienības apzīmējums; bez tā rīks pārbauda abus.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>• M1–M6: jūsu manuālās pārbaudes atbilde katram modulim. Sāciet ar vienu no: «Ir: …» (atrasts, īsi ko), «Nav», «Nav datu» (objekts nav atrasts / nav ģeometrijas), «Nav pārklājuma» (avotā šai teritorijai nav datu, piem., nav plūdu kartes). Pēc tam īss paskaidrojums.</t>
+          <t>• Pieteicēja reģ. Nr. (tikai juridiskām personām): pieteicēja juridiskās personas reģistrācijas numurs (ja ir). Fizisko personu vārdus un personas kodus neievadiet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Pārbaudes datums: datums, kad veicāt pārbaudi (GGGG-MM-DD). Svarīgi, jo dati laika gaitā mainās.</t>
+          <t>• M1–M6: jūsu manuālās pārbaudes atbilde katram modulim. Sāciet ar vienu no: «Ir: …» (atrasts, īsi ko), «Nav», «Nav datu» (objekts nav atrasts / nav ģeometrijas), «Nav pārklājuma» (avotā šai teritorijai nav datu, piem., nav plūdu kartes). Pēc tam īss paskaidrojums.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>• Pārbaudes datums: datums, kad veicāt pārbaudi (GGGG-MM-DD). Svarīgi, jo dati laika gaitā mainās.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>• Avoti un piezīmes: kurus portālus izmantojāt un citas piezīmes.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Kolonnu krāsas: tumši zila = obligāta, gaiši zila = neobligāta. Virsrakstu piezīmēs (sarkanais stūrītis) – paskaidrojums.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Kolonnu krāsas: tumši zila = obligāta, gaiši zila = neobligāta. Virsrakstu piezīmēs (sarkanais stūrītis) – paskaidrojums.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Kolonnu nosaukumus nemainiet; der arī vecie nosaukumi (vertiba, projekta_nr, pieteicejs_reg_nr, adrese, veids).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Moduļi:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>m1 Kadastra dati: zemes vienības / būves, platība, lietošanas mērķis, būves uz zemes vienības.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>m2 Adreses atbilstība: vai norādītā adrese atbilst kadastra objektam («Neatbilst»).</t>
+          <t>m1 Kadastra dati: zemes vienības / būves, platība, lietošanas mērķis, būves uz zemes vienības.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>m3 Aizsargājamā daba: ĪADT, mikroliegums, mikrolieguma buferzona, dabas piemineklis, aizsargājams biotops (katru atsevišķi).</t>
+          <t>m2 Adreses atbilstība: vai adrese pieteikumā (kolonna „Adrese pieteikumā”) atbilst kadastra objektam («Neatbilst»).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>m4 Plūdi: 3. cikla pavasara palu karte, reizi 10 gados (10 % varbūtība). Vai objekts ir plūdu zonā, aptuvenais pārklājums.</t>
+          <t>m3 Aizsargājamā daba: ĪADT, mikroliegums, mikrolieguma buferzona, dabas piemineklis, aizsargājams biotops (katru atsevišķi).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>m5 Būvniecības lietas (BIS): lietas uz šī objekta; norādiet BIS lietas numurus un vai tās ir tieši uz objekta vai blakus.</t>
+          <t>m4 Plūdi: 3. cikla pavasara palu karte, reizi 10 gados (10 % varbūtība). Vai objekts ir plūdu zonā, aptuvenais pārklājums.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>m5 Būvniecības lietas (BIS): lietas uz šī objekta; norādiet BIS lietas numurus un vai tās ir tieši uz objekta vai blakus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>m6 Apgrūtinājumi: kadastrā reģistrētie apgrūtinājumi (kods vai nosaukums).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Lūdzam testa kopā iekļaut:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>• vismaz vienu zemes vienību, kas atrodas 10 gadu plūdu zonā;</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• vismaz vienu objektu ārpus plūdu karšu pārklājuma (teritorijā, kurai plūdu karte nav izstrādāta);</t>
+          <t>• vismaz vienu zemes vienību, kas atrodas 10 gadu plūdu zonā;</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>• vismaz vienu objektu ārpus plūdu karšu pārklājuma (teritorijā, kurai plūdu karte nav izstrādāta);</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>• ja iespējams: objektu ar būvniecības lietu, objektu dabas teritorijā un objektu ar vairākām zemes vienībām vai būvēm.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Dzeltenās rindas ir piemēri: izdzēsiet tās vai aizstājiet ar saviem datiem.</t>
         </is>
@@ -750,21 +762,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L501"/>
+  <dimension ref="A1:M501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -780,50 +793,55 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Adrese pieteikumā (atbilstības pārbaudei)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Objekta veids: īpašums / zemes vienība / būve (ja numurs divdomīgs)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Pieteicēja reģ. Nr. (tikai juridiskām personām)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>M1 Kadastra dati</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>M2 Adreses atbilstība</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>M3 Aizsargājamā daba</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>M4 Plūdi (10 gadi)</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>M5 Būvniecības lietas (BIS)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>M6 Apgrūtinājumi</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Pārbaudes datums</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Avoti un piezīmes</t>
         </is>
@@ -842,46 +860,51 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
+          <t>Tautas iela 11, Daugavpils</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
           <t>īpašums</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>90000077325</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="8" t="n"/>
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>Piemērs no sākotnējiem datiem: Daugavpils, Tautas iela 11. Atbildes aizpilda kolēģis.</t>
         </is>
@@ -900,38 +923,39 @@
       </c>
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>‹Ir: … / Nav / Nav datu / Nav pārklājuma›</t>
         </is>
       </c>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="8" t="n"/>
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Piemērs no sākotnējiem datiem: Jelgava. Atbildes aizpilda kolēģis.</t>
         </is>
@@ -942,3493 +966,3991 @@
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="9" t="n"/>
       <c r="D4" s="9" t="n"/>
-      <c r="K4" s="10" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="L4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>
-      <c r="K5" s="10" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="L5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="9" t="n"/>
       <c r="D6" s="9" t="n"/>
-      <c r="K6" s="10" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="L6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="9" t="n"/>
       <c r="D7" s="9" t="n"/>
-      <c r="K7" s="10" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="L7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="9" t="n"/>
-      <c r="K8" s="10" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="L8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
-      <c r="K9" s="10" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="L9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="9" t="n"/>
-      <c r="K10" s="10" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="L10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n"/>
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="n"/>
-      <c r="K11" s="10" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="L11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
-      <c r="K12" s="10" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="L12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="9" t="n"/>
-      <c r="K13" s="10" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="L13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n"/>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
-      <c r="K14" s="10" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="L14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="9" t="n"/>
-      <c r="K15" s="10" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="L15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
-      <c r="K16" s="10" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="L16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="9" t="n"/>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="9" t="n"/>
-      <c r="K17" s="10" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="L17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n"/>
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9" t="n"/>
-      <c r="K18" s="10" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="L18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n"/>
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="9" t="n"/>
-      <c r="K19" s="10" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="L19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n"/>
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9" t="n"/>
-      <c r="K20" s="10" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="L20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n"/>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="n"/>
-      <c r="K21" s="10" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="L21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="n"/>
-      <c r="K22" s="10" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="L22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n"/>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
-      <c r="K23" s="10" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="L23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n"/>
       <c r="B24" s="9" t="n"/>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
-      <c r="K24" s="10" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="L24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="n"/>
-      <c r="K25" s="10" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="L25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n"/>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
-      <c r="K26" s="10" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="L26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
-      <c r="K27" s="10" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="L27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
-      <c r="K28" s="10" t="n"/>
+      <c r="E28" s="9" t="n"/>
+      <c r="L28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="9" t="n"/>
-      <c r="K29" s="10" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="L29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n"/>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="n"/>
-      <c r="K30" s="10" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="L30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
       <c r="B31" s="9" t="n"/>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="n"/>
-      <c r="K31" s="10" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="L31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n"/>
       <c r="B32" s="9" t="n"/>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
-      <c r="K32" s="10" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="L32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="9" t="n"/>
       <c r="D33" s="9" t="n"/>
-      <c r="K33" s="10" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="L33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n"/>
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
-      <c r="K34" s="10" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="L34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n"/>
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="n"/>
-      <c r="K35" s="10" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="L35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n"/>
       <c r="B36" s="9" t="n"/>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="n"/>
-      <c r="K36" s="10" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="L36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
       <c r="B37" s="9" t="n"/>
       <c r="C37" s="9" t="n"/>
       <c r="D37" s="9" t="n"/>
-      <c r="K37" s="10" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="L37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n"/>
       <c r="B38" s="9" t="n"/>
       <c r="C38" s="9" t="n"/>
       <c r="D38" s="9" t="n"/>
-      <c r="K38" s="10" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="L38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
       <c r="B39" s="9" t="n"/>
       <c r="C39" s="9" t="n"/>
       <c r="D39" s="9" t="n"/>
-      <c r="K39" s="10" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="L39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n"/>
       <c r="B40" s="9" t="n"/>
       <c r="C40" s="9" t="n"/>
       <c r="D40" s="9" t="n"/>
-      <c r="K40" s="10" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="L40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
       <c r="B41" s="9" t="n"/>
       <c r="C41" s="9" t="n"/>
       <c r="D41" s="9" t="n"/>
-      <c r="K41" s="10" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="L41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n"/>
       <c r="B42" s="9" t="n"/>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="9" t="n"/>
-      <c r="K42" s="10" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="L42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n"/>
       <c r="B43" s="9" t="n"/>
       <c r="C43" s="9" t="n"/>
       <c r="D43" s="9" t="n"/>
-      <c r="K43" s="10" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="L43" s="10" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n"/>
       <c r="B44" s="9" t="n"/>
       <c r="C44" s="9" t="n"/>
       <c r="D44" s="9" t="n"/>
-      <c r="K44" s="10" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="L44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
       <c r="B45" s="9" t="n"/>
       <c r="C45" s="9" t="n"/>
       <c r="D45" s="9" t="n"/>
-      <c r="K45" s="10" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="L45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n"/>
       <c r="B46" s="9" t="n"/>
       <c r="C46" s="9" t="n"/>
       <c r="D46" s="9" t="n"/>
-      <c r="K46" s="10" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="L46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n"/>
       <c r="B47" s="9" t="n"/>
       <c r="C47" s="9" t="n"/>
       <c r="D47" s="9" t="n"/>
-      <c r="K47" s="10" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="L47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n"/>
       <c r="B48" s="9" t="n"/>
       <c r="C48" s="9" t="n"/>
       <c r="D48" s="9" t="n"/>
-      <c r="K48" s="10" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="L48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
       <c r="B49" s="9" t="n"/>
       <c r="C49" s="9" t="n"/>
       <c r="D49" s="9" t="n"/>
-      <c r="K49" s="10" t="n"/>
+      <c r="E49" s="9" t="n"/>
+      <c r="L49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n"/>
       <c r="B50" s="9" t="n"/>
       <c r="C50" s="9" t="n"/>
       <c r="D50" s="9" t="n"/>
-      <c r="K50" s="10" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="L50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n"/>
       <c r="B51" s="9" t="n"/>
       <c r="C51" s="9" t="n"/>
       <c r="D51" s="9" t="n"/>
-      <c r="K51" s="10" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="L51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n"/>
       <c r="B52" s="9" t="n"/>
       <c r="C52" s="9" t="n"/>
       <c r="D52" s="9" t="n"/>
-      <c r="K52" s="10" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="L52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n"/>
       <c r="B53" s="9" t="n"/>
       <c r="C53" s="9" t="n"/>
       <c r="D53" s="9" t="n"/>
-      <c r="K53" s="10" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="L53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n"/>
       <c r="B54" s="9" t="n"/>
       <c r="C54" s="9" t="n"/>
       <c r="D54" s="9" t="n"/>
-      <c r="K54" s="10" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="L54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n"/>
       <c r="B55" s="9" t="n"/>
       <c r="C55" s="9" t="n"/>
       <c r="D55" s="9" t="n"/>
-      <c r="K55" s="10" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="L55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n"/>
       <c r="B56" s="9" t="n"/>
       <c r="C56" s="9" t="n"/>
       <c r="D56" s="9" t="n"/>
-      <c r="K56" s="10" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="L56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n"/>
       <c r="B57" s="9" t="n"/>
       <c r="C57" s="9" t="n"/>
       <c r="D57" s="9" t="n"/>
-      <c r="K57" s="10" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="L57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n"/>
       <c r="B58" s="9" t="n"/>
       <c r="C58" s="9" t="n"/>
       <c r="D58" s="9" t="n"/>
-      <c r="K58" s="10" t="n"/>
+      <c r="E58" s="9" t="n"/>
+      <c r="L58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n"/>
       <c r="B59" s="9" t="n"/>
       <c r="C59" s="9" t="n"/>
       <c r="D59" s="9" t="n"/>
-      <c r="K59" s="10" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="L59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n"/>
       <c r="B60" s="9" t="n"/>
       <c r="C60" s="9" t="n"/>
       <c r="D60" s="9" t="n"/>
-      <c r="K60" s="10" t="n"/>
+      <c r="E60" s="9" t="n"/>
+      <c r="L60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n"/>
       <c r="B61" s="9" t="n"/>
       <c r="C61" s="9" t="n"/>
       <c r="D61" s="9" t="n"/>
-      <c r="K61" s="10" t="n"/>
+      <c r="E61" s="9" t="n"/>
+      <c r="L61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n"/>
       <c r="B62" s="9" t="n"/>
       <c r="C62" s="9" t="n"/>
       <c r="D62" s="9" t="n"/>
-      <c r="K62" s="10" t="n"/>
+      <c r="E62" s="9" t="n"/>
+      <c r="L62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n"/>
       <c r="B63" s="9" t="n"/>
       <c r="C63" s="9" t="n"/>
       <c r="D63" s="9" t="n"/>
-      <c r="K63" s="10" t="n"/>
+      <c r="E63" s="9" t="n"/>
+      <c r="L63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n"/>
       <c r="B64" s="9" t="n"/>
       <c r="C64" s="9" t="n"/>
       <c r="D64" s="9" t="n"/>
-      <c r="K64" s="10" t="n"/>
+      <c r="E64" s="9" t="n"/>
+      <c r="L64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n"/>
       <c r="B65" s="9" t="n"/>
       <c r="C65" s="9" t="n"/>
       <c r="D65" s="9" t="n"/>
-      <c r="K65" s="10" t="n"/>
+      <c r="E65" s="9" t="n"/>
+      <c r="L65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n"/>
       <c r="B66" s="9" t="n"/>
       <c r="C66" s="9" t="n"/>
       <c r="D66" s="9" t="n"/>
-      <c r="K66" s="10" t="n"/>
+      <c r="E66" s="9" t="n"/>
+      <c r="L66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n"/>
       <c r="B67" s="9" t="n"/>
       <c r="C67" s="9" t="n"/>
       <c r="D67" s="9" t="n"/>
-      <c r="K67" s="10" t="n"/>
+      <c r="E67" s="9" t="n"/>
+      <c r="L67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n"/>
       <c r="B68" s="9" t="n"/>
       <c r="C68" s="9" t="n"/>
       <c r="D68" s="9" t="n"/>
-      <c r="K68" s="10" t="n"/>
+      <c r="E68" s="9" t="n"/>
+      <c r="L68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n"/>
       <c r="B69" s="9" t="n"/>
       <c r="C69" s="9" t="n"/>
       <c r="D69" s="9" t="n"/>
-      <c r="K69" s="10" t="n"/>
+      <c r="E69" s="9" t="n"/>
+      <c r="L69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n"/>
       <c r="B70" s="9" t="n"/>
       <c r="C70" s="9" t="n"/>
       <c r="D70" s="9" t="n"/>
-      <c r="K70" s="10" t="n"/>
+      <c r="E70" s="9" t="n"/>
+      <c r="L70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n"/>
       <c r="B71" s="9" t="n"/>
       <c r="C71" s="9" t="n"/>
       <c r="D71" s="9" t="n"/>
-      <c r="K71" s="10" t="n"/>
+      <c r="E71" s="9" t="n"/>
+      <c r="L71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n"/>
       <c r="B72" s="9" t="n"/>
       <c r="C72" s="9" t="n"/>
       <c r="D72" s="9" t="n"/>
-      <c r="K72" s="10" t="n"/>
+      <c r="E72" s="9" t="n"/>
+      <c r="L72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n"/>
       <c r="B73" s="9" t="n"/>
       <c r="C73" s="9" t="n"/>
       <c r="D73" s="9" t="n"/>
-      <c r="K73" s="10" t="n"/>
+      <c r="E73" s="9" t="n"/>
+      <c r="L73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n"/>
       <c r="B74" s="9" t="n"/>
       <c r="C74" s="9" t="n"/>
       <c r="D74" s="9" t="n"/>
-      <c r="K74" s="10" t="n"/>
+      <c r="E74" s="9" t="n"/>
+      <c r="L74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n"/>
       <c r="B75" s="9" t="n"/>
       <c r="C75" s="9" t="n"/>
       <c r="D75" s="9" t="n"/>
-      <c r="K75" s="10" t="n"/>
+      <c r="E75" s="9" t="n"/>
+      <c r="L75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n"/>
       <c r="B76" s="9" t="n"/>
       <c r="C76" s="9" t="n"/>
       <c r="D76" s="9" t="n"/>
-      <c r="K76" s="10" t="n"/>
+      <c r="E76" s="9" t="n"/>
+      <c r="L76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n"/>
       <c r="B77" s="9" t="n"/>
       <c r="C77" s="9" t="n"/>
       <c r="D77" s="9" t="n"/>
-      <c r="K77" s="10" t="n"/>
+      <c r="E77" s="9" t="n"/>
+      <c r="L77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n"/>
       <c r="B78" s="9" t="n"/>
       <c r="C78" s="9" t="n"/>
       <c r="D78" s="9" t="n"/>
-      <c r="K78" s="10" t="n"/>
+      <c r="E78" s="9" t="n"/>
+      <c r="L78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n"/>
       <c r="B79" s="9" t="n"/>
       <c r="C79" s="9" t="n"/>
       <c r="D79" s="9" t="n"/>
-      <c r="K79" s="10" t="n"/>
+      <c r="E79" s="9" t="n"/>
+      <c r="L79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n"/>
       <c r="B80" s="9" t="n"/>
       <c r="C80" s="9" t="n"/>
       <c r="D80" s="9" t="n"/>
-      <c r="K80" s="10" t="n"/>
+      <c r="E80" s="9" t="n"/>
+      <c r="L80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n"/>
       <c r="B81" s="9" t="n"/>
       <c r="C81" s="9" t="n"/>
       <c r="D81" s="9" t="n"/>
-      <c r="K81" s="10" t="n"/>
+      <c r="E81" s="9" t="n"/>
+      <c r="L81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n"/>
       <c r="B82" s="9" t="n"/>
       <c r="C82" s="9" t="n"/>
       <c r="D82" s="9" t="n"/>
-      <c r="K82" s="10" t="n"/>
+      <c r="E82" s="9" t="n"/>
+      <c r="L82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n"/>
       <c r="B83" s="9" t="n"/>
       <c r="C83" s="9" t="n"/>
       <c r="D83" s="9" t="n"/>
-      <c r="K83" s="10" t="n"/>
+      <c r="E83" s="9" t="n"/>
+      <c r="L83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n"/>
       <c r="B84" s="9" t="n"/>
       <c r="C84" s="9" t="n"/>
       <c r="D84" s="9" t="n"/>
-      <c r="K84" s="10" t="n"/>
+      <c r="E84" s="9" t="n"/>
+      <c r="L84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n"/>
       <c r="B85" s="9" t="n"/>
       <c r="C85" s="9" t="n"/>
       <c r="D85" s="9" t="n"/>
-      <c r="K85" s="10" t="n"/>
+      <c r="E85" s="9" t="n"/>
+      <c r="L85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n"/>
       <c r="B86" s="9" t="n"/>
       <c r="C86" s="9" t="n"/>
       <c r="D86" s="9" t="n"/>
-      <c r="K86" s="10" t="n"/>
+      <c r="E86" s="9" t="n"/>
+      <c r="L86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n"/>
       <c r="B87" s="9" t="n"/>
       <c r="C87" s="9" t="n"/>
       <c r="D87" s="9" t="n"/>
-      <c r="K87" s="10" t="n"/>
+      <c r="E87" s="9" t="n"/>
+      <c r="L87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n"/>
       <c r="B88" s="9" t="n"/>
       <c r="C88" s="9" t="n"/>
       <c r="D88" s="9" t="n"/>
-      <c r="K88" s="10" t="n"/>
+      <c r="E88" s="9" t="n"/>
+      <c r="L88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n"/>
       <c r="B89" s="9" t="n"/>
       <c r="C89" s="9" t="n"/>
       <c r="D89" s="9" t="n"/>
-      <c r="K89" s="10" t="n"/>
+      <c r="E89" s="9" t="n"/>
+      <c r="L89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n"/>
       <c r="B90" s="9" t="n"/>
       <c r="C90" s="9" t="n"/>
       <c r="D90" s="9" t="n"/>
-      <c r="K90" s="10" t="n"/>
+      <c r="E90" s="9" t="n"/>
+      <c r="L90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n"/>
       <c r="B91" s="9" t="n"/>
       <c r="C91" s="9" t="n"/>
       <c r="D91" s="9" t="n"/>
-      <c r="K91" s="10" t="n"/>
+      <c r="E91" s="9" t="n"/>
+      <c r="L91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="9" t="n"/>
       <c r="B92" s="9" t="n"/>
       <c r="C92" s="9" t="n"/>
       <c r="D92" s="9" t="n"/>
-      <c r="K92" s="10" t="n"/>
+      <c r="E92" s="9" t="n"/>
+      <c r="L92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n"/>
       <c r="B93" s="9" t="n"/>
       <c r="C93" s="9" t="n"/>
       <c r="D93" s="9" t="n"/>
-      <c r="K93" s="10" t="n"/>
+      <c r="E93" s="9" t="n"/>
+      <c r="L93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="9" t="n"/>
       <c r="B94" s="9" t="n"/>
       <c r="C94" s="9" t="n"/>
       <c r="D94" s="9" t="n"/>
-      <c r="K94" s="10" t="n"/>
+      <c r="E94" s="9" t="n"/>
+      <c r="L94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n"/>
       <c r="B95" s="9" t="n"/>
       <c r="C95" s="9" t="n"/>
       <c r="D95" s="9" t="n"/>
-      <c r="K95" s="10" t="n"/>
+      <c r="E95" s="9" t="n"/>
+      <c r="L95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="9" t="n"/>
       <c r="B96" s="9" t="n"/>
       <c r="C96" s="9" t="n"/>
       <c r="D96" s="9" t="n"/>
-      <c r="K96" s="10" t="n"/>
+      <c r="E96" s="9" t="n"/>
+      <c r="L96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n"/>
       <c r="B97" s="9" t="n"/>
       <c r="C97" s="9" t="n"/>
       <c r="D97" s="9" t="n"/>
-      <c r="K97" s="10" t="n"/>
+      <c r="E97" s="9" t="n"/>
+      <c r="L97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n"/>
       <c r="B98" s="9" t="n"/>
       <c r="C98" s="9" t="n"/>
       <c r="D98" s="9" t="n"/>
-      <c r="K98" s="10" t="n"/>
+      <c r="E98" s="9" t="n"/>
+      <c r="L98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n"/>
       <c r="B99" s="9" t="n"/>
       <c r="C99" s="9" t="n"/>
       <c r="D99" s="9" t="n"/>
-      <c r="K99" s="10" t="n"/>
+      <c r="E99" s="9" t="n"/>
+      <c r="L99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n"/>
       <c r="B100" s="9" t="n"/>
       <c r="C100" s="9" t="n"/>
       <c r="D100" s="9" t="n"/>
-      <c r="K100" s="10" t="n"/>
+      <c r="E100" s="9" t="n"/>
+      <c r="L100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n"/>
       <c r="B101" s="9" t="n"/>
       <c r="C101" s="9" t="n"/>
       <c r="D101" s="9" t="n"/>
-      <c r="K101" s="10" t="n"/>
+      <c r="E101" s="9" t="n"/>
+      <c r="L101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n"/>
       <c r="B102" s="9" t="n"/>
       <c r="C102" s="9" t="n"/>
       <c r="D102" s="9" t="n"/>
-      <c r="K102" s="10" t="n"/>
+      <c r="E102" s="9" t="n"/>
+      <c r="L102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n"/>
       <c r="B103" s="9" t="n"/>
       <c r="C103" s="9" t="n"/>
       <c r="D103" s="9" t="n"/>
-      <c r="K103" s="10" t="n"/>
+      <c r="E103" s="9" t="n"/>
+      <c r="L103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n"/>
       <c r="B104" s="9" t="n"/>
       <c r="C104" s="9" t="n"/>
       <c r="D104" s="9" t="n"/>
-      <c r="K104" s="10" t="n"/>
+      <c r="E104" s="9" t="n"/>
+      <c r="L104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n"/>
       <c r="B105" s="9" t="n"/>
       <c r="C105" s="9" t="n"/>
       <c r="D105" s="9" t="n"/>
-      <c r="K105" s="10" t="n"/>
+      <c r="E105" s="9" t="n"/>
+      <c r="L105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n"/>
       <c r="B106" s="9" t="n"/>
       <c r="C106" s="9" t="n"/>
       <c r="D106" s="9" t="n"/>
-      <c r="K106" s="10" t="n"/>
+      <c r="E106" s="9" t="n"/>
+      <c r="L106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n"/>
       <c r="B107" s="9" t="n"/>
       <c r="C107" s="9" t="n"/>
       <c r="D107" s="9" t="n"/>
-      <c r="K107" s="10" t="n"/>
+      <c r="E107" s="9" t="n"/>
+      <c r="L107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n"/>
       <c r="B108" s="9" t="n"/>
       <c r="C108" s="9" t="n"/>
       <c r="D108" s="9" t="n"/>
-      <c r="K108" s="10" t="n"/>
+      <c r="E108" s="9" t="n"/>
+      <c r="L108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n"/>
       <c r="B109" s="9" t="n"/>
       <c r="C109" s="9" t="n"/>
       <c r="D109" s="9" t="n"/>
-      <c r="K109" s="10" t="n"/>
+      <c r="E109" s="9" t="n"/>
+      <c r="L109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n"/>
       <c r="B110" s="9" t="n"/>
       <c r="C110" s="9" t="n"/>
       <c r="D110" s="9" t="n"/>
-      <c r="K110" s="10" t="n"/>
+      <c r="E110" s="9" t="n"/>
+      <c r="L110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="9" t="n"/>
       <c r="B111" s="9" t="n"/>
       <c r="C111" s="9" t="n"/>
       <c r="D111" s="9" t="n"/>
-      <c r="K111" s="10" t="n"/>
+      <c r="E111" s="9" t="n"/>
+      <c r="L111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="9" t="n"/>
       <c r="B112" s="9" t="n"/>
       <c r="C112" s="9" t="n"/>
       <c r="D112" s="9" t="n"/>
-      <c r="K112" s="10" t="n"/>
+      <c r="E112" s="9" t="n"/>
+      <c r="L112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="9" t="n"/>
       <c r="B113" s="9" t="n"/>
       <c r="C113" s="9" t="n"/>
       <c r="D113" s="9" t="n"/>
-      <c r="K113" s="10" t="n"/>
+      <c r="E113" s="9" t="n"/>
+      <c r="L113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="9" t="n"/>
       <c r="B114" s="9" t="n"/>
       <c r="C114" s="9" t="n"/>
       <c r="D114" s="9" t="n"/>
-      <c r="K114" s="10" t="n"/>
+      <c r="E114" s="9" t="n"/>
+      <c r="L114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n"/>
       <c r="B115" s="9" t="n"/>
       <c r="C115" s="9" t="n"/>
       <c r="D115" s="9" t="n"/>
-      <c r="K115" s="10" t="n"/>
+      <c r="E115" s="9" t="n"/>
+      <c r="L115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="9" t="n"/>
       <c r="B116" s="9" t="n"/>
       <c r="C116" s="9" t="n"/>
       <c r="D116" s="9" t="n"/>
-      <c r="K116" s="10" t="n"/>
+      <c r="E116" s="9" t="n"/>
+      <c r="L116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="9" t="n"/>
       <c r="B117" s="9" t="n"/>
       <c r="C117" s="9" t="n"/>
       <c r="D117" s="9" t="n"/>
-      <c r="K117" s="10" t="n"/>
+      <c r="E117" s="9" t="n"/>
+      <c r="L117" s="10" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="9" t="n"/>
       <c r="B118" s="9" t="n"/>
       <c r="C118" s="9" t="n"/>
       <c r="D118" s="9" t="n"/>
-      <c r="K118" s="10" t="n"/>
+      <c r="E118" s="9" t="n"/>
+      <c r="L118" s="10" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="9" t="n"/>
       <c r="B119" s="9" t="n"/>
       <c r="C119" s="9" t="n"/>
       <c r="D119" s="9" t="n"/>
-      <c r="K119" s="10" t="n"/>
+      <c r="E119" s="9" t="n"/>
+      <c r="L119" s="10" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="9" t="n"/>
       <c r="B120" s="9" t="n"/>
       <c r="C120" s="9" t="n"/>
       <c r="D120" s="9" t="n"/>
-      <c r="K120" s="10" t="n"/>
+      <c r="E120" s="9" t="n"/>
+      <c r="L120" s="10" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="9" t="n"/>
       <c r="B121" s="9" t="n"/>
       <c r="C121" s="9" t="n"/>
       <c r="D121" s="9" t="n"/>
-      <c r="K121" s="10" t="n"/>
+      <c r="E121" s="9" t="n"/>
+      <c r="L121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="9" t="n"/>
       <c r="B122" s="9" t="n"/>
       <c r="C122" s="9" t="n"/>
       <c r="D122" s="9" t="n"/>
-      <c r="K122" s="10" t="n"/>
+      <c r="E122" s="9" t="n"/>
+      <c r="L122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="9" t="n"/>
       <c r="B123" s="9" t="n"/>
       <c r="C123" s="9" t="n"/>
       <c r="D123" s="9" t="n"/>
-      <c r="K123" s="10" t="n"/>
+      <c r="E123" s="9" t="n"/>
+      <c r="L123" s="10" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="9" t="n"/>
       <c r="B124" s="9" t="n"/>
       <c r="C124" s="9" t="n"/>
       <c r="D124" s="9" t="n"/>
-      <c r="K124" s="10" t="n"/>
+      <c r="E124" s="9" t="n"/>
+      <c r="L124" s="10" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="9" t="n"/>
       <c r="B125" s="9" t="n"/>
       <c r="C125" s="9" t="n"/>
       <c r="D125" s="9" t="n"/>
-      <c r="K125" s="10" t="n"/>
+      <c r="E125" s="9" t="n"/>
+      <c r="L125" s="10" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="9" t="n"/>
       <c r="B126" s="9" t="n"/>
       <c r="C126" s="9" t="n"/>
       <c r="D126" s="9" t="n"/>
-      <c r="K126" s="10" t="n"/>
+      <c r="E126" s="9" t="n"/>
+      <c r="L126" s="10" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="9" t="n"/>
       <c r="B127" s="9" t="n"/>
       <c r="C127" s="9" t="n"/>
       <c r="D127" s="9" t="n"/>
-      <c r="K127" s="10" t="n"/>
+      <c r="E127" s="9" t="n"/>
+      <c r="L127" s="10" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="9" t="n"/>
       <c r="B128" s="9" t="n"/>
       <c r="C128" s="9" t="n"/>
       <c r="D128" s="9" t="n"/>
-      <c r="K128" s="10" t="n"/>
+      <c r="E128" s="9" t="n"/>
+      <c r="L128" s="10" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="9" t="n"/>
       <c r="B129" s="9" t="n"/>
       <c r="C129" s="9" t="n"/>
       <c r="D129" s="9" t="n"/>
-      <c r="K129" s="10" t="n"/>
+      <c r="E129" s="9" t="n"/>
+      <c r="L129" s="10" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="9" t="n"/>
       <c r="B130" s="9" t="n"/>
       <c r="C130" s="9" t="n"/>
       <c r="D130" s="9" t="n"/>
-      <c r="K130" s="10" t="n"/>
+      <c r="E130" s="9" t="n"/>
+      <c r="L130" s="10" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="9" t="n"/>
       <c r="B131" s="9" t="n"/>
       <c r="C131" s="9" t="n"/>
       <c r="D131" s="9" t="n"/>
-      <c r="K131" s="10" t="n"/>
+      <c r="E131" s="9" t="n"/>
+      <c r="L131" s="10" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="9" t="n"/>
       <c r="B132" s="9" t="n"/>
       <c r="C132" s="9" t="n"/>
       <c r="D132" s="9" t="n"/>
-      <c r="K132" s="10" t="n"/>
+      <c r="E132" s="9" t="n"/>
+      <c r="L132" s="10" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="9" t="n"/>
       <c r="B133" s="9" t="n"/>
       <c r="C133" s="9" t="n"/>
       <c r="D133" s="9" t="n"/>
-      <c r="K133" s="10" t="n"/>
+      <c r="E133" s="9" t="n"/>
+      <c r="L133" s="10" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="9" t="n"/>
       <c r="B134" s="9" t="n"/>
       <c r="C134" s="9" t="n"/>
       <c r="D134" s="9" t="n"/>
-      <c r="K134" s="10" t="n"/>
+      <c r="E134" s="9" t="n"/>
+      <c r="L134" s="10" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="9" t="n"/>
       <c r="B135" s="9" t="n"/>
       <c r="C135" s="9" t="n"/>
       <c r="D135" s="9" t="n"/>
-      <c r="K135" s="10" t="n"/>
+      <c r="E135" s="9" t="n"/>
+      <c r="L135" s="10" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="9" t="n"/>
       <c r="B136" s="9" t="n"/>
       <c r="C136" s="9" t="n"/>
       <c r="D136" s="9" t="n"/>
-      <c r="K136" s="10" t="n"/>
+      <c r="E136" s="9" t="n"/>
+      <c r="L136" s="10" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="9" t="n"/>
       <c r="B137" s="9" t="n"/>
       <c r="C137" s="9" t="n"/>
       <c r="D137" s="9" t="n"/>
-      <c r="K137" s="10" t="n"/>
+      <c r="E137" s="9" t="n"/>
+      <c r="L137" s="10" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="9" t="n"/>
       <c r="B138" s="9" t="n"/>
       <c r="C138" s="9" t="n"/>
       <c r="D138" s="9" t="n"/>
-      <c r="K138" s="10" t="n"/>
+      <c r="E138" s="9" t="n"/>
+      <c r="L138" s="10" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="9" t="n"/>
       <c r="B139" s="9" t="n"/>
       <c r="C139" s="9" t="n"/>
       <c r="D139" s="9" t="n"/>
-      <c r="K139" s="10" t="n"/>
+      <c r="E139" s="9" t="n"/>
+      <c r="L139" s="10" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="9" t="n"/>
       <c r="B140" s="9" t="n"/>
       <c r="C140" s="9" t="n"/>
       <c r="D140" s="9" t="n"/>
-      <c r="K140" s="10" t="n"/>
+      <c r="E140" s="9" t="n"/>
+      <c r="L140" s="10" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="9" t="n"/>
       <c r="B141" s="9" t="n"/>
       <c r="C141" s="9" t="n"/>
       <c r="D141" s="9" t="n"/>
-      <c r="K141" s="10" t="n"/>
+      <c r="E141" s="9" t="n"/>
+      <c r="L141" s="10" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="n"/>
       <c r="B142" s="9" t="n"/>
       <c r="C142" s="9" t="n"/>
       <c r="D142" s="9" t="n"/>
-      <c r="K142" s="10" t="n"/>
+      <c r="E142" s="9" t="n"/>
+      <c r="L142" s="10" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="9" t="n"/>
       <c r="B143" s="9" t="n"/>
       <c r="C143" s="9" t="n"/>
       <c r="D143" s="9" t="n"/>
-      <c r="K143" s="10" t="n"/>
+      <c r="E143" s="9" t="n"/>
+      <c r="L143" s="10" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="9" t="n"/>
       <c r="B144" s="9" t="n"/>
       <c r="C144" s="9" t="n"/>
       <c r="D144" s="9" t="n"/>
-      <c r="K144" s="10" t="n"/>
+      <c r="E144" s="9" t="n"/>
+      <c r="L144" s="10" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="9" t="n"/>
       <c r="B145" s="9" t="n"/>
       <c r="C145" s="9" t="n"/>
       <c r="D145" s="9" t="n"/>
-      <c r="K145" s="10" t="n"/>
+      <c r="E145" s="9" t="n"/>
+      <c r="L145" s="10" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="9" t="n"/>
       <c r="B146" s="9" t="n"/>
       <c r="C146" s="9" t="n"/>
       <c r="D146" s="9" t="n"/>
-      <c r="K146" s="10" t="n"/>
+      <c r="E146" s="9" t="n"/>
+      <c r="L146" s="10" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="n"/>
       <c r="B147" s="9" t="n"/>
       <c r="C147" s="9" t="n"/>
       <c r="D147" s="9" t="n"/>
-      <c r="K147" s="10" t="n"/>
+      <c r="E147" s="9" t="n"/>
+      <c r="L147" s="10" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="9" t="n"/>
       <c r="B148" s="9" t="n"/>
       <c r="C148" s="9" t="n"/>
       <c r="D148" s="9" t="n"/>
-      <c r="K148" s="10" t="n"/>
+      <c r="E148" s="9" t="n"/>
+      <c r="L148" s="10" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="9" t="n"/>
       <c r="B149" s="9" t="n"/>
       <c r="C149" s="9" t="n"/>
       <c r="D149" s="9" t="n"/>
-      <c r="K149" s="10" t="n"/>
+      <c r="E149" s="9" t="n"/>
+      <c r="L149" s="10" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="9" t="n"/>
       <c r="B150" s="9" t="n"/>
       <c r="C150" s="9" t="n"/>
       <c r="D150" s="9" t="n"/>
-      <c r="K150" s="10" t="n"/>
+      <c r="E150" s="9" t="n"/>
+      <c r="L150" s="10" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="9" t="n"/>
       <c r="B151" s="9" t="n"/>
       <c r="C151" s="9" t="n"/>
       <c r="D151" s="9" t="n"/>
-      <c r="K151" s="10" t="n"/>
+      <c r="E151" s="9" t="n"/>
+      <c r="L151" s="10" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="9" t="n"/>
       <c r="B152" s="9" t="n"/>
       <c r="C152" s="9" t="n"/>
       <c r="D152" s="9" t="n"/>
-      <c r="K152" s="10" t="n"/>
+      <c r="E152" s="9" t="n"/>
+      <c r="L152" s="10" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="9" t="n"/>
       <c r="B153" s="9" t="n"/>
       <c r="C153" s="9" t="n"/>
       <c r="D153" s="9" t="n"/>
-      <c r="K153" s="10" t="n"/>
+      <c r="E153" s="9" t="n"/>
+      <c r="L153" s="10" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="9" t="n"/>
       <c r="B154" s="9" t="n"/>
       <c r="C154" s="9" t="n"/>
       <c r="D154" s="9" t="n"/>
-      <c r="K154" s="10" t="n"/>
+      <c r="E154" s="9" t="n"/>
+      <c r="L154" s="10" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="9" t="n"/>
       <c r="B155" s="9" t="n"/>
       <c r="C155" s="9" t="n"/>
       <c r="D155" s="9" t="n"/>
-      <c r="K155" s="10" t="n"/>
+      <c r="E155" s="9" t="n"/>
+      <c r="L155" s="10" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="9" t="n"/>
       <c r="B156" s="9" t="n"/>
       <c r="C156" s="9" t="n"/>
       <c r="D156" s="9" t="n"/>
-      <c r="K156" s="10" t="n"/>
+      <c r="E156" s="9" t="n"/>
+      <c r="L156" s="10" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="9" t="n"/>
       <c r="B157" s="9" t="n"/>
       <c r="C157" s="9" t="n"/>
       <c r="D157" s="9" t="n"/>
-      <c r="K157" s="10" t="n"/>
+      <c r="E157" s="9" t="n"/>
+      <c r="L157" s="10" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="9" t="n"/>
       <c r="B158" s="9" t="n"/>
       <c r="C158" s="9" t="n"/>
       <c r="D158" s="9" t="n"/>
-      <c r="K158" s="10" t="n"/>
+      <c r="E158" s="9" t="n"/>
+      <c r="L158" s="10" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="9" t="n"/>
       <c r="B159" s="9" t="n"/>
       <c r="C159" s="9" t="n"/>
       <c r="D159" s="9" t="n"/>
-      <c r="K159" s="10" t="n"/>
+      <c r="E159" s="9" t="n"/>
+      <c r="L159" s="10" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="9" t="n"/>
       <c r="B160" s="9" t="n"/>
       <c r="C160" s="9" t="n"/>
       <c r="D160" s="9" t="n"/>
-      <c r="K160" s="10" t="n"/>
+      <c r="E160" s="9" t="n"/>
+      <c r="L160" s="10" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="9" t="n"/>
       <c r="B161" s="9" t="n"/>
       <c r="C161" s="9" t="n"/>
       <c r="D161" s="9" t="n"/>
-      <c r="K161" s="10" t="n"/>
+      <c r="E161" s="9" t="n"/>
+      <c r="L161" s="10" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="9" t="n"/>
       <c r="B162" s="9" t="n"/>
       <c r="C162" s="9" t="n"/>
       <c r="D162" s="9" t="n"/>
-      <c r="K162" s="10" t="n"/>
+      <c r="E162" s="9" t="n"/>
+      <c r="L162" s="10" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="9" t="n"/>
       <c r="B163" s="9" t="n"/>
       <c r="C163" s="9" t="n"/>
       <c r="D163" s="9" t="n"/>
-      <c r="K163" s="10" t="n"/>
+      <c r="E163" s="9" t="n"/>
+      <c r="L163" s="10" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="9" t="n"/>
       <c r="B164" s="9" t="n"/>
       <c r="C164" s="9" t="n"/>
       <c r="D164" s="9" t="n"/>
-      <c r="K164" s="10" t="n"/>
+      <c r="E164" s="9" t="n"/>
+      <c r="L164" s="10" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="9" t="n"/>
       <c r="B165" s="9" t="n"/>
       <c r="C165" s="9" t="n"/>
       <c r="D165" s="9" t="n"/>
-      <c r="K165" s="10" t="n"/>
+      <c r="E165" s="9" t="n"/>
+      <c r="L165" s="10" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="9" t="n"/>
       <c r="B166" s="9" t="n"/>
       <c r="C166" s="9" t="n"/>
       <c r="D166" s="9" t="n"/>
-      <c r="K166" s="10" t="n"/>
+      <c r="E166" s="9" t="n"/>
+      <c r="L166" s="10" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="9" t="n"/>
       <c r="B167" s="9" t="n"/>
       <c r="C167" s="9" t="n"/>
       <c r="D167" s="9" t="n"/>
-      <c r="K167" s="10" t="n"/>
+      <c r="E167" s="9" t="n"/>
+      <c r="L167" s="10" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="9" t="n"/>
       <c r="B168" s="9" t="n"/>
       <c r="C168" s="9" t="n"/>
       <c r="D168" s="9" t="n"/>
-      <c r="K168" s="10" t="n"/>
+      <c r="E168" s="9" t="n"/>
+      <c r="L168" s="10" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="9" t="n"/>
       <c r="B169" s="9" t="n"/>
       <c r="C169" s="9" t="n"/>
       <c r="D169" s="9" t="n"/>
-      <c r="K169" s="10" t="n"/>
+      <c r="E169" s="9" t="n"/>
+      <c r="L169" s="10" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="9" t="n"/>
       <c r="B170" s="9" t="n"/>
       <c r="C170" s="9" t="n"/>
       <c r="D170" s="9" t="n"/>
-      <c r="K170" s="10" t="n"/>
+      <c r="E170" s="9" t="n"/>
+      <c r="L170" s="10" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="9" t="n"/>
       <c r="B171" s="9" t="n"/>
       <c r="C171" s="9" t="n"/>
       <c r="D171" s="9" t="n"/>
-      <c r="K171" s="10" t="n"/>
+      <c r="E171" s="9" t="n"/>
+      <c r="L171" s="10" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="9" t="n"/>
       <c r="B172" s="9" t="n"/>
       <c r="C172" s="9" t="n"/>
       <c r="D172" s="9" t="n"/>
-      <c r="K172" s="10" t="n"/>
+      <c r="E172" s="9" t="n"/>
+      <c r="L172" s="10" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="9" t="n"/>
       <c r="B173" s="9" t="n"/>
       <c r="C173" s="9" t="n"/>
       <c r="D173" s="9" t="n"/>
-      <c r="K173" s="10" t="n"/>
+      <c r="E173" s="9" t="n"/>
+      <c r="L173" s="10" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="9" t="n"/>
       <c r="B174" s="9" t="n"/>
       <c r="C174" s="9" t="n"/>
       <c r="D174" s="9" t="n"/>
-      <c r="K174" s="10" t="n"/>
+      <c r="E174" s="9" t="n"/>
+      <c r="L174" s="10" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="9" t="n"/>
       <c r="B175" s="9" t="n"/>
       <c r="C175" s="9" t="n"/>
       <c r="D175" s="9" t="n"/>
-      <c r="K175" s="10" t="n"/>
+      <c r="E175" s="9" t="n"/>
+      <c r="L175" s="10" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="9" t="n"/>
       <c r="B176" s="9" t="n"/>
       <c r="C176" s="9" t="n"/>
       <c r="D176" s="9" t="n"/>
-      <c r="K176" s="10" t="n"/>
+      <c r="E176" s="9" t="n"/>
+      <c r="L176" s="10" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="9" t="n"/>
       <c r="B177" s="9" t="n"/>
       <c r="C177" s="9" t="n"/>
       <c r="D177" s="9" t="n"/>
-      <c r="K177" s="10" t="n"/>
+      <c r="E177" s="9" t="n"/>
+      <c r="L177" s="10" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="9" t="n"/>
       <c r="B178" s="9" t="n"/>
       <c r="C178" s="9" t="n"/>
       <c r="D178" s="9" t="n"/>
-      <c r="K178" s="10" t="n"/>
+      <c r="E178" s="9" t="n"/>
+      <c r="L178" s="10" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="9" t="n"/>
       <c r="B179" s="9" t="n"/>
       <c r="C179" s="9" t="n"/>
       <c r="D179" s="9" t="n"/>
-      <c r="K179" s="10" t="n"/>
+      <c r="E179" s="9" t="n"/>
+      <c r="L179" s="10" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="9" t="n"/>
       <c r="B180" s="9" t="n"/>
       <c r="C180" s="9" t="n"/>
       <c r="D180" s="9" t="n"/>
-      <c r="K180" s="10" t="n"/>
+      <c r="E180" s="9" t="n"/>
+      <c r="L180" s="10" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="9" t="n"/>
       <c r="B181" s="9" t="n"/>
       <c r="C181" s="9" t="n"/>
       <c r="D181" s="9" t="n"/>
-      <c r="K181" s="10" t="n"/>
+      <c r="E181" s="9" t="n"/>
+      <c r="L181" s="10" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="9" t="n"/>
       <c r="B182" s="9" t="n"/>
       <c r="C182" s="9" t="n"/>
       <c r="D182" s="9" t="n"/>
-      <c r="K182" s="10" t="n"/>
+      <c r="E182" s="9" t="n"/>
+      <c r="L182" s="10" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="9" t="n"/>
       <c r="B183" s="9" t="n"/>
       <c r="C183" s="9" t="n"/>
       <c r="D183" s="9" t="n"/>
-      <c r="K183" s="10" t="n"/>
+      <c r="E183" s="9" t="n"/>
+      <c r="L183" s="10" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="9" t="n"/>
       <c r="B184" s="9" t="n"/>
       <c r="C184" s="9" t="n"/>
       <c r="D184" s="9" t="n"/>
-      <c r="K184" s="10" t="n"/>
+      <c r="E184" s="9" t="n"/>
+      <c r="L184" s="10" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="9" t="n"/>
       <c r="B185" s="9" t="n"/>
       <c r="C185" s="9" t="n"/>
       <c r="D185" s="9" t="n"/>
-      <c r="K185" s="10" t="n"/>
+      <c r="E185" s="9" t="n"/>
+      <c r="L185" s="10" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="9" t="n"/>
       <c r="B186" s="9" t="n"/>
       <c r="C186" s="9" t="n"/>
       <c r="D186" s="9" t="n"/>
-      <c r="K186" s="10" t="n"/>
+      <c r="E186" s="9" t="n"/>
+      <c r="L186" s="10" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="9" t="n"/>
       <c r="B187" s="9" t="n"/>
       <c r="C187" s="9" t="n"/>
       <c r="D187" s="9" t="n"/>
-      <c r="K187" s="10" t="n"/>
+      <c r="E187" s="9" t="n"/>
+      <c r="L187" s="10" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="9" t="n"/>
       <c r="B188" s="9" t="n"/>
       <c r="C188" s="9" t="n"/>
       <c r="D188" s="9" t="n"/>
-      <c r="K188" s="10" t="n"/>
+      <c r="E188" s="9" t="n"/>
+      <c r="L188" s="10" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="9" t="n"/>
       <c r="B189" s="9" t="n"/>
       <c r="C189" s="9" t="n"/>
       <c r="D189" s="9" t="n"/>
-      <c r="K189" s="10" t="n"/>
+      <c r="E189" s="9" t="n"/>
+      <c r="L189" s="10" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="9" t="n"/>
       <c r="B190" s="9" t="n"/>
       <c r="C190" s="9" t="n"/>
       <c r="D190" s="9" t="n"/>
-      <c r="K190" s="10" t="n"/>
+      <c r="E190" s="9" t="n"/>
+      <c r="L190" s="10" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="9" t="n"/>
       <c r="B191" s="9" t="n"/>
       <c r="C191" s="9" t="n"/>
       <c r="D191" s="9" t="n"/>
-      <c r="K191" s="10" t="n"/>
+      <c r="E191" s="9" t="n"/>
+      <c r="L191" s="10" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="9" t="n"/>
       <c r="B192" s="9" t="n"/>
       <c r="C192" s="9" t="n"/>
       <c r="D192" s="9" t="n"/>
-      <c r="K192" s="10" t="n"/>
+      <c r="E192" s="9" t="n"/>
+      <c r="L192" s="10" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="9" t="n"/>
       <c r="B193" s="9" t="n"/>
       <c r="C193" s="9" t="n"/>
       <c r="D193" s="9" t="n"/>
-      <c r="K193" s="10" t="n"/>
+      <c r="E193" s="9" t="n"/>
+      <c r="L193" s="10" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="9" t="n"/>
       <c r="B194" s="9" t="n"/>
       <c r="C194" s="9" t="n"/>
       <c r="D194" s="9" t="n"/>
-      <c r="K194" s="10" t="n"/>
+      <c r="E194" s="9" t="n"/>
+      <c r="L194" s="10" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="9" t="n"/>
       <c r="B195" s="9" t="n"/>
       <c r="C195" s="9" t="n"/>
       <c r="D195" s="9" t="n"/>
-      <c r="K195" s="10" t="n"/>
+      <c r="E195" s="9" t="n"/>
+      <c r="L195" s="10" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="9" t="n"/>
       <c r="B196" s="9" t="n"/>
       <c r="C196" s="9" t="n"/>
       <c r="D196" s="9" t="n"/>
-      <c r="K196" s="10" t="n"/>
+      <c r="E196" s="9" t="n"/>
+      <c r="L196" s="10" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="9" t="n"/>
       <c r="B197" s="9" t="n"/>
       <c r="C197" s="9" t="n"/>
       <c r="D197" s="9" t="n"/>
-      <c r="K197" s="10" t="n"/>
+      <c r="E197" s="9" t="n"/>
+      <c r="L197" s="10" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="9" t="n"/>
       <c r="B198" s="9" t="n"/>
       <c r="C198" s="9" t="n"/>
       <c r="D198" s="9" t="n"/>
-      <c r="K198" s="10" t="n"/>
+      <c r="E198" s="9" t="n"/>
+      <c r="L198" s="10" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="9" t="n"/>
       <c r="B199" s="9" t="n"/>
       <c r="C199" s="9" t="n"/>
       <c r="D199" s="9" t="n"/>
-      <c r="K199" s="10" t="n"/>
+      <c r="E199" s="9" t="n"/>
+      <c r="L199" s="10" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="9" t="n"/>
       <c r="B200" s="9" t="n"/>
       <c r="C200" s="9" t="n"/>
       <c r="D200" s="9" t="n"/>
-      <c r="K200" s="10" t="n"/>
+      <c r="E200" s="9" t="n"/>
+      <c r="L200" s="10" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="9" t="n"/>
       <c r="B201" s="9" t="n"/>
       <c r="C201" s="9" t="n"/>
       <c r="D201" s="9" t="n"/>
-      <c r="K201" s="10" t="n"/>
+      <c r="E201" s="9" t="n"/>
+      <c r="L201" s="10" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="9" t="n"/>
       <c r="B202" s="9" t="n"/>
       <c r="C202" s="9" t="n"/>
       <c r="D202" s="9" t="n"/>
-      <c r="K202" s="10" t="n"/>
+      <c r="E202" s="9" t="n"/>
+      <c r="L202" s="10" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="9" t="n"/>
       <c r="B203" s="9" t="n"/>
       <c r="C203" s="9" t="n"/>
       <c r="D203" s="9" t="n"/>
-      <c r="K203" s="10" t="n"/>
+      <c r="E203" s="9" t="n"/>
+      <c r="L203" s="10" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="9" t="n"/>
       <c r="B204" s="9" t="n"/>
       <c r="C204" s="9" t="n"/>
       <c r="D204" s="9" t="n"/>
-      <c r="K204" s="10" t="n"/>
+      <c r="E204" s="9" t="n"/>
+      <c r="L204" s="10" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="9" t="n"/>
       <c r="B205" s="9" t="n"/>
       <c r="C205" s="9" t="n"/>
       <c r="D205" s="9" t="n"/>
-      <c r="K205" s="10" t="n"/>
+      <c r="E205" s="9" t="n"/>
+      <c r="L205" s="10" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="9" t="n"/>
       <c r="B206" s="9" t="n"/>
       <c r="C206" s="9" t="n"/>
       <c r="D206" s="9" t="n"/>
-      <c r="K206" s="10" t="n"/>
+      <c r="E206" s="9" t="n"/>
+      <c r="L206" s="10" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="9" t="n"/>
       <c r="B207" s="9" t="n"/>
       <c r="C207" s="9" t="n"/>
       <c r="D207" s="9" t="n"/>
-      <c r="K207" s="10" t="n"/>
+      <c r="E207" s="9" t="n"/>
+      <c r="L207" s="10" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="9" t="n"/>
       <c r="B208" s="9" t="n"/>
       <c r="C208" s="9" t="n"/>
       <c r="D208" s="9" t="n"/>
-      <c r="K208" s="10" t="n"/>
+      <c r="E208" s="9" t="n"/>
+      <c r="L208" s="10" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="9" t="n"/>
       <c r="B209" s="9" t="n"/>
       <c r="C209" s="9" t="n"/>
       <c r="D209" s="9" t="n"/>
-      <c r="K209" s="10" t="n"/>
+      <c r="E209" s="9" t="n"/>
+      <c r="L209" s="10" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="9" t="n"/>
       <c r="B210" s="9" t="n"/>
       <c r="C210" s="9" t="n"/>
       <c r="D210" s="9" t="n"/>
-      <c r="K210" s="10" t="n"/>
+      <c r="E210" s="9" t="n"/>
+      <c r="L210" s="10" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="9" t="n"/>
       <c r="B211" s="9" t="n"/>
       <c r="C211" s="9" t="n"/>
       <c r="D211" s="9" t="n"/>
-      <c r="K211" s="10" t="n"/>
+      <c r="E211" s="9" t="n"/>
+      <c r="L211" s="10" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="9" t="n"/>
       <c r="B212" s="9" t="n"/>
       <c r="C212" s="9" t="n"/>
       <c r="D212" s="9" t="n"/>
-      <c r="K212" s="10" t="n"/>
+      <c r="E212" s="9" t="n"/>
+      <c r="L212" s="10" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="9" t="n"/>
       <c r="B213" s="9" t="n"/>
       <c r="C213" s="9" t="n"/>
       <c r="D213" s="9" t="n"/>
-      <c r="K213" s="10" t="n"/>
+      <c r="E213" s="9" t="n"/>
+      <c r="L213" s="10" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="9" t="n"/>
       <c r="B214" s="9" t="n"/>
       <c r="C214" s="9" t="n"/>
       <c r="D214" s="9" t="n"/>
-      <c r="K214" s="10" t="n"/>
+      <c r="E214" s="9" t="n"/>
+      <c r="L214" s="10" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="9" t="n"/>
       <c r="B215" s="9" t="n"/>
       <c r="C215" s="9" t="n"/>
       <c r="D215" s="9" t="n"/>
-      <c r="K215" s="10" t="n"/>
+      <c r="E215" s="9" t="n"/>
+      <c r="L215" s="10" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="9" t="n"/>
       <c r="B216" s="9" t="n"/>
       <c r="C216" s="9" t="n"/>
       <c r="D216" s="9" t="n"/>
-      <c r="K216" s="10" t="n"/>
+      <c r="E216" s="9" t="n"/>
+      <c r="L216" s="10" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="9" t="n"/>
       <c r="B217" s="9" t="n"/>
       <c r="C217" s="9" t="n"/>
       <c r="D217" s="9" t="n"/>
-      <c r="K217" s="10" t="n"/>
+      <c r="E217" s="9" t="n"/>
+      <c r="L217" s="10" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="9" t="n"/>
       <c r="B218" s="9" t="n"/>
       <c r="C218" s="9" t="n"/>
       <c r="D218" s="9" t="n"/>
-      <c r="K218" s="10" t="n"/>
+      <c r="E218" s="9" t="n"/>
+      <c r="L218" s="10" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="9" t="n"/>
       <c r="B219" s="9" t="n"/>
       <c r="C219" s="9" t="n"/>
       <c r="D219" s="9" t="n"/>
-      <c r="K219" s="10" t="n"/>
+      <c r="E219" s="9" t="n"/>
+      <c r="L219" s="10" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="9" t="n"/>
       <c r="B220" s="9" t="n"/>
       <c r="C220" s="9" t="n"/>
       <c r="D220" s="9" t="n"/>
-      <c r="K220" s="10" t="n"/>
+      <c r="E220" s="9" t="n"/>
+      <c r="L220" s="10" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="9" t="n"/>
       <c r="B221" s="9" t="n"/>
       <c r="C221" s="9" t="n"/>
       <c r="D221" s="9" t="n"/>
-      <c r="K221" s="10" t="n"/>
+      <c r="E221" s="9" t="n"/>
+      <c r="L221" s="10" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="9" t="n"/>
       <c r="B222" s="9" t="n"/>
       <c r="C222" s="9" t="n"/>
       <c r="D222" s="9" t="n"/>
-      <c r="K222" s="10" t="n"/>
+      <c r="E222" s="9" t="n"/>
+      <c r="L222" s="10" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="9" t="n"/>
       <c r="B223" s="9" t="n"/>
       <c r="C223" s="9" t="n"/>
       <c r="D223" s="9" t="n"/>
-      <c r="K223" s="10" t="n"/>
+      <c r="E223" s="9" t="n"/>
+      <c r="L223" s="10" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="9" t="n"/>
       <c r="B224" s="9" t="n"/>
       <c r="C224" s="9" t="n"/>
       <c r="D224" s="9" t="n"/>
-      <c r="K224" s="10" t="n"/>
+      <c r="E224" s="9" t="n"/>
+      <c r="L224" s="10" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="9" t="n"/>
       <c r="B225" s="9" t="n"/>
       <c r="C225" s="9" t="n"/>
       <c r="D225" s="9" t="n"/>
-      <c r="K225" s="10" t="n"/>
+      <c r="E225" s="9" t="n"/>
+      <c r="L225" s="10" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="9" t="n"/>
       <c r="B226" s="9" t="n"/>
       <c r="C226" s="9" t="n"/>
       <c r="D226" s="9" t="n"/>
-      <c r="K226" s="10" t="n"/>
+      <c r="E226" s="9" t="n"/>
+      <c r="L226" s="10" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="9" t="n"/>
       <c r="B227" s="9" t="n"/>
       <c r="C227" s="9" t="n"/>
       <c r="D227" s="9" t="n"/>
-      <c r="K227" s="10" t="n"/>
+      <c r="E227" s="9" t="n"/>
+      <c r="L227" s="10" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="9" t="n"/>
       <c r="B228" s="9" t="n"/>
       <c r="C228" s="9" t="n"/>
       <c r="D228" s="9" t="n"/>
-      <c r="K228" s="10" t="n"/>
+      <c r="E228" s="9" t="n"/>
+      <c r="L228" s="10" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="9" t="n"/>
       <c r="B229" s="9" t="n"/>
       <c r="C229" s="9" t="n"/>
       <c r="D229" s="9" t="n"/>
-      <c r="K229" s="10" t="n"/>
+      <c r="E229" s="9" t="n"/>
+      <c r="L229" s="10" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="9" t="n"/>
       <c r="B230" s="9" t="n"/>
       <c r="C230" s="9" t="n"/>
       <c r="D230" s="9" t="n"/>
-      <c r="K230" s="10" t="n"/>
+      <c r="E230" s="9" t="n"/>
+      <c r="L230" s="10" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="9" t="n"/>
       <c r="B231" s="9" t="n"/>
       <c r="C231" s="9" t="n"/>
       <c r="D231" s="9" t="n"/>
-      <c r="K231" s="10" t="n"/>
+      <c r="E231" s="9" t="n"/>
+      <c r="L231" s="10" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="9" t="n"/>
       <c r="B232" s="9" t="n"/>
       <c r="C232" s="9" t="n"/>
       <c r="D232" s="9" t="n"/>
-      <c r="K232" s="10" t="n"/>
+      <c r="E232" s="9" t="n"/>
+      <c r="L232" s="10" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="9" t="n"/>
       <c r="B233" s="9" t="n"/>
       <c r="C233" s="9" t="n"/>
       <c r="D233" s="9" t="n"/>
-      <c r="K233" s="10" t="n"/>
+      <c r="E233" s="9" t="n"/>
+      <c r="L233" s="10" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="9" t="n"/>
       <c r="B234" s="9" t="n"/>
       <c r="C234" s="9" t="n"/>
       <c r="D234" s="9" t="n"/>
-      <c r="K234" s="10" t="n"/>
+      <c r="E234" s="9" t="n"/>
+      <c r="L234" s="10" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="9" t="n"/>
       <c r="B235" s="9" t="n"/>
       <c r="C235" s="9" t="n"/>
       <c r="D235" s="9" t="n"/>
-      <c r="K235" s="10" t="n"/>
+      <c r="E235" s="9" t="n"/>
+      <c r="L235" s="10" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="9" t="n"/>
       <c r="B236" s="9" t="n"/>
       <c r="C236" s="9" t="n"/>
       <c r="D236" s="9" t="n"/>
-      <c r="K236" s="10" t="n"/>
+      <c r="E236" s="9" t="n"/>
+      <c r="L236" s="10" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="9" t="n"/>
       <c r="B237" s="9" t="n"/>
       <c r="C237" s="9" t="n"/>
       <c r="D237" s="9" t="n"/>
-      <c r="K237" s="10" t="n"/>
+      <c r="E237" s="9" t="n"/>
+      <c r="L237" s="10" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="9" t="n"/>
       <c r="B238" s="9" t="n"/>
       <c r="C238" s="9" t="n"/>
       <c r="D238" s="9" t="n"/>
-      <c r="K238" s="10" t="n"/>
+      <c r="E238" s="9" t="n"/>
+      <c r="L238" s="10" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="9" t="n"/>
       <c r="B239" s="9" t="n"/>
       <c r="C239" s="9" t="n"/>
       <c r="D239" s="9" t="n"/>
-      <c r="K239" s="10" t="n"/>
+      <c r="E239" s="9" t="n"/>
+      <c r="L239" s="10" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="9" t="n"/>
       <c r="B240" s="9" t="n"/>
       <c r="C240" s="9" t="n"/>
       <c r="D240" s="9" t="n"/>
-      <c r="K240" s="10" t="n"/>
+      <c r="E240" s="9" t="n"/>
+      <c r="L240" s="10" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="9" t="n"/>
       <c r="B241" s="9" t="n"/>
       <c r="C241" s="9" t="n"/>
       <c r="D241" s="9" t="n"/>
-      <c r="K241" s="10" t="n"/>
+      <c r="E241" s="9" t="n"/>
+      <c r="L241" s="10" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="9" t="n"/>
       <c r="B242" s="9" t="n"/>
       <c r="C242" s="9" t="n"/>
       <c r="D242" s="9" t="n"/>
-      <c r="K242" s="10" t="n"/>
+      <c r="E242" s="9" t="n"/>
+      <c r="L242" s="10" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="9" t="n"/>
       <c r="B243" s="9" t="n"/>
       <c r="C243" s="9" t="n"/>
       <c r="D243" s="9" t="n"/>
-      <c r="K243" s="10" t="n"/>
+      <c r="E243" s="9" t="n"/>
+      <c r="L243" s="10" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="9" t="n"/>
       <c r="B244" s="9" t="n"/>
       <c r="C244" s="9" t="n"/>
       <c r="D244" s="9" t="n"/>
-      <c r="K244" s="10" t="n"/>
+      <c r="E244" s="9" t="n"/>
+      <c r="L244" s="10" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="9" t="n"/>
       <c r="B245" s="9" t="n"/>
       <c r="C245" s="9" t="n"/>
       <c r="D245" s="9" t="n"/>
-      <c r="K245" s="10" t="n"/>
+      <c r="E245" s="9" t="n"/>
+      <c r="L245" s="10" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="9" t="n"/>
       <c r="B246" s="9" t="n"/>
       <c r="C246" s="9" t="n"/>
       <c r="D246" s="9" t="n"/>
-      <c r="K246" s="10" t="n"/>
+      <c r="E246" s="9" t="n"/>
+      <c r="L246" s="10" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="9" t="n"/>
       <c r="B247" s="9" t="n"/>
       <c r="C247" s="9" t="n"/>
       <c r="D247" s="9" t="n"/>
-      <c r="K247" s="10" t="n"/>
+      <c r="E247" s="9" t="n"/>
+      <c r="L247" s="10" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="9" t="n"/>
       <c r="B248" s="9" t="n"/>
       <c r="C248" s="9" t="n"/>
       <c r="D248" s="9" t="n"/>
-      <c r="K248" s="10" t="n"/>
+      <c r="E248" s="9" t="n"/>
+      <c r="L248" s="10" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="9" t="n"/>
       <c r="B249" s="9" t="n"/>
       <c r="C249" s="9" t="n"/>
       <c r="D249" s="9" t="n"/>
-      <c r="K249" s="10" t="n"/>
+      <c r="E249" s="9" t="n"/>
+      <c r="L249" s="10" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="9" t="n"/>
       <c r="B250" s="9" t="n"/>
       <c r="C250" s="9" t="n"/>
       <c r="D250" s="9" t="n"/>
-      <c r="K250" s="10" t="n"/>
+      <c r="E250" s="9" t="n"/>
+      <c r="L250" s="10" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="9" t="n"/>
       <c r="B251" s="9" t="n"/>
       <c r="C251" s="9" t="n"/>
       <c r="D251" s="9" t="n"/>
-      <c r="K251" s="10" t="n"/>
+      <c r="E251" s="9" t="n"/>
+      <c r="L251" s="10" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="9" t="n"/>
       <c r="B252" s="9" t="n"/>
       <c r="C252" s="9" t="n"/>
       <c r="D252" s="9" t="n"/>
-      <c r="K252" s="10" t="n"/>
+      <c r="E252" s="9" t="n"/>
+      <c r="L252" s="10" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="9" t="n"/>
       <c r="B253" s="9" t="n"/>
       <c r="C253" s="9" t="n"/>
       <c r="D253" s="9" t="n"/>
-      <c r="K253" s="10" t="n"/>
+      <c r="E253" s="9" t="n"/>
+      <c r="L253" s="10" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="9" t="n"/>
       <c r="B254" s="9" t="n"/>
       <c r="C254" s="9" t="n"/>
       <c r="D254" s="9" t="n"/>
-      <c r="K254" s="10" t="n"/>
+      <c r="E254" s="9" t="n"/>
+      <c r="L254" s="10" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="9" t="n"/>
       <c r="B255" s="9" t="n"/>
       <c r="C255" s="9" t="n"/>
       <c r="D255" s="9" t="n"/>
-      <c r="K255" s="10" t="n"/>
+      <c r="E255" s="9" t="n"/>
+      <c r="L255" s="10" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="9" t="n"/>
       <c r="B256" s="9" t="n"/>
       <c r="C256" s="9" t="n"/>
       <c r="D256" s="9" t="n"/>
-      <c r="K256" s="10" t="n"/>
+      <c r="E256" s="9" t="n"/>
+      <c r="L256" s="10" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="9" t="n"/>
       <c r="B257" s="9" t="n"/>
       <c r="C257" s="9" t="n"/>
       <c r="D257" s="9" t="n"/>
-      <c r="K257" s="10" t="n"/>
+      <c r="E257" s="9" t="n"/>
+      <c r="L257" s="10" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="9" t="n"/>
       <c r="B258" s="9" t="n"/>
       <c r="C258" s="9" t="n"/>
       <c r="D258" s="9" t="n"/>
-      <c r="K258" s="10" t="n"/>
+      <c r="E258" s="9" t="n"/>
+      <c r="L258" s="10" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="9" t="n"/>
       <c r="B259" s="9" t="n"/>
       <c r="C259" s="9" t="n"/>
       <c r="D259" s="9" t="n"/>
-      <c r="K259" s="10" t="n"/>
+      <c r="E259" s="9" t="n"/>
+      <c r="L259" s="10" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="9" t="n"/>
       <c r="B260" s="9" t="n"/>
       <c r="C260" s="9" t="n"/>
       <c r="D260" s="9" t="n"/>
-      <c r="K260" s="10" t="n"/>
+      <c r="E260" s="9" t="n"/>
+      <c r="L260" s="10" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="9" t="n"/>
       <c r="B261" s="9" t="n"/>
       <c r="C261" s="9" t="n"/>
       <c r="D261" s="9" t="n"/>
-      <c r="K261" s="10" t="n"/>
+      <c r="E261" s="9" t="n"/>
+      <c r="L261" s="10" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="9" t="n"/>
       <c r="B262" s="9" t="n"/>
       <c r="C262" s="9" t="n"/>
       <c r="D262" s="9" t="n"/>
-      <c r="K262" s="10" t="n"/>
+      <c r="E262" s="9" t="n"/>
+      <c r="L262" s="10" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="9" t="n"/>
       <c r="B263" s="9" t="n"/>
       <c r="C263" s="9" t="n"/>
       <c r="D263" s="9" t="n"/>
-      <c r="K263" s="10" t="n"/>
+      <c r="E263" s="9" t="n"/>
+      <c r="L263" s="10" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="9" t="n"/>
       <c r="B264" s="9" t="n"/>
       <c r="C264" s="9" t="n"/>
       <c r="D264" s="9" t="n"/>
-      <c r="K264" s="10" t="n"/>
+      <c r="E264" s="9" t="n"/>
+      <c r="L264" s="10" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="9" t="n"/>
       <c r="B265" s="9" t="n"/>
       <c r="C265" s="9" t="n"/>
       <c r="D265" s="9" t="n"/>
-      <c r="K265" s="10" t="n"/>
+      <c r="E265" s="9" t="n"/>
+      <c r="L265" s="10" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="9" t="n"/>
       <c r="B266" s="9" t="n"/>
       <c r="C266" s="9" t="n"/>
       <c r="D266" s="9" t="n"/>
-      <c r="K266" s="10" t="n"/>
+      <c r="E266" s="9" t="n"/>
+      <c r="L266" s="10" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="9" t="n"/>
       <c r="B267" s="9" t="n"/>
       <c r="C267" s="9" t="n"/>
       <c r="D267" s="9" t="n"/>
-      <c r="K267" s="10" t="n"/>
+      <c r="E267" s="9" t="n"/>
+      <c r="L267" s="10" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="9" t="n"/>
       <c r="B268" s="9" t="n"/>
       <c r="C268" s="9" t="n"/>
       <c r="D268" s="9" t="n"/>
-      <c r="K268" s="10" t="n"/>
+      <c r="E268" s="9" t="n"/>
+      <c r="L268" s="10" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="9" t="n"/>
       <c r="B269" s="9" t="n"/>
       <c r="C269" s="9" t="n"/>
       <c r="D269" s="9" t="n"/>
-      <c r="K269" s="10" t="n"/>
+      <c r="E269" s="9" t="n"/>
+      <c r="L269" s="10" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="9" t="n"/>
       <c r="B270" s="9" t="n"/>
       <c r="C270" s="9" t="n"/>
       <c r="D270" s="9" t="n"/>
-      <c r="K270" s="10" t="n"/>
+      <c r="E270" s="9" t="n"/>
+      <c r="L270" s="10" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="9" t="n"/>
       <c r="B271" s="9" t="n"/>
       <c r="C271" s="9" t="n"/>
       <c r="D271" s="9" t="n"/>
-      <c r="K271" s="10" t="n"/>
+      <c r="E271" s="9" t="n"/>
+      <c r="L271" s="10" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="9" t="n"/>
       <c r="B272" s="9" t="n"/>
       <c r="C272" s="9" t="n"/>
       <c r="D272" s="9" t="n"/>
-      <c r="K272" s="10" t="n"/>
+      <c r="E272" s="9" t="n"/>
+      <c r="L272" s="10" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="9" t="n"/>
       <c r="B273" s="9" t="n"/>
       <c r="C273" s="9" t="n"/>
       <c r="D273" s="9" t="n"/>
-      <c r="K273" s="10" t="n"/>
+      <c r="E273" s="9" t="n"/>
+      <c r="L273" s="10" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="9" t="n"/>
       <c r="B274" s="9" t="n"/>
       <c r="C274" s="9" t="n"/>
       <c r="D274" s="9" t="n"/>
-      <c r="K274" s="10" t="n"/>
+      <c r="E274" s="9" t="n"/>
+      <c r="L274" s="10" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="9" t="n"/>
       <c r="B275" s="9" t="n"/>
       <c r="C275" s="9" t="n"/>
       <c r="D275" s="9" t="n"/>
-      <c r="K275" s="10" t="n"/>
+      <c r="E275" s="9" t="n"/>
+      <c r="L275" s="10" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="9" t="n"/>
       <c r="B276" s="9" t="n"/>
       <c r="C276" s="9" t="n"/>
       <c r="D276" s="9" t="n"/>
-      <c r="K276" s="10" t="n"/>
+      <c r="E276" s="9" t="n"/>
+      <c r="L276" s="10" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="9" t="n"/>
       <c r="B277" s="9" t="n"/>
       <c r="C277" s="9" t="n"/>
       <c r="D277" s="9" t="n"/>
-      <c r="K277" s="10" t="n"/>
+      <c r="E277" s="9" t="n"/>
+      <c r="L277" s="10" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="9" t="n"/>
       <c r="B278" s="9" t="n"/>
       <c r="C278" s="9" t="n"/>
       <c r="D278" s="9" t="n"/>
-      <c r="K278" s="10" t="n"/>
+      <c r="E278" s="9" t="n"/>
+      <c r="L278" s="10" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="9" t="n"/>
       <c r="B279" s="9" t="n"/>
       <c r="C279" s="9" t="n"/>
       <c r="D279" s="9" t="n"/>
-      <c r="K279" s="10" t="n"/>
+      <c r="E279" s="9" t="n"/>
+      <c r="L279" s="10" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="9" t="n"/>
       <c r="B280" s="9" t="n"/>
       <c r="C280" s="9" t="n"/>
       <c r="D280" s="9" t="n"/>
-      <c r="K280" s="10" t="n"/>
+      <c r="E280" s="9" t="n"/>
+      <c r="L280" s="10" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="9" t="n"/>
       <c r="B281" s="9" t="n"/>
       <c r="C281" s="9" t="n"/>
       <c r="D281" s="9" t="n"/>
-      <c r="K281" s="10" t="n"/>
+      <c r="E281" s="9" t="n"/>
+      <c r="L281" s="10" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="9" t="n"/>
       <c r="B282" s="9" t="n"/>
       <c r="C282" s="9" t="n"/>
       <c r="D282" s="9" t="n"/>
-      <c r="K282" s="10" t="n"/>
+      <c r="E282" s="9" t="n"/>
+      <c r="L282" s="10" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="9" t="n"/>
       <c r="B283" s="9" t="n"/>
       <c r="C283" s="9" t="n"/>
       <c r="D283" s="9" t="n"/>
-      <c r="K283" s="10" t="n"/>
+      <c r="E283" s="9" t="n"/>
+      <c r="L283" s="10" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="9" t="n"/>
       <c r="B284" s="9" t="n"/>
       <c r="C284" s="9" t="n"/>
       <c r="D284" s="9" t="n"/>
-      <c r="K284" s="10" t="n"/>
+      <c r="E284" s="9" t="n"/>
+      <c r="L284" s="10" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="9" t="n"/>
       <c r="B285" s="9" t="n"/>
       <c r="C285" s="9" t="n"/>
       <c r="D285" s="9" t="n"/>
-      <c r="K285" s="10" t="n"/>
+      <c r="E285" s="9" t="n"/>
+      <c r="L285" s="10" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="9" t="n"/>
       <c r="B286" s="9" t="n"/>
       <c r="C286" s="9" t="n"/>
       <c r="D286" s="9" t="n"/>
-      <c r="K286" s="10" t="n"/>
+      <c r="E286" s="9" t="n"/>
+      <c r="L286" s="10" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="9" t="n"/>
       <c r="B287" s="9" t="n"/>
       <c r="C287" s="9" t="n"/>
       <c r="D287" s="9" t="n"/>
-      <c r="K287" s="10" t="n"/>
+      <c r="E287" s="9" t="n"/>
+      <c r="L287" s="10" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="9" t="n"/>
       <c r="B288" s="9" t="n"/>
       <c r="C288" s="9" t="n"/>
       <c r="D288" s="9" t="n"/>
-      <c r="K288" s="10" t="n"/>
+      <c r="E288" s="9" t="n"/>
+      <c r="L288" s="10" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="9" t="n"/>
       <c r="B289" s="9" t="n"/>
       <c r="C289" s="9" t="n"/>
       <c r="D289" s="9" t="n"/>
-      <c r="K289" s="10" t="n"/>
+      <c r="E289" s="9" t="n"/>
+      <c r="L289" s="10" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="9" t="n"/>
       <c r="B290" s="9" t="n"/>
       <c r="C290" s="9" t="n"/>
       <c r="D290" s="9" t="n"/>
-      <c r="K290" s="10" t="n"/>
+      <c r="E290" s="9" t="n"/>
+      <c r="L290" s="10" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="9" t="n"/>
       <c r="B291" s="9" t="n"/>
       <c r="C291" s="9" t="n"/>
       <c r="D291" s="9" t="n"/>
-      <c r="K291" s="10" t="n"/>
+      <c r="E291" s="9" t="n"/>
+      <c r="L291" s="10" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="9" t="n"/>
       <c r="B292" s="9" t="n"/>
       <c r="C292" s="9" t="n"/>
       <c r="D292" s="9" t="n"/>
-      <c r="K292" s="10" t="n"/>
+      <c r="E292" s="9" t="n"/>
+      <c r="L292" s="10" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="9" t="n"/>
       <c r="B293" s="9" t="n"/>
       <c r="C293" s="9" t="n"/>
       <c r="D293" s="9" t="n"/>
-      <c r="K293" s="10" t="n"/>
+      <c r="E293" s="9" t="n"/>
+      <c r="L293" s="10" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="9" t="n"/>
       <c r="B294" s="9" t="n"/>
       <c r="C294" s="9" t="n"/>
       <c r="D294" s="9" t="n"/>
-      <c r="K294" s="10" t="n"/>
+      <c r="E294" s="9" t="n"/>
+      <c r="L294" s="10" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="9" t="n"/>
       <c r="B295" s="9" t="n"/>
       <c r="C295" s="9" t="n"/>
       <c r="D295" s="9" t="n"/>
-      <c r="K295" s="10" t="n"/>
+      <c r="E295" s="9" t="n"/>
+      <c r="L295" s="10" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="9" t="n"/>
       <c r="B296" s="9" t="n"/>
       <c r="C296" s="9" t="n"/>
       <c r="D296" s="9" t="n"/>
-      <c r="K296" s="10" t="n"/>
+      <c r="E296" s="9" t="n"/>
+      <c r="L296" s="10" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="9" t="n"/>
       <c r="B297" s="9" t="n"/>
       <c r="C297" s="9" t="n"/>
       <c r="D297" s="9" t="n"/>
-      <c r="K297" s="10" t="n"/>
+      <c r="E297" s="9" t="n"/>
+      <c r="L297" s="10" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="9" t="n"/>
       <c r="B298" s="9" t="n"/>
       <c r="C298" s="9" t="n"/>
       <c r="D298" s="9" t="n"/>
-      <c r="K298" s="10" t="n"/>
+      <c r="E298" s="9" t="n"/>
+      <c r="L298" s="10" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="9" t="n"/>
       <c r="B299" s="9" t="n"/>
       <c r="C299" s="9" t="n"/>
       <c r="D299" s="9" t="n"/>
-      <c r="K299" s="10" t="n"/>
+      <c r="E299" s="9" t="n"/>
+      <c r="L299" s="10" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="9" t="n"/>
       <c r="B300" s="9" t="n"/>
       <c r="C300" s="9" t="n"/>
       <c r="D300" s="9" t="n"/>
-      <c r="K300" s="10" t="n"/>
+      <c r="E300" s="9" t="n"/>
+      <c r="L300" s="10" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="9" t="n"/>
       <c r="B301" s="9" t="n"/>
       <c r="C301" s="9" t="n"/>
       <c r="D301" s="9" t="n"/>
-      <c r="K301" s="10" t="n"/>
+      <c r="E301" s="9" t="n"/>
+      <c r="L301" s="10" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="9" t="n"/>
       <c r="B302" s="9" t="n"/>
       <c r="C302" s="9" t="n"/>
       <c r="D302" s="9" t="n"/>
-      <c r="K302" s="10" t="n"/>
+      <c r="E302" s="9" t="n"/>
+      <c r="L302" s="10" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="9" t="n"/>
       <c r="B303" s="9" t="n"/>
       <c r="C303" s="9" t="n"/>
       <c r="D303" s="9" t="n"/>
-      <c r="K303" s="10" t="n"/>
+      <c r="E303" s="9" t="n"/>
+      <c r="L303" s="10" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="9" t="n"/>
       <c r="B304" s="9" t="n"/>
       <c r="C304" s="9" t="n"/>
       <c r="D304" s="9" t="n"/>
-      <c r="K304" s="10" t="n"/>
+      <c r="E304" s="9" t="n"/>
+      <c r="L304" s="10" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="9" t="n"/>
       <c r="B305" s="9" t="n"/>
       <c r="C305" s="9" t="n"/>
       <c r="D305" s="9" t="n"/>
-      <c r="K305" s="10" t="n"/>
+      <c r="E305" s="9" t="n"/>
+      <c r="L305" s="10" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="9" t="n"/>
       <c r="B306" s="9" t="n"/>
       <c r="C306" s="9" t="n"/>
       <c r="D306" s="9" t="n"/>
-      <c r="K306" s="10" t="n"/>
+      <c r="E306" s="9" t="n"/>
+      <c r="L306" s="10" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="9" t="n"/>
       <c r="B307" s="9" t="n"/>
       <c r="C307" s="9" t="n"/>
       <c r="D307" s="9" t="n"/>
-      <c r="K307" s="10" t="n"/>
+      <c r="E307" s="9" t="n"/>
+      <c r="L307" s="10" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="9" t="n"/>
       <c r="B308" s="9" t="n"/>
       <c r="C308" s="9" t="n"/>
       <c r="D308" s="9" t="n"/>
-      <c r="K308" s="10" t="n"/>
+      <c r="E308" s="9" t="n"/>
+      <c r="L308" s="10" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="9" t="n"/>
       <c r="B309" s="9" t="n"/>
       <c r="C309" s="9" t="n"/>
       <c r="D309" s="9" t="n"/>
-      <c r="K309" s="10" t="n"/>
+      <c r="E309" s="9" t="n"/>
+      <c r="L309" s="10" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="9" t="n"/>
       <c r="B310" s="9" t="n"/>
       <c r="C310" s="9" t="n"/>
       <c r="D310" s="9" t="n"/>
-      <c r="K310" s="10" t="n"/>
+      <c r="E310" s="9" t="n"/>
+      <c r="L310" s="10" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="9" t="n"/>
       <c r="B311" s="9" t="n"/>
       <c r="C311" s="9" t="n"/>
       <c r="D311" s="9" t="n"/>
-      <c r="K311" s="10" t="n"/>
+      <c r="E311" s="9" t="n"/>
+      <c r="L311" s="10" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="9" t="n"/>
       <c r="B312" s="9" t="n"/>
       <c r="C312" s="9" t="n"/>
       <c r="D312" s="9" t="n"/>
-      <c r="K312" s="10" t="n"/>
+      <c r="E312" s="9" t="n"/>
+      <c r="L312" s="10" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="9" t="n"/>
       <c r="B313" s="9" t="n"/>
       <c r="C313" s="9" t="n"/>
       <c r="D313" s="9" t="n"/>
-      <c r="K313" s="10" t="n"/>
+      <c r="E313" s="9" t="n"/>
+      <c r="L313" s="10" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="9" t="n"/>
       <c r="B314" s="9" t="n"/>
       <c r="C314" s="9" t="n"/>
       <c r="D314" s="9" t="n"/>
-      <c r="K314" s="10" t="n"/>
+      <c r="E314" s="9" t="n"/>
+      <c r="L314" s="10" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="9" t="n"/>
       <c r="B315" s="9" t="n"/>
       <c r="C315" s="9" t="n"/>
       <c r="D315" s="9" t="n"/>
-      <c r="K315" s="10" t="n"/>
+      <c r="E315" s="9" t="n"/>
+      <c r="L315" s="10" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="9" t="n"/>
       <c r="B316" s="9" t="n"/>
       <c r="C316" s="9" t="n"/>
       <c r="D316" s="9" t="n"/>
-      <c r="K316" s="10" t="n"/>
+      <c r="E316" s="9" t="n"/>
+      <c r="L316" s="10" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="9" t="n"/>
       <c r="B317" s="9" t="n"/>
       <c r="C317" s="9" t="n"/>
       <c r="D317" s="9" t="n"/>
-      <c r="K317" s="10" t="n"/>
+      <c r="E317" s="9" t="n"/>
+      <c r="L317" s="10" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="9" t="n"/>
       <c r="B318" s="9" t="n"/>
       <c r="C318" s="9" t="n"/>
       <c r="D318" s="9" t="n"/>
-      <c r="K318" s="10" t="n"/>
+      <c r="E318" s="9" t="n"/>
+      <c r="L318" s="10" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="9" t="n"/>
       <c r="B319" s="9" t="n"/>
       <c r="C319" s="9" t="n"/>
       <c r="D319" s="9" t="n"/>
-      <c r="K319" s="10" t="n"/>
+      <c r="E319" s="9" t="n"/>
+      <c r="L319" s="10" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="9" t="n"/>
       <c r="B320" s="9" t="n"/>
       <c r="C320" s="9" t="n"/>
       <c r="D320" s="9" t="n"/>
-      <c r="K320" s="10" t="n"/>
+      <c r="E320" s="9" t="n"/>
+      <c r="L320" s="10" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="9" t="n"/>
       <c r="B321" s="9" t="n"/>
       <c r="C321" s="9" t="n"/>
       <c r="D321" s="9" t="n"/>
-      <c r="K321" s="10" t="n"/>
+      <c r="E321" s="9" t="n"/>
+      <c r="L321" s="10" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="9" t="n"/>
       <c r="B322" s="9" t="n"/>
       <c r="C322" s="9" t="n"/>
       <c r="D322" s="9" t="n"/>
-      <c r="K322" s="10" t="n"/>
+      <c r="E322" s="9" t="n"/>
+      <c r="L322" s="10" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="9" t="n"/>
       <c r="B323" s="9" t="n"/>
       <c r="C323" s="9" t="n"/>
       <c r="D323" s="9" t="n"/>
-      <c r="K323" s="10" t="n"/>
+      <c r="E323" s="9" t="n"/>
+      <c r="L323" s="10" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="9" t="n"/>
       <c r="B324" s="9" t="n"/>
       <c r="C324" s="9" t="n"/>
       <c r="D324" s="9" t="n"/>
-      <c r="K324" s="10" t="n"/>
+      <c r="E324" s="9" t="n"/>
+      <c r="L324" s="10" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="9" t="n"/>
       <c r="B325" s="9" t="n"/>
       <c r="C325" s="9" t="n"/>
       <c r="D325" s="9" t="n"/>
-      <c r="K325" s="10" t="n"/>
+      <c r="E325" s="9" t="n"/>
+      <c r="L325" s="10" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="9" t="n"/>
       <c r="B326" s="9" t="n"/>
       <c r="C326" s="9" t="n"/>
       <c r="D326" s="9" t="n"/>
-      <c r="K326" s="10" t="n"/>
+      <c r="E326" s="9" t="n"/>
+      <c r="L326" s="10" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="9" t="n"/>
       <c r="B327" s="9" t="n"/>
       <c r="C327" s="9" t="n"/>
       <c r="D327" s="9" t="n"/>
-      <c r="K327" s="10" t="n"/>
+      <c r="E327" s="9" t="n"/>
+      <c r="L327" s="10" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="9" t="n"/>
       <c r="B328" s="9" t="n"/>
       <c r="C328" s="9" t="n"/>
       <c r="D328" s="9" t="n"/>
-      <c r="K328" s="10" t="n"/>
+      <c r="E328" s="9" t="n"/>
+      <c r="L328" s="10" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="9" t="n"/>
       <c r="B329" s="9" t="n"/>
       <c r="C329" s="9" t="n"/>
       <c r="D329" s="9" t="n"/>
-      <c r="K329" s="10" t="n"/>
+      <c r="E329" s="9" t="n"/>
+      <c r="L329" s="10" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="9" t="n"/>
       <c r="B330" s="9" t="n"/>
       <c r="C330" s="9" t="n"/>
       <c r="D330" s="9" t="n"/>
-      <c r="K330" s="10" t="n"/>
+      <c r="E330" s="9" t="n"/>
+      <c r="L330" s="10" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="9" t="n"/>
       <c r="B331" s="9" t="n"/>
       <c r="C331" s="9" t="n"/>
       <c r="D331" s="9" t="n"/>
-      <c r="K331" s="10" t="n"/>
+      <c r="E331" s="9" t="n"/>
+      <c r="L331" s="10" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="9" t="n"/>
       <c r="B332" s="9" t="n"/>
       <c r="C332" s="9" t="n"/>
       <c r="D332" s="9" t="n"/>
-      <c r="K332" s="10" t="n"/>
+      <c r="E332" s="9" t="n"/>
+      <c r="L332" s="10" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="9" t="n"/>
       <c r="B333" s="9" t="n"/>
       <c r="C333" s="9" t="n"/>
       <c r="D333" s="9" t="n"/>
-      <c r="K333" s="10" t="n"/>
+      <c r="E333" s="9" t="n"/>
+      <c r="L333" s="10" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="9" t="n"/>
       <c r="B334" s="9" t="n"/>
       <c r="C334" s="9" t="n"/>
       <c r="D334" s="9" t="n"/>
-      <c r="K334" s="10" t="n"/>
+      <c r="E334" s="9" t="n"/>
+      <c r="L334" s="10" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="9" t="n"/>
       <c r="B335" s="9" t="n"/>
       <c r="C335" s="9" t="n"/>
       <c r="D335" s="9" t="n"/>
-      <c r="K335" s="10" t="n"/>
+      <c r="E335" s="9" t="n"/>
+      <c r="L335" s="10" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="9" t="n"/>
       <c r="B336" s="9" t="n"/>
       <c r="C336" s="9" t="n"/>
       <c r="D336" s="9" t="n"/>
-      <c r="K336" s="10" t="n"/>
+      <c r="E336" s="9" t="n"/>
+      <c r="L336" s="10" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="9" t="n"/>
       <c r="B337" s="9" t="n"/>
       <c r="C337" s="9" t="n"/>
       <c r="D337" s="9" t="n"/>
-      <c r="K337" s="10" t="n"/>
+      <c r="E337" s="9" t="n"/>
+      <c r="L337" s="10" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="9" t="n"/>
       <c r="B338" s="9" t="n"/>
       <c r="C338" s="9" t="n"/>
       <c r="D338" s="9" t="n"/>
-      <c r="K338" s="10" t="n"/>
+      <c r="E338" s="9" t="n"/>
+      <c r="L338" s="10" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="9" t="n"/>
       <c r="B339" s="9" t="n"/>
       <c r="C339" s="9" t="n"/>
       <c r="D339" s="9" t="n"/>
-      <c r="K339" s="10" t="n"/>
+      <c r="E339" s="9" t="n"/>
+      <c r="L339" s="10" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="9" t="n"/>
       <c r="B340" s="9" t="n"/>
       <c r="C340" s="9" t="n"/>
       <c r="D340" s="9" t="n"/>
-      <c r="K340" s="10" t="n"/>
+      <c r="E340" s="9" t="n"/>
+      <c r="L340" s="10" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="9" t="n"/>
       <c r="B341" s="9" t="n"/>
       <c r="C341" s="9" t="n"/>
       <c r="D341" s="9" t="n"/>
-      <c r="K341" s="10" t="n"/>
+      <c r="E341" s="9" t="n"/>
+      <c r="L341" s="10" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="9" t="n"/>
       <c r="B342" s="9" t="n"/>
       <c r="C342" s="9" t="n"/>
       <c r="D342" s="9" t="n"/>
-      <c r="K342" s="10" t="n"/>
+      <c r="E342" s="9" t="n"/>
+      <c r="L342" s="10" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="9" t="n"/>
       <c r="B343" s="9" t="n"/>
       <c r="C343" s="9" t="n"/>
       <c r="D343" s="9" t="n"/>
-      <c r="K343" s="10" t="n"/>
+      <c r="E343" s="9" t="n"/>
+      <c r="L343" s="10" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="9" t="n"/>
       <c r="B344" s="9" t="n"/>
       <c r="C344" s="9" t="n"/>
       <c r="D344" s="9" t="n"/>
-      <c r="K344" s="10" t="n"/>
+      <c r="E344" s="9" t="n"/>
+      <c r="L344" s="10" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="9" t="n"/>
       <c r="B345" s="9" t="n"/>
       <c r="C345" s="9" t="n"/>
       <c r="D345" s="9" t="n"/>
-      <c r="K345" s="10" t="n"/>
+      <c r="E345" s="9" t="n"/>
+      <c r="L345" s="10" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="9" t="n"/>
       <c r="B346" s="9" t="n"/>
       <c r="C346" s="9" t="n"/>
       <c r="D346" s="9" t="n"/>
-      <c r="K346" s="10" t="n"/>
+      <c r="E346" s="9" t="n"/>
+      <c r="L346" s="10" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="9" t="n"/>
       <c r="B347" s="9" t="n"/>
       <c r="C347" s="9" t="n"/>
       <c r="D347" s="9" t="n"/>
-      <c r="K347" s="10" t="n"/>
+      <c r="E347" s="9" t="n"/>
+      <c r="L347" s="10" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="9" t="n"/>
       <c r="B348" s="9" t="n"/>
       <c r="C348" s="9" t="n"/>
       <c r="D348" s="9" t="n"/>
-      <c r="K348" s="10" t="n"/>
+      <c r="E348" s="9" t="n"/>
+      <c r="L348" s="10" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="9" t="n"/>
       <c r="B349" s="9" t="n"/>
       <c r="C349" s="9" t="n"/>
       <c r="D349" s="9" t="n"/>
-      <c r="K349" s="10" t="n"/>
+      <c r="E349" s="9" t="n"/>
+      <c r="L349" s="10" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="9" t="n"/>
       <c r="B350" s="9" t="n"/>
       <c r="C350" s="9" t="n"/>
       <c r="D350" s="9" t="n"/>
-      <c r="K350" s="10" t="n"/>
+      <c r="E350" s="9" t="n"/>
+      <c r="L350" s="10" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="9" t="n"/>
       <c r="B351" s="9" t="n"/>
       <c r="C351" s="9" t="n"/>
       <c r="D351" s="9" t="n"/>
-      <c r="K351" s="10" t="n"/>
+      <c r="E351" s="9" t="n"/>
+      <c r="L351" s="10" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="9" t="n"/>
       <c r="B352" s="9" t="n"/>
       <c r="C352" s="9" t="n"/>
       <c r="D352" s="9" t="n"/>
-      <c r="K352" s="10" t="n"/>
+      <c r="E352" s="9" t="n"/>
+      <c r="L352" s="10" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="9" t="n"/>
       <c r="B353" s="9" t="n"/>
       <c r="C353" s="9" t="n"/>
       <c r="D353" s="9" t="n"/>
-      <c r="K353" s="10" t="n"/>
+      <c r="E353" s="9" t="n"/>
+      <c r="L353" s="10" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="9" t="n"/>
       <c r="B354" s="9" t="n"/>
       <c r="C354" s="9" t="n"/>
       <c r="D354" s="9" t="n"/>
-      <c r="K354" s="10" t="n"/>
+      <c r="E354" s="9" t="n"/>
+      <c r="L354" s="10" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="9" t="n"/>
       <c r="B355" s="9" t="n"/>
       <c r="C355" s="9" t="n"/>
       <c r="D355" s="9" t="n"/>
-      <c r="K355" s="10" t="n"/>
+      <c r="E355" s="9" t="n"/>
+      <c r="L355" s="10" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="9" t="n"/>
       <c r="B356" s="9" t="n"/>
       <c r="C356" s="9" t="n"/>
       <c r="D356" s="9" t="n"/>
-      <c r="K356" s="10" t="n"/>
+      <c r="E356" s="9" t="n"/>
+      <c r="L356" s="10" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="9" t="n"/>
       <c r="B357" s="9" t="n"/>
       <c r="C357" s="9" t="n"/>
       <c r="D357" s="9" t="n"/>
-      <c r="K357" s="10" t="n"/>
+      <c r="E357" s="9" t="n"/>
+      <c r="L357" s="10" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="9" t="n"/>
       <c r="B358" s="9" t="n"/>
       <c r="C358" s="9" t="n"/>
       <c r="D358" s="9" t="n"/>
-      <c r="K358" s="10" t="n"/>
+      <c r="E358" s="9" t="n"/>
+      <c r="L358" s="10" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="9" t="n"/>
       <c r="B359" s="9" t="n"/>
       <c r="C359" s="9" t="n"/>
       <c r="D359" s="9" t="n"/>
-      <c r="K359" s="10" t="n"/>
+      <c r="E359" s="9" t="n"/>
+      <c r="L359" s="10" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="9" t="n"/>
       <c r="B360" s="9" t="n"/>
       <c r="C360" s="9" t="n"/>
       <c r="D360" s="9" t="n"/>
-      <c r="K360" s="10" t="n"/>
+      <c r="E360" s="9" t="n"/>
+      <c r="L360" s="10" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="9" t="n"/>
       <c r="B361" s="9" t="n"/>
       <c r="C361" s="9" t="n"/>
       <c r="D361" s="9" t="n"/>
-      <c r="K361" s="10" t="n"/>
+      <c r="E361" s="9" t="n"/>
+      <c r="L361" s="10" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="9" t="n"/>
       <c r="B362" s="9" t="n"/>
       <c r="C362" s="9" t="n"/>
       <c r="D362" s="9" t="n"/>
-      <c r="K362" s="10" t="n"/>
+      <c r="E362" s="9" t="n"/>
+      <c r="L362" s="10" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="9" t="n"/>
       <c r="B363" s="9" t="n"/>
       <c r="C363" s="9" t="n"/>
       <c r="D363" s="9" t="n"/>
-      <c r="K363" s="10" t="n"/>
+      <c r="E363" s="9" t="n"/>
+      <c r="L363" s="10" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="9" t="n"/>
       <c r="B364" s="9" t="n"/>
       <c r="C364" s="9" t="n"/>
       <c r="D364" s="9" t="n"/>
-      <c r="K364" s="10" t="n"/>
+      <c r="E364" s="9" t="n"/>
+      <c r="L364" s="10" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="9" t="n"/>
       <c r="B365" s="9" t="n"/>
       <c r="C365" s="9" t="n"/>
       <c r="D365" s="9" t="n"/>
-      <c r="K365" s="10" t="n"/>
+      <c r="E365" s="9" t="n"/>
+      <c r="L365" s="10" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="9" t="n"/>
       <c r="B366" s="9" t="n"/>
       <c r="C366" s="9" t="n"/>
       <c r="D366" s="9" t="n"/>
-      <c r="K366" s="10" t="n"/>
+      <c r="E366" s="9" t="n"/>
+      <c r="L366" s="10" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="9" t="n"/>
       <c r="B367" s="9" t="n"/>
       <c r="C367" s="9" t="n"/>
       <c r="D367" s="9" t="n"/>
-      <c r="K367" s="10" t="n"/>
+      <c r="E367" s="9" t="n"/>
+      <c r="L367" s="10" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="9" t="n"/>
       <c r="B368" s="9" t="n"/>
       <c r="C368" s="9" t="n"/>
       <c r="D368" s="9" t="n"/>
-      <c r="K368" s="10" t="n"/>
+      <c r="E368" s="9" t="n"/>
+      <c r="L368" s="10" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="9" t="n"/>
       <c r="B369" s="9" t="n"/>
       <c r="C369" s="9" t="n"/>
       <c r="D369" s="9" t="n"/>
-      <c r="K369" s="10" t="n"/>
+      <c r="E369" s="9" t="n"/>
+      <c r="L369" s="10" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="9" t="n"/>
       <c r="B370" s="9" t="n"/>
       <c r="C370" s="9" t="n"/>
       <c r="D370" s="9" t="n"/>
-      <c r="K370" s="10" t="n"/>
+      <c r="E370" s="9" t="n"/>
+      <c r="L370" s="10" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="9" t="n"/>
       <c r="B371" s="9" t="n"/>
       <c r="C371" s="9" t="n"/>
       <c r="D371" s="9" t="n"/>
-      <c r="K371" s="10" t="n"/>
+      <c r="E371" s="9" t="n"/>
+      <c r="L371" s="10" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="9" t="n"/>
       <c r="B372" s="9" t="n"/>
       <c r="C372" s="9" t="n"/>
       <c r="D372" s="9" t="n"/>
-      <c r="K372" s="10" t="n"/>
+      <c r="E372" s="9" t="n"/>
+      <c r="L372" s="10" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="9" t="n"/>
       <c r="B373" s="9" t="n"/>
       <c r="C373" s="9" t="n"/>
       <c r="D373" s="9" t="n"/>
-      <c r="K373" s="10" t="n"/>
+      <c r="E373" s="9" t="n"/>
+      <c r="L373" s="10" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="9" t="n"/>
       <c r="B374" s="9" t="n"/>
       <c r="C374" s="9" t="n"/>
       <c r="D374" s="9" t="n"/>
-      <c r="K374" s="10" t="n"/>
+      <c r="E374" s="9" t="n"/>
+      <c r="L374" s="10" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="9" t="n"/>
       <c r="B375" s="9" t="n"/>
       <c r="C375" s="9" t="n"/>
       <c r="D375" s="9" t="n"/>
-      <c r="K375" s="10" t="n"/>
+      <c r="E375" s="9" t="n"/>
+      <c r="L375" s="10" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="9" t="n"/>
       <c r="B376" s="9" t="n"/>
       <c r="C376" s="9" t="n"/>
       <c r="D376" s="9" t="n"/>
-      <c r="K376" s="10" t="n"/>
+      <c r="E376" s="9" t="n"/>
+      <c r="L376" s="10" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="9" t="n"/>
       <c r="B377" s="9" t="n"/>
       <c r="C377" s="9" t="n"/>
       <c r="D377" s="9" t="n"/>
-      <c r="K377" s="10" t="n"/>
+      <c r="E377" s="9" t="n"/>
+      <c r="L377" s="10" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="9" t="n"/>
       <c r="B378" s="9" t="n"/>
       <c r="C378" s="9" t="n"/>
       <c r="D378" s="9" t="n"/>
-      <c r="K378" s="10" t="n"/>
+      <c r="E378" s="9" t="n"/>
+      <c r="L378" s="10" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="9" t="n"/>
       <c r="B379" s="9" t="n"/>
       <c r="C379" s="9" t="n"/>
       <c r="D379" s="9" t="n"/>
-      <c r="K379" s="10" t="n"/>
+      <c r="E379" s="9" t="n"/>
+      <c r="L379" s="10" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="9" t="n"/>
       <c r="B380" s="9" t="n"/>
       <c r="C380" s="9" t="n"/>
       <c r="D380" s="9" t="n"/>
-      <c r="K380" s="10" t="n"/>
+      <c r="E380" s="9" t="n"/>
+      <c r="L380" s="10" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="9" t="n"/>
       <c r="B381" s="9" t="n"/>
       <c r="C381" s="9" t="n"/>
       <c r="D381" s="9" t="n"/>
-      <c r="K381" s="10" t="n"/>
+      <c r="E381" s="9" t="n"/>
+      <c r="L381" s="10" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="9" t="n"/>
       <c r="B382" s="9" t="n"/>
       <c r="C382" s="9" t="n"/>
       <c r="D382" s="9" t="n"/>
-      <c r="K382" s="10" t="n"/>
+      <c r="E382" s="9" t="n"/>
+      <c r="L382" s="10" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="9" t="n"/>
       <c r="B383" s="9" t="n"/>
       <c r="C383" s="9" t="n"/>
       <c r="D383" s="9" t="n"/>
-      <c r="K383" s="10" t="n"/>
+      <c r="E383" s="9" t="n"/>
+      <c r="L383" s="10" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="9" t="n"/>
       <c r="B384" s="9" t="n"/>
       <c r="C384" s="9" t="n"/>
       <c r="D384" s="9" t="n"/>
-      <c r="K384" s="10" t="n"/>
+      <c r="E384" s="9" t="n"/>
+      <c r="L384" s="10" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="9" t="n"/>
       <c r="B385" s="9" t="n"/>
       <c r="C385" s="9" t="n"/>
       <c r="D385" s="9" t="n"/>
-      <c r="K385" s="10" t="n"/>
+      <c r="E385" s="9" t="n"/>
+      <c r="L385" s="10" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="9" t="n"/>
       <c r="B386" s="9" t="n"/>
       <c r="C386" s="9" t="n"/>
       <c r="D386" s="9" t="n"/>
-      <c r="K386" s="10" t="n"/>
+      <c r="E386" s="9" t="n"/>
+      <c r="L386" s="10" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="9" t="n"/>
       <c r="B387" s="9" t="n"/>
       <c r="C387" s="9" t="n"/>
       <c r="D387" s="9" t="n"/>
-      <c r="K387" s="10" t="n"/>
+      <c r="E387" s="9" t="n"/>
+      <c r="L387" s="10" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="9" t="n"/>
       <c r="B388" s="9" t="n"/>
       <c r="C388" s="9" t="n"/>
       <c r="D388" s="9" t="n"/>
-      <c r="K388" s="10" t="n"/>
+      <c r="E388" s="9" t="n"/>
+      <c r="L388" s="10" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="9" t="n"/>
       <c r="B389" s="9" t="n"/>
       <c r="C389" s="9" t="n"/>
       <c r="D389" s="9" t="n"/>
-      <c r="K389" s="10" t="n"/>
+      <c r="E389" s="9" t="n"/>
+      <c r="L389" s="10" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="9" t="n"/>
       <c r="B390" s="9" t="n"/>
       <c r="C390" s="9" t="n"/>
       <c r="D390" s="9" t="n"/>
-      <c r="K390" s="10" t="n"/>
+      <c r="E390" s="9" t="n"/>
+      <c r="L390" s="10" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="9" t="n"/>
       <c r="B391" s="9" t="n"/>
       <c r="C391" s="9" t="n"/>
       <c r="D391" s="9" t="n"/>
-      <c r="K391" s="10" t="n"/>
+      <c r="E391" s="9" t="n"/>
+      <c r="L391" s="10" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="9" t="n"/>
       <c r="B392" s="9" t="n"/>
       <c r="C392" s="9" t="n"/>
       <c r="D392" s="9" t="n"/>
-      <c r="K392" s="10" t="n"/>
+      <c r="E392" s="9" t="n"/>
+      <c r="L392" s="10" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="9" t="n"/>
       <c r="B393" s="9" t="n"/>
       <c r="C393" s="9" t="n"/>
       <c r="D393" s="9" t="n"/>
-      <c r="K393" s="10" t="n"/>
+      <c r="E393" s="9" t="n"/>
+      <c r="L393" s="10" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="9" t="n"/>
       <c r="B394" s="9" t="n"/>
       <c r="C394" s="9" t="n"/>
       <c r="D394" s="9" t="n"/>
-      <c r="K394" s="10" t="n"/>
+      <c r="E394" s="9" t="n"/>
+      <c r="L394" s="10" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="9" t="n"/>
       <c r="B395" s="9" t="n"/>
       <c r="C395" s="9" t="n"/>
       <c r="D395" s="9" t="n"/>
-      <c r="K395" s="10" t="n"/>
+      <c r="E395" s="9" t="n"/>
+      <c r="L395" s="10" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="9" t="n"/>
       <c r="B396" s="9" t="n"/>
       <c r="C396" s="9" t="n"/>
       <c r="D396" s="9" t="n"/>
-      <c r="K396" s="10" t="n"/>
+      <c r="E396" s="9" t="n"/>
+      <c r="L396" s="10" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="9" t="n"/>
       <c r="B397" s="9" t="n"/>
       <c r="C397" s="9" t="n"/>
       <c r="D397" s="9" t="n"/>
-      <c r="K397" s="10" t="n"/>
+      <c r="E397" s="9" t="n"/>
+      <c r="L397" s="10" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="9" t="n"/>
       <c r="B398" s="9" t="n"/>
       <c r="C398" s="9" t="n"/>
       <c r="D398" s="9" t="n"/>
-      <c r="K398" s="10" t="n"/>
+      <c r="E398" s="9" t="n"/>
+      <c r="L398" s="10" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="9" t="n"/>
       <c r="B399" s="9" t="n"/>
       <c r="C399" s="9" t="n"/>
       <c r="D399" s="9" t="n"/>
-      <c r="K399" s="10" t="n"/>
+      <c r="E399" s="9" t="n"/>
+      <c r="L399" s="10" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="9" t="n"/>
       <c r="B400" s="9" t="n"/>
       <c r="C400" s="9" t="n"/>
       <c r="D400" s="9" t="n"/>
-      <c r="K400" s="10" t="n"/>
+      <c r="E400" s="9" t="n"/>
+      <c r="L400" s="10" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="9" t="n"/>
       <c r="B401" s="9" t="n"/>
       <c r="C401" s="9" t="n"/>
       <c r="D401" s="9" t="n"/>
-      <c r="K401" s="10" t="n"/>
+      <c r="E401" s="9" t="n"/>
+      <c r="L401" s="10" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="9" t="n"/>
       <c r="B402" s="9" t="n"/>
       <c r="C402" s="9" t="n"/>
       <c r="D402" s="9" t="n"/>
-      <c r="K402" s="10" t="n"/>
+      <c r="E402" s="9" t="n"/>
+      <c r="L402" s="10" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="9" t="n"/>
       <c r="B403" s="9" t="n"/>
       <c r="C403" s="9" t="n"/>
       <c r="D403" s="9" t="n"/>
-      <c r="K403" s="10" t="n"/>
+      <c r="E403" s="9" t="n"/>
+      <c r="L403" s="10" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="9" t="n"/>
       <c r="B404" s="9" t="n"/>
       <c r="C404" s="9" t="n"/>
       <c r="D404" s="9" t="n"/>
-      <c r="K404" s="10" t="n"/>
+      <c r="E404" s="9" t="n"/>
+      <c r="L404" s="10" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="9" t="n"/>
       <c r="B405" s="9" t="n"/>
       <c r="C405" s="9" t="n"/>
       <c r="D405" s="9" t="n"/>
-      <c r="K405" s="10" t="n"/>
+      <c r="E405" s="9" t="n"/>
+      <c r="L405" s="10" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="9" t="n"/>
       <c r="B406" s="9" t="n"/>
       <c r="C406" s="9" t="n"/>
       <c r="D406" s="9" t="n"/>
-      <c r="K406" s="10" t="n"/>
+      <c r="E406" s="9" t="n"/>
+      <c r="L406" s="10" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="9" t="n"/>
       <c r="B407" s="9" t="n"/>
       <c r="C407" s="9" t="n"/>
       <c r="D407" s="9" t="n"/>
-      <c r="K407" s="10" t="n"/>
+      <c r="E407" s="9" t="n"/>
+      <c r="L407" s="10" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="9" t="n"/>
       <c r="B408" s="9" t="n"/>
       <c r="C408" s="9" t="n"/>
       <c r="D408" s="9" t="n"/>
-      <c r="K408" s="10" t="n"/>
+      <c r="E408" s="9" t="n"/>
+      <c r="L408" s="10" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="9" t="n"/>
       <c r="B409" s="9" t="n"/>
       <c r="C409" s="9" t="n"/>
       <c r="D409" s="9" t="n"/>
-      <c r="K409" s="10" t="n"/>
+      <c r="E409" s="9" t="n"/>
+      <c r="L409" s="10" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="9" t="n"/>
       <c r="B410" s="9" t="n"/>
       <c r="C410" s="9" t="n"/>
       <c r="D410" s="9" t="n"/>
-      <c r="K410" s="10" t="n"/>
+      <c r="E410" s="9" t="n"/>
+      <c r="L410" s="10" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="9" t="n"/>
       <c r="B411" s="9" t="n"/>
       <c r="C411" s="9" t="n"/>
       <c r="D411" s="9" t="n"/>
-      <c r="K411" s="10" t="n"/>
+      <c r="E411" s="9" t="n"/>
+      <c r="L411" s="10" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="9" t="n"/>
       <c r="B412" s="9" t="n"/>
       <c r="C412" s="9" t="n"/>
       <c r="D412" s="9" t="n"/>
-      <c r="K412" s="10" t="n"/>
+      <c r="E412" s="9" t="n"/>
+      <c r="L412" s="10" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="9" t="n"/>
       <c r="B413" s="9" t="n"/>
       <c r="C413" s="9" t="n"/>
       <c r="D413" s="9" t="n"/>
-      <c r="K413" s="10" t="n"/>
+      <c r="E413" s="9" t="n"/>
+      <c r="L413" s="10" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="9" t="n"/>
       <c r="B414" s="9" t="n"/>
       <c r="C414" s="9" t="n"/>
       <c r="D414" s="9" t="n"/>
-      <c r="K414" s="10" t="n"/>
+      <c r="E414" s="9" t="n"/>
+      <c r="L414" s="10" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="9" t="n"/>
       <c r="B415" s="9" t="n"/>
       <c r="C415" s="9" t="n"/>
       <c r="D415" s="9" t="n"/>
-      <c r="K415" s="10" t="n"/>
+      <c r="E415" s="9" t="n"/>
+      <c r="L415" s="10" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="9" t="n"/>
       <c r="B416" s="9" t="n"/>
       <c r="C416" s="9" t="n"/>
       <c r="D416" s="9" t="n"/>
-      <c r="K416" s="10" t="n"/>
+      <c r="E416" s="9" t="n"/>
+      <c r="L416" s="10" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="9" t="n"/>
       <c r="B417" s="9" t="n"/>
       <c r="C417" s="9" t="n"/>
       <c r="D417" s="9" t="n"/>
-      <c r="K417" s="10" t="n"/>
+      <c r="E417" s="9" t="n"/>
+      <c r="L417" s="10" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="9" t="n"/>
       <c r="B418" s="9" t="n"/>
       <c r="C418" s="9" t="n"/>
       <c r="D418" s="9" t="n"/>
-      <c r="K418" s="10" t="n"/>
+      <c r="E418" s="9" t="n"/>
+      <c r="L418" s="10" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="9" t="n"/>
       <c r="B419" s="9" t="n"/>
       <c r="C419" s="9" t="n"/>
       <c r="D419" s="9" t="n"/>
-      <c r="K419" s="10" t="n"/>
+      <c r="E419" s="9" t="n"/>
+      <c r="L419" s="10" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="9" t="n"/>
       <c r="B420" s="9" t="n"/>
       <c r="C420" s="9" t="n"/>
       <c r="D420" s="9" t="n"/>
-      <c r="K420" s="10" t="n"/>
+      <c r="E420" s="9" t="n"/>
+      <c r="L420" s="10" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="9" t="n"/>
       <c r="B421" s="9" t="n"/>
       <c r="C421" s="9" t="n"/>
       <c r="D421" s="9" t="n"/>
-      <c r="K421" s="10" t="n"/>
+      <c r="E421" s="9" t="n"/>
+      <c r="L421" s="10" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="9" t="n"/>
       <c r="B422" s="9" t="n"/>
       <c r="C422" s="9" t="n"/>
       <c r="D422" s="9" t="n"/>
-      <c r="K422" s="10" t="n"/>
+      <c r="E422" s="9" t="n"/>
+      <c r="L422" s="10" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="9" t="n"/>
       <c r="B423" s="9" t="n"/>
       <c r="C423" s="9" t="n"/>
       <c r="D423" s="9" t="n"/>
-      <c r="K423" s="10" t="n"/>
+      <c r="E423" s="9" t="n"/>
+      <c r="L423" s="10" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="9" t="n"/>
       <c r="B424" s="9" t="n"/>
       <c r="C424" s="9" t="n"/>
       <c r="D424" s="9" t="n"/>
-      <c r="K424" s="10" t="n"/>
+      <c r="E424" s="9" t="n"/>
+      <c r="L424" s="10" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="9" t="n"/>
       <c r="B425" s="9" t="n"/>
       <c r="C425" s="9" t="n"/>
       <c r="D425" s="9" t="n"/>
-      <c r="K425" s="10" t="n"/>
+      <c r="E425" s="9" t="n"/>
+      <c r="L425" s="10" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="9" t="n"/>
       <c r="B426" s="9" t="n"/>
       <c r="C426" s="9" t="n"/>
       <c r="D426" s="9" t="n"/>
-      <c r="K426" s="10" t="n"/>
+      <c r="E426" s="9" t="n"/>
+      <c r="L426" s="10" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="9" t="n"/>
       <c r="B427" s="9" t="n"/>
       <c r="C427" s="9" t="n"/>
       <c r="D427" s="9" t="n"/>
-      <c r="K427" s="10" t="n"/>
+      <c r="E427" s="9" t="n"/>
+      <c r="L427" s="10" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="9" t="n"/>
       <c r="B428" s="9" t="n"/>
       <c r="C428" s="9" t="n"/>
       <c r="D428" s="9" t="n"/>
-      <c r="K428" s="10" t="n"/>
+      <c r="E428" s="9" t="n"/>
+      <c r="L428" s="10" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="9" t="n"/>
       <c r="B429" s="9" t="n"/>
       <c r="C429" s="9" t="n"/>
       <c r="D429" s="9" t="n"/>
-      <c r="K429" s="10" t="n"/>
+      <c r="E429" s="9" t="n"/>
+      <c r="L429" s="10" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="9" t="n"/>
       <c r="B430" s="9" t="n"/>
       <c r="C430" s="9" t="n"/>
       <c r="D430" s="9" t="n"/>
-      <c r="K430" s="10" t="n"/>
+      <c r="E430" s="9" t="n"/>
+      <c r="L430" s="10" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="9" t="n"/>
       <c r="B431" s="9" t="n"/>
       <c r="C431" s="9" t="n"/>
       <c r="D431" s="9" t="n"/>
-      <c r="K431" s="10" t="n"/>
+      <c r="E431" s="9" t="n"/>
+      <c r="L431" s="10" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="9" t="n"/>
       <c r="B432" s="9" t="n"/>
       <c r="C432" s="9" t="n"/>
       <c r="D432" s="9" t="n"/>
-      <c r="K432" s="10" t="n"/>
+      <c r="E432" s="9" t="n"/>
+      <c r="L432" s="10" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="9" t="n"/>
       <c r="B433" s="9" t="n"/>
       <c r="C433" s="9" t="n"/>
       <c r="D433" s="9" t="n"/>
-      <c r="K433" s="10" t="n"/>
+      <c r="E433" s="9" t="n"/>
+      <c r="L433" s="10" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="9" t="n"/>
       <c r="B434" s="9" t="n"/>
       <c r="C434" s="9" t="n"/>
       <c r="D434" s="9" t="n"/>
-      <c r="K434" s="10" t="n"/>
+      <c r="E434" s="9" t="n"/>
+      <c r="L434" s="10" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="9" t="n"/>
       <c r="B435" s="9" t="n"/>
       <c r="C435" s="9" t="n"/>
       <c r="D435" s="9" t="n"/>
-      <c r="K435" s="10" t="n"/>
+      <c r="E435" s="9" t="n"/>
+      <c r="L435" s="10" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="9" t="n"/>
       <c r="B436" s="9" t="n"/>
       <c r="C436" s="9" t="n"/>
       <c r="D436" s="9" t="n"/>
-      <c r="K436" s="10" t="n"/>
+      <c r="E436" s="9" t="n"/>
+      <c r="L436" s="10" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="9" t="n"/>
       <c r="B437" s="9" t="n"/>
       <c r="C437" s="9" t="n"/>
       <c r="D437" s="9" t="n"/>
-      <c r="K437" s="10" t="n"/>
+      <c r="E437" s="9" t="n"/>
+      <c r="L437" s="10" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="9" t="n"/>
       <c r="B438" s="9" t="n"/>
       <c r="C438" s="9" t="n"/>
       <c r="D438" s="9" t="n"/>
-      <c r="K438" s="10" t="n"/>
+      <c r="E438" s="9" t="n"/>
+      <c r="L438" s="10" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="9" t="n"/>
       <c r="B439" s="9" t="n"/>
       <c r="C439" s="9" t="n"/>
       <c r="D439" s="9" t="n"/>
-      <c r="K439" s="10" t="n"/>
+      <c r="E439" s="9" t="n"/>
+      <c r="L439" s="10" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="9" t="n"/>
       <c r="B440" s="9" t="n"/>
       <c r="C440" s="9" t="n"/>
       <c r="D440" s="9" t="n"/>
-      <c r="K440" s="10" t="n"/>
+      <c r="E440" s="9" t="n"/>
+      <c r="L440" s="10" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="9" t="n"/>
       <c r="B441" s="9" t="n"/>
       <c r="C441" s="9" t="n"/>
       <c r="D441" s="9" t="n"/>
-      <c r="K441" s="10" t="n"/>
+      <c r="E441" s="9" t="n"/>
+      <c r="L441" s="10" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="9" t="n"/>
       <c r="B442" s="9" t="n"/>
       <c r="C442" s="9" t="n"/>
       <c r="D442" s="9" t="n"/>
-      <c r="K442" s="10" t="n"/>
+      <c r="E442" s="9" t="n"/>
+      <c r="L442" s="10" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="9" t="n"/>
       <c r="B443" s="9" t="n"/>
       <c r="C443" s="9" t="n"/>
       <c r="D443" s="9" t="n"/>
-      <c r="K443" s="10" t="n"/>
+      <c r="E443" s="9" t="n"/>
+      <c r="L443" s="10" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="9" t="n"/>
       <c r="B444" s="9" t="n"/>
       <c r="C444" s="9" t="n"/>
       <c r="D444" s="9" t="n"/>
-      <c r="K444" s="10" t="n"/>
+      <c r="E444" s="9" t="n"/>
+      <c r="L444" s="10" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="9" t="n"/>
       <c r="B445" s="9" t="n"/>
       <c r="C445" s="9" t="n"/>
       <c r="D445" s="9" t="n"/>
-      <c r="K445" s="10" t="n"/>
+      <c r="E445" s="9" t="n"/>
+      <c r="L445" s="10" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="9" t="n"/>
       <c r="B446" s="9" t="n"/>
       <c r="C446" s="9" t="n"/>
       <c r="D446" s="9" t="n"/>
-      <c r="K446" s="10" t="n"/>
+      <c r="E446" s="9" t="n"/>
+      <c r="L446" s="10" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="9" t="n"/>
       <c r="B447" s="9" t="n"/>
       <c r="C447" s="9" t="n"/>
       <c r="D447" s="9" t="n"/>
-      <c r="K447" s="10" t="n"/>
+      <c r="E447" s="9" t="n"/>
+      <c r="L447" s="10" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="9" t="n"/>
       <c r="B448" s="9" t="n"/>
       <c r="C448" s="9" t="n"/>
       <c r="D448" s="9" t="n"/>
-      <c r="K448" s="10" t="n"/>
+      <c r="E448" s="9" t="n"/>
+      <c r="L448" s="10" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="9" t="n"/>
       <c r="B449" s="9" t="n"/>
       <c r="C449" s="9" t="n"/>
       <c r="D449" s="9" t="n"/>
-      <c r="K449" s="10" t="n"/>
+      <c r="E449" s="9" t="n"/>
+      <c r="L449" s="10" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="9" t="n"/>
       <c r="B450" s="9" t="n"/>
       <c r="C450" s="9" t="n"/>
       <c r="D450" s="9" t="n"/>
-      <c r="K450" s="10" t="n"/>
+      <c r="E450" s="9" t="n"/>
+      <c r="L450" s="10" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="9" t="n"/>
       <c r="B451" s="9" t="n"/>
       <c r="C451" s="9" t="n"/>
       <c r="D451" s="9" t="n"/>
-      <c r="K451" s="10" t="n"/>
+      <c r="E451" s="9" t="n"/>
+      <c r="L451" s="10" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="9" t="n"/>
       <c r="B452" s="9" t="n"/>
       <c r="C452" s="9" t="n"/>
       <c r="D452" s="9" t="n"/>
-      <c r="K452" s="10" t="n"/>
+      <c r="E452" s="9" t="n"/>
+      <c r="L452" s="10" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="9" t="n"/>
       <c r="B453" s="9" t="n"/>
       <c r="C453" s="9" t="n"/>
       <c r="D453" s="9" t="n"/>
-      <c r="K453" s="10" t="n"/>
+      <c r="E453" s="9" t="n"/>
+      <c r="L453" s="10" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="9" t="n"/>
       <c r="B454" s="9" t="n"/>
       <c r="C454" s="9" t="n"/>
       <c r="D454" s="9" t="n"/>
-      <c r="K454" s="10" t="n"/>
+      <c r="E454" s="9" t="n"/>
+      <c r="L454" s="10" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="9" t="n"/>
       <c r="B455" s="9" t="n"/>
       <c r="C455" s="9" t="n"/>
       <c r="D455" s="9" t="n"/>
-      <c r="K455" s="10" t="n"/>
+      <c r="E455" s="9" t="n"/>
+      <c r="L455" s="10" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="9" t="n"/>
       <c r="B456" s="9" t="n"/>
       <c r="C456" s="9" t="n"/>
       <c r="D456" s="9" t="n"/>
-      <c r="K456" s="10" t="n"/>
+      <c r="E456" s="9" t="n"/>
+      <c r="L456" s="10" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="9" t="n"/>
       <c r="B457" s="9" t="n"/>
       <c r="C457" s="9" t="n"/>
       <c r="D457" s="9" t="n"/>
-      <c r="K457" s="10" t="n"/>
+      <c r="E457" s="9" t="n"/>
+      <c r="L457" s="10" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="9" t="n"/>
       <c r="B458" s="9" t="n"/>
       <c r="C458" s="9" t="n"/>
       <c r="D458" s="9" t="n"/>
-      <c r="K458" s="10" t="n"/>
+      <c r="E458" s="9" t="n"/>
+      <c r="L458" s="10" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="9" t="n"/>
       <c r="B459" s="9" t="n"/>
       <c r="C459" s="9" t="n"/>
       <c r="D459" s="9" t="n"/>
-      <c r="K459" s="10" t="n"/>
+      <c r="E459" s="9" t="n"/>
+      <c r="L459" s="10" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="9" t="n"/>
       <c r="B460" s="9" t="n"/>
       <c r="C460" s="9" t="n"/>
       <c r="D460" s="9" t="n"/>
-      <c r="K460" s="10" t="n"/>
+      <c r="E460" s="9" t="n"/>
+      <c r="L460" s="10" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="9" t="n"/>
       <c r="B461" s="9" t="n"/>
       <c r="C461" s="9" t="n"/>
       <c r="D461" s="9" t="n"/>
-      <c r="K461" s="10" t="n"/>
+      <c r="E461" s="9" t="n"/>
+      <c r="L461" s="10" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="9" t="n"/>
       <c r="B462" s="9" t="n"/>
       <c r="C462" s="9" t="n"/>
       <c r="D462" s="9" t="n"/>
-      <c r="K462" s="10" t="n"/>
+      <c r="E462" s="9" t="n"/>
+      <c r="L462" s="10" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="9" t="n"/>
       <c r="B463" s="9" t="n"/>
       <c r="C463" s="9" t="n"/>
       <c r="D463" s="9" t="n"/>
-      <c r="K463" s="10" t="n"/>
+      <c r="E463" s="9" t="n"/>
+      <c r="L463" s="10" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="9" t="n"/>
       <c r="B464" s="9" t="n"/>
       <c r="C464" s="9" t="n"/>
       <c r="D464" s="9" t="n"/>
-      <c r="K464" s="10" t="n"/>
+      <c r="E464" s="9" t="n"/>
+      <c r="L464" s="10" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="9" t="n"/>
       <c r="B465" s="9" t="n"/>
       <c r="C465" s="9" t="n"/>
       <c r="D465" s="9" t="n"/>
-      <c r="K465" s="10" t="n"/>
+      <c r="E465" s="9" t="n"/>
+      <c r="L465" s="10" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="9" t="n"/>
       <c r="B466" s="9" t="n"/>
       <c r="C466" s="9" t="n"/>
       <c r="D466" s="9" t="n"/>
-      <c r="K466" s="10" t="n"/>
+      <c r="E466" s="9" t="n"/>
+      <c r="L466" s="10" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="9" t="n"/>
       <c r="B467" s="9" t="n"/>
       <c r="C467" s="9" t="n"/>
       <c r="D467" s="9" t="n"/>
-      <c r="K467" s="10" t="n"/>
+      <c r="E467" s="9" t="n"/>
+      <c r="L467" s="10" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="9" t="n"/>
       <c r="B468" s="9" t="n"/>
       <c r="C468" s="9" t="n"/>
       <c r="D468" s="9" t="n"/>
-      <c r="K468" s="10" t="n"/>
+      <c r="E468" s="9" t="n"/>
+      <c r="L468" s="10" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="9" t="n"/>
       <c r="B469" s="9" t="n"/>
       <c r="C469" s="9" t="n"/>
       <c r="D469" s="9" t="n"/>
-      <c r="K469" s="10" t="n"/>
+      <c r="E469" s="9" t="n"/>
+      <c r="L469" s="10" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="9" t="n"/>
       <c r="B470" s="9" t="n"/>
       <c r="C470" s="9" t="n"/>
       <c r="D470" s="9" t="n"/>
-      <c r="K470" s="10" t="n"/>
+      <c r="E470" s="9" t="n"/>
+      <c r="L470" s="10" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="9" t="n"/>
       <c r="B471" s="9" t="n"/>
       <c r="C471" s="9" t="n"/>
       <c r="D471" s="9" t="n"/>
-      <c r="K471" s="10" t="n"/>
+      <c r="E471" s="9" t="n"/>
+      <c r="L471" s="10" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="9" t="n"/>
       <c r="B472" s="9" t="n"/>
       <c r="C472" s="9" t="n"/>
       <c r="D472" s="9" t="n"/>
-      <c r="K472" s="10" t="n"/>
+      <c r="E472" s="9" t="n"/>
+      <c r="L472" s="10" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="9" t="n"/>
       <c r="B473" s="9" t="n"/>
       <c r="C473" s="9" t="n"/>
       <c r="D473" s="9" t="n"/>
-      <c r="K473" s="10" t="n"/>
+      <c r="E473" s="9" t="n"/>
+      <c r="L473" s="10" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="9" t="n"/>
       <c r="B474" s="9" t="n"/>
       <c r="C474" s="9" t="n"/>
       <c r="D474" s="9" t="n"/>
-      <c r="K474" s="10" t="n"/>
+      <c r="E474" s="9" t="n"/>
+      <c r="L474" s="10" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="9" t="n"/>
       <c r="B475" s="9" t="n"/>
       <c r="C475" s="9" t="n"/>
       <c r="D475" s="9" t="n"/>
-      <c r="K475" s="10" t="n"/>
+      <c r="E475" s="9" t="n"/>
+      <c r="L475" s="10" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="9" t="n"/>
       <c r="B476" s="9" t="n"/>
       <c r="C476" s="9" t="n"/>
       <c r="D476" s="9" t="n"/>
-      <c r="K476" s="10" t="n"/>
+      <c r="E476" s="9" t="n"/>
+      <c r="L476" s="10" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="9" t="n"/>
       <c r="B477" s="9" t="n"/>
       <c r="C477" s="9" t="n"/>
       <c r="D477" s="9" t="n"/>
-      <c r="K477" s="10" t="n"/>
+      <c r="E477" s="9" t="n"/>
+      <c r="L477" s="10" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="9" t="n"/>
       <c r="B478" s="9" t="n"/>
       <c r="C478" s="9" t="n"/>
       <c r="D478" s="9" t="n"/>
-      <c r="K478" s="10" t="n"/>
+      <c r="E478" s="9" t="n"/>
+      <c r="L478" s="10" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="9" t="n"/>
       <c r="B479" s="9" t="n"/>
       <c r="C479" s="9" t="n"/>
       <c r="D479" s="9" t="n"/>
-      <c r="K479" s="10" t="n"/>
+      <c r="E479" s="9" t="n"/>
+      <c r="L479" s="10" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="9" t="n"/>
       <c r="B480" s="9" t="n"/>
       <c r="C480" s="9" t="n"/>
       <c r="D480" s="9" t="n"/>
-      <c r="K480" s="10" t="n"/>
+      <c r="E480" s="9" t="n"/>
+      <c r="L480" s="10" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="9" t="n"/>
       <c r="B481" s="9" t="n"/>
       <c r="C481" s="9" t="n"/>
       <c r="D481" s="9" t="n"/>
-      <c r="K481" s="10" t="n"/>
+      <c r="E481" s="9" t="n"/>
+      <c r="L481" s="10" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="9" t="n"/>
       <c r="B482" s="9" t="n"/>
       <c r="C482" s="9" t="n"/>
       <c r="D482" s="9" t="n"/>
-      <c r="K482" s="10" t="n"/>
+      <c r="E482" s="9" t="n"/>
+      <c r="L482" s="10" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="9" t="n"/>
       <c r="B483" s="9" t="n"/>
       <c r="C483" s="9" t="n"/>
       <c r="D483" s="9" t="n"/>
-      <c r="K483" s="10" t="n"/>
+      <c r="E483" s="9" t="n"/>
+      <c r="L483" s="10" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="9" t="n"/>
       <c r="B484" s="9" t="n"/>
       <c r="C484" s="9" t="n"/>
       <c r="D484" s="9" t="n"/>
-      <c r="K484" s="10" t="n"/>
+      <c r="E484" s="9" t="n"/>
+      <c r="L484" s="10" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="9" t="n"/>
       <c r="B485" s="9" t="n"/>
       <c r="C485" s="9" t="n"/>
       <c r="D485" s="9" t="n"/>
-      <c r="K485" s="10" t="n"/>
+      <c r="E485" s="9" t="n"/>
+      <c r="L485" s="10" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="9" t="n"/>
       <c r="B486" s="9" t="n"/>
       <c r="C486" s="9" t="n"/>
       <c r="D486" s="9" t="n"/>
-      <c r="K486" s="10" t="n"/>
+      <c r="E486" s="9" t="n"/>
+      <c r="L486" s="10" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="9" t="n"/>
       <c r="B487" s="9" t="n"/>
       <c r="C487" s="9" t="n"/>
       <c r="D487" s="9" t="n"/>
-      <c r="K487" s="10" t="n"/>
+      <c r="E487" s="9" t="n"/>
+      <c r="L487" s="10" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="9" t="n"/>
       <c r="B488" s="9" t="n"/>
       <c r="C488" s="9" t="n"/>
       <c r="D488" s="9" t="n"/>
-      <c r="K488" s="10" t="n"/>
+      <c r="E488" s="9" t="n"/>
+      <c r="L488" s="10" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="9" t="n"/>
       <c r="B489" s="9" t="n"/>
       <c r="C489" s="9" t="n"/>
       <c r="D489" s="9" t="n"/>
-      <c r="K489" s="10" t="n"/>
+      <c r="E489" s="9" t="n"/>
+      <c r="L489" s="10" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="9" t="n"/>
       <c r="B490" s="9" t="n"/>
       <c r="C490" s="9" t="n"/>
       <c r="D490" s="9" t="n"/>
-      <c r="K490" s="10" t="n"/>
+      <c r="E490" s="9" t="n"/>
+      <c r="L490" s="10" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="9" t="n"/>
       <c r="B491" s="9" t="n"/>
       <c r="C491" s="9" t="n"/>
       <c r="D491" s="9" t="n"/>
-      <c r="K491" s="10" t="n"/>
+      <c r="E491" s="9" t="n"/>
+      <c r="L491" s="10" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="9" t="n"/>
       <c r="B492" s="9" t="n"/>
       <c r="C492" s="9" t="n"/>
       <c r="D492" s="9" t="n"/>
-      <c r="K492" s="10" t="n"/>
+      <c r="E492" s="9" t="n"/>
+      <c r="L492" s="10" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="9" t="n"/>
       <c r="B493" s="9" t="n"/>
       <c r="C493" s="9" t="n"/>
       <c r="D493" s="9" t="n"/>
-      <c r="K493" s="10" t="n"/>
+      <c r="E493" s="9" t="n"/>
+      <c r="L493" s="10" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="9" t="n"/>
       <c r="B494" s="9" t="n"/>
       <c r="C494" s="9" t="n"/>
       <c r="D494" s="9" t="n"/>
-      <c r="K494" s="10" t="n"/>
+      <c r="E494" s="9" t="n"/>
+      <c r="L494" s="10" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="9" t="n"/>
       <c r="B495" s="9" t="n"/>
       <c r="C495" s="9" t="n"/>
       <c r="D495" s="9" t="n"/>
-      <c r="K495" s="10" t="n"/>
+      <c r="E495" s="9" t="n"/>
+      <c r="L495" s="10" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="9" t="n"/>
       <c r="B496" s="9" t="n"/>
       <c r="C496" s="9" t="n"/>
       <c r="D496" s="9" t="n"/>
-      <c r="K496" s="10" t="n"/>
+      <c r="E496" s="9" t="n"/>
+      <c r="L496" s="10" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="9" t="n"/>
       <c r="B497" s="9" t="n"/>
       <c r="C497" s="9" t="n"/>
       <c r="D497" s="9" t="n"/>
-      <c r="K497" s="10" t="n"/>
+      <c r="E497" s="9" t="n"/>
+      <c r="L497" s="10" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="9" t="n"/>
       <c r="B498" s="9" t="n"/>
       <c r="C498" s="9" t="n"/>
       <c r="D498" s="9" t="n"/>
-      <c r="K498" s="10" t="n"/>
+      <c r="E498" s="9" t="n"/>
+      <c r="L498" s="10" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="9" t="n"/>
       <c r="B499" s="9" t="n"/>
       <c r="C499" s="9" t="n"/>
       <c r="D499" s="9" t="n"/>
-      <c r="K499" s="10" t="n"/>
+      <c r="E499" s="9" t="n"/>
+      <c r="L499" s="10" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="9" t="n"/>
       <c r="B500" s="9" t="n"/>
       <c r="C500" s="9" t="n"/>
       <c r="D500" s="9" t="n"/>
-      <c r="K500" s="10" t="n"/>
+      <c r="E500" s="9" t="n"/>
+      <c r="L500" s="10" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="9" t="n"/>
       <c r="B501" s="9" t="n"/>
       <c r="C501" s="9" t="n"/>
       <c r="D501" s="9" t="n"/>
-      <c r="K501" s="10" t="n"/>
+      <c r="E501" s="9" t="n"/>
+      <c r="L501" s="10" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Objekta veids" error="Izvēlieties: īpašums, zemes vienība, būve." type="list">
+    <dataValidation sqref="D2:D501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Objekta veids" error="Izvēlieties: īpašums, zemes vienība, būve." type="list">
       <formula1>"īpašums,zemes vienība,būve"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Datums" error="Ievadiet datumu (GGGG-MM-DD)." type="date" operator="greaterThan">
+    <dataValidation sqref="L2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Datums" error="Ievadiet datumu (GGGG-MM-DD)." type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>